<commit_message>
V. 143 "Muertos S.L."
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7995AC5-21DE-454D-BBD5-887D265ED830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14805AAD-8F54-4796-9DCA-CCC3EDC639AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -72,6 +72,7 @@
     <author>tc={BC097833-5E05-4B57-A72A-B55B23EF385A}</author>
     <author>tc={D69ACFED-A245-418D-8836-7787A10A08B4}</author>
     <author>tc={FE4CA59D-CA2D-4361-94E4-6EA24C8AD9DE}</author>
+    <author>tc={45CF8DED-8FF7-438A-B23B-D9A4345C4CDA}</author>
     <author>tc={0372C847-801C-4993-BA73-8301D595FCF1}</author>
     <author>tc={64FF07EB-F3D4-47C4-B23E-4905CF85CACC}</author>
     <author>tc={ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}</author>
@@ -361,7 +362,7 @@
     5 temporadas</t>
       </text>
     </comment>
-    <comment ref="B41" authorId="33" shapeId="0" xr:uid="{0372C847-801C-4993-BA73-8301D595FCF1}">
+    <comment ref="B40" authorId="33" shapeId="0" xr:uid="{45CF8DED-8FF7-438A-B23B-D9A4345C4CDA}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -369,7 +370,15 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B42" authorId="34" shapeId="0" xr:uid="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
+    <comment ref="B42" authorId="34" shapeId="0" xr:uid="{0372C847-801C-4993-BA73-8301D595FCF1}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    1 temporada</t>
+      </text>
+    </comment>
+    <comment ref="B43" authorId="35" shapeId="0" xr:uid="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -377,7 +386,7 @@
     2 temporadas</t>
       </text>
     </comment>
-    <comment ref="B43" authorId="35" shapeId="0" xr:uid="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
+    <comment ref="B44" authorId="36" shapeId="0" xr:uid="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -385,7 +394,7 @@
     6 temporadas</t>
       </text>
     </comment>
-    <comment ref="B45" authorId="36" shapeId="0" xr:uid="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
+    <comment ref="B46" authorId="37" shapeId="0" xr:uid="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -393,7 +402,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B46" authorId="37" shapeId="0" xr:uid="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
+    <comment ref="B47" authorId="38" shapeId="0" xr:uid="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -401,7 +410,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B47" authorId="38" shapeId="0" xr:uid="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
+    <comment ref="B48" authorId="39" shapeId="0" xr:uid="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -409,7 +418,7 @@
     6 temporadas</t>
       </text>
     </comment>
-    <comment ref="B48" authorId="39" shapeId="0" xr:uid="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
+    <comment ref="B49" authorId="40" shapeId="0" xr:uid="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -417,7 +426,7 @@
     14 temporadas</t>
       </text>
     </comment>
-    <comment ref="B50" authorId="40" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -425,7 +434,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -433,7 +442,7 @@
     5 temporadas</t>
       </text>
     </comment>
-    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -441,7 +450,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+    <comment ref="B54" authorId="44" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -449,7 +458,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B54" authorId="44" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+    <comment ref="B55" authorId="45" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -457,7 +466,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B57" authorId="45" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -465,7 +474,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -473,7 +482,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -481,7 +490,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+    <comment ref="B61" authorId="49" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -489,7 +498,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B61" authorId="49" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+    <comment ref="B62" authorId="50" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -497,7 +506,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B67" authorId="50" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -505,7 +514,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -513,7 +522,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -521,7 +530,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -529,7 +538,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -537,7 +546,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+    <comment ref="B73" authorId="56" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -612,7 +621,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="248">
   <si>
     <t>Película</t>
   </si>
@@ -1353,6 +1362,9 @@
   </si>
   <si>
     <t>La leyenda de Tarzán</t>
+  </si>
+  <si>
+    <t>Muertos S.L.</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1374,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1398,6 +1410,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1441,7 +1459,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1464,9 +1482,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1679,10 +1694,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M72" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="B2:M72" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M72">
-    <sortCondition descending="1" ref="C2:C72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M73" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="B2:M73" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M73">
+    <sortCondition descending="1" ref="C2:C73"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
@@ -2088,73 +2103,76 @@
   <threadedComment ref="B39" dT="2024-07-08T19:08:20.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{FE4CA59D-CA2D-4361-94E4-6EA24C8AD9DE}">
     <text>5 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B41" dT="2025-10-21T19:53:14.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{0372C847-801C-4993-BA73-8301D595FCF1}">
+  <threadedComment ref="B40" dT="2026-07-22T14:40:30.01" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{45CF8DED-8FF7-438A-B23B-D9A4345C4CDA}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B42" dT="2024-07-08T19:04:29.42" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
+  <threadedComment ref="B42" dT="2025-10-21T19:53:14.38" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{0372C847-801C-4993-BA73-8301D595FCF1}">
+    <text>1 temporada</text>
+  </threadedComment>
+  <threadedComment ref="B43" dT="2024-07-08T19:04:29.42" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{64FF07EB-F3D4-47C4-B23E-4905CF85CACC}">
     <text>2 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B43" dT="2024-12-19T19:39:49.29" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
+  <threadedComment ref="B44" dT="2024-12-19T19:39:49.29" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ACBD2AE4-B2D6-490A-B6A8-26BE6D3CC6C9}">
     <text>6 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B45" dT="2024-07-08T19:08:48.45" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
+  <threadedComment ref="B46" dT="2024-07-08T19:08:48.45" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{500EEDC0-7745-4F10-8309-4ED19BDF789B}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B46" dT="2025-04-09T21:18:34.74" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
+  <threadedComment ref="B47" dT="2025-04-09T21:18:34.74" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3E762906-7E78-4A82-82BD-91226BEEE65F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B47" dT="2024-07-08T19:09:26.44" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
+  <threadedComment ref="B48" dT="2024-07-08T19:09:26.44" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{A836A830-A167-47D8-ADFF-FC6A88D1B4AF}">
     <text>6 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B48" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
+  <threadedComment ref="B49" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
     <text>14 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B50" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+  <threadedComment ref="B51" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B51" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+  <threadedComment ref="B52" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
     <text>5 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B52" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+  <threadedComment ref="B53" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B53" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+  <threadedComment ref="B54" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B54" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+  <threadedComment ref="B55" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B57" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+  <threadedComment ref="B58" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B58" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+  <threadedComment ref="B59" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B59" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+  <threadedComment ref="B60" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B60" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+  <threadedComment ref="B61" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B61" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+  <threadedComment ref="B62" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B67" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+  <threadedComment ref="B68" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B68" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+  <threadedComment ref="B69" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B69" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+  <threadedComment ref="B70" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B70" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+  <threadedComment ref="B71" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B71" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+  <threadedComment ref="B72" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B72" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+  <threadedComment ref="B73" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
     <text>4 temporadas</text>
   </threadedComment>
 </ThreadedComments>
@@ -2166,7 +2184,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O72"/>
+  <dimension ref="B2:O73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.140625" customWidth="1"/>
@@ -2228,7 +2246,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2262,7 +2280,7 @@
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2295,7 +2313,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2331,7 +2349,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2367,7 +2385,7 @@
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2401,7 +2419,7 @@
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2434,7 +2452,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2467,7 +2485,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2500,7 +2518,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2533,7 +2551,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2568,7 +2586,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2603,7 +2621,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2636,7 +2654,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2669,7 +2687,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2704,7 +2722,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2737,7 +2755,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2770,7 +2788,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2803,7 +2821,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2834,7 +2852,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2867,7 +2885,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2900,7 +2918,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2933,7 +2951,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2966,7 +2984,7 @@
         <v>238</v>
       </c>
       <c r="C25" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
         <v>7.8874999999999993</v>
       </c>
       <c r="D25" s="1">
@@ -2999,7 +3017,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
         <v>7.8750000000000009</v>
       </c>
       <c r="D26" s="1">
@@ -3032,7 +3050,7 @@
         <v>43</v>
       </c>
       <c r="C27" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
         <v>7.8125000000000009</v>
       </c>
       <c r="D27" s="1">
@@ -3065,7 +3083,7 @@
         <v>138</v>
       </c>
       <c r="C28" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
         <v>7.8125</v>
       </c>
       <c r="D28" s="1">
@@ -3098,7 +3116,7 @@
         <v>82</v>
       </c>
       <c r="C29" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
         <v>7.7874999999999996</v>
       </c>
       <c r="D29" s="1">
@@ -3131,7 +3149,7 @@
         <v>73</v>
       </c>
       <c r="C30" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
         <v>7.7250000000000005</v>
       </c>
       <c r="D30" s="1">
@@ -3166,7 +3184,7 @@
         <v>142</v>
       </c>
       <c r="C31" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3199,7 +3217,7 @@
         <v>192</v>
       </c>
       <c r="C32" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D32" s="1">
@@ -3232,7 +3250,7 @@
         <v>47</v>
       </c>
       <c r="C33" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
         <v>7.6000000000000005</v>
       </c>
       <c r="D33" s="1">
@@ -3265,7 +3283,7 @@
         <v>198</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
         <v>7.5625</v>
       </c>
       <c r="D34" s="1">
@@ -3298,7 +3316,7 @@
         <v>15</v>
       </c>
       <c r="C35" s="5">
-        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
@@ -3334,7 +3352,7 @@
         <v>210</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D36" s="1">
@@ -3367,7 +3385,7 @@
         <v>105</v>
       </c>
       <c r="C37" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
@@ -3402,7 +3420,7 @@
         <v>141</v>
       </c>
       <c r="C38" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D38" s="1">
@@ -3435,7 +3453,7 @@
         <v>16</v>
       </c>
       <c r="C39" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
         <v>7.4874999999999989</v>
       </c>
       <c r="D39" s="1">
@@ -3464,94 +3482,94 @@
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B40" s="2" t="s">
-        <v>50</v>
+        <v>247</v>
       </c>
       <c r="C40" s="5">
-        <f t="shared" si="1"/>
-        <v>7.35</v>
+        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
+        <v>7.4625000000000004</v>
       </c>
       <c r="D40" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E40" s="1">
         <v>7</v>
       </c>
       <c r="F40" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G40" s="1">
         <v>7</v>
       </c>
       <c r="H40" s="3">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="I40" s="3">
-        <v>7.8</v>
-      </c>
-      <c r="J40" s="1"/>
+        <v>6.7</v>
+      </c>
+      <c r="J40" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K40" s="1"/>
-      <c r="L40" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41" s="2" t="s">
-        <v>185</v>
+        <v>50</v>
       </c>
       <c r="C41" s="5">
-        <f t="shared" si="1"/>
-        <v>7.3</v>
+        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
+        <v>7.35</v>
       </c>
       <c r="D41" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E41" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F41" s="1">
         <v>7</v>
       </c>
       <c r="G41" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H41" s="3">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="I41" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J41" t="e" vm="1">
+        <v>7.8</v>
+      </c>
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+      <c r="L41" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
-        <v>80</v>
+        <v>185</v>
       </c>
       <c r="C42" s="5">
-        <f t="shared" si="1"/>
-        <v>7.2500000000000009</v>
+        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
+        <v>7.3</v>
       </c>
       <c r="D42" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E42" s="1">
         <v>8</v>
       </c>
       <c r="F42" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G42" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H42" s="3">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="I42" s="3">
-        <v>4.5999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="J42" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3562,29 +3580,29 @@
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="C43" s="5">
-        <f t="shared" si="1"/>
-        <v>7.25</v>
+        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
+        <v>7.2500000000000009</v>
       </c>
       <c r="D43" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E43" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F43" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G43" s="1">
         <v>7</v>
       </c>
       <c r="H43" s="3">
-        <v>8.4</v>
+        <v>6.7</v>
       </c>
       <c r="I43" s="3">
-        <v>7.2</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="J43" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3595,129 +3613,129 @@
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="C44" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
+        <v>7.25</v>
+      </c>
+      <c r="D44" s="1">
+        <v>8</v>
+      </c>
+      <c r="E44" s="1">
+        <v>5</v>
+      </c>
+      <c r="F44" s="1">
+        <v>7</v>
+      </c>
+      <c r="G44" s="1">
+        <v>7</v>
+      </c>
+      <c r="H44" s="3">
+        <v>8.4</v>
+      </c>
+      <c r="I44" s="3">
         <v>7.2</v>
-      </c>
-      <c r="D44" s="1">
-        <v>8</v>
-      </c>
-      <c r="E44" s="1">
-        <v>8</v>
-      </c>
-      <c r="F44" s="1">
-        <v>7</v>
-      </c>
-      <c r="G44" s="1">
-        <v>5</v>
-      </c>
-      <c r="H44" s="3">
-        <v>8</v>
-      </c>
-      <c r="I44" s="3">
-        <v>6.6</v>
       </c>
       <c r="J44" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K44" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C45" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
         <v>7.2</v>
       </c>
       <c r="D45" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E45" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F45" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G45" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H45" s="3">
-        <v>8.6</v>
+        <v>8</v>
       </c>
       <c r="I45" s="3">
-        <v>7.4</v>
-      </c>
-      <c r="J45" s="1"/>
-      <c r="K45" s="1"/>
-      <c r="L45" t="e" vm="5">
+        <v>6.6</v>
+      </c>
+      <c r="J45" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K45" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
-        <v>140</v>
+        <v>22</v>
       </c>
       <c r="C46" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1875000000000009</v>
+        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
+        <v>7.2</v>
       </c>
       <c r="D46" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E46" s="1">
         <v>7</v>
       </c>
       <c r="F46" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G46" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H46" s="3">
-        <v>6.7</v>
+        <v>8.6</v>
       </c>
       <c r="I46" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="J46" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="L46" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K46" s="1"/>
-      <c r="L46" s="1"/>
-      <c r="M46" s="1"/>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="C47" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1875</v>
+        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
+        <v>7.1875000000000009</v>
       </c>
       <c r="D47" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E47" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F47" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G47" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H47" s="3">
-        <v>9.1</v>
+        <v>6.7</v>
       </c>
       <c r="I47" s="3">
-        <v>8.3000000000000007</v>
+        <v>6.1</v>
       </c>
       <c r="J47" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3728,129 +3746,129 @@
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="C48" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1749999999999998</v>
+        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
+        <v>7.1875</v>
       </c>
       <c r="D48" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E48" s="1">
         <v>6</v>
       </c>
       <c r="F48" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G48" s="1">
         <v>7</v>
       </c>
       <c r="H48" s="3">
-        <v>7.5</v>
+        <v>9.1</v>
       </c>
       <c r="I48" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J48" s="1"/>
-      <c r="K48" t="e" vm="2">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="J48" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="L48" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C49" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D49" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E49" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F49" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G49" s="1">
         <v>7</v>
       </c>
       <c r="H49" s="3">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="I49" s="3">
-        <v>7.4</v>
+        <v>5.4</v>
       </c>
       <c r="J49" s="1"/>
       <c r="K49" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="L49" s="1"/>
-      <c r="M49" s="1"/>
+      <c r="L49" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>234</v>
+        <v>49</v>
       </c>
       <c r="C50" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1000000000000005</v>
+        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
+        <v>7.1749999999999998</v>
       </c>
       <c r="D50" s="1">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E50" s="1">
         <v>8</v>
       </c>
       <c r="F50" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G50" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H50" s="3">
-        <v>6.7</v>
+        <v>8.5</v>
       </c>
       <c r="I50" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J50" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J50" s="1"/>
+      <c r="K50" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C51" s="5">
-        <f t="shared" si="1"/>
-        <v>7.0875000000000004</v>
+        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
+        <v>7.1000000000000005</v>
       </c>
       <c r="D51" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E51" s="1">
         <v>8</v>
       </c>
       <c r="F51" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G51" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H51" s="3">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="I51" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="J51" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3861,14 +3879,14 @@
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C52" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
         <v>7.0875000000000004</v>
       </c>
       <c r="D52" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E52" s="1">
         <v>8</v>
@@ -3877,144 +3895,145 @@
         <v>7</v>
       </c>
       <c r="G52" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H52" s="3">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="I52" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="J52" s="1"/>
+        <v>6.3</v>
+      </c>
+      <c r="J52" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>71</v>
+        <v>231</v>
       </c>
       <c r="C53" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9750000000000005</v>
+        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D53" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E53" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F53" s="1">
         <v>7</v>
       </c>
       <c r="G53" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H53" s="3">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="I53" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J53" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K53" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+        <v>5.5</v>
+      </c>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C54" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9</v>
+        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <v>6.9750000000000005</v>
       </c>
       <c r="D54" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E54" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F54" s="1">
         <v>7</v>
       </c>
       <c r="G54" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H54" s="3">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="I54" s="3">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="J54" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K54" s="1"/>
+      <c r="K54" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="C55" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8750000000000009</v>
+        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <v>6.9</v>
       </c>
       <c r="D55" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E55" s="1">
         <v>6</v>
       </c>
       <c r="F55" s="1">
+        <v>7</v>
+      </c>
+      <c r="G55" s="1">
         <v>5</v>
       </c>
-      <c r="G55" s="1">
-        <v>7</v>
-      </c>
       <c r="H55" s="3">
-        <v>8.6999999999999993</v>
+        <v>8</v>
       </c>
       <c r="I55" s="3">
-        <v>8.6</v>
-      </c>
-      <c r="J55" s="1"/>
+        <v>7.2</v>
+      </c>
+      <c r="J55" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K55" s="1"/>
-      <c r="L55" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C56" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8</v>
+        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <v>6.8750000000000009</v>
       </c>
       <c r="D56" s="1">
         <v>6</v>
       </c>
       <c r="E56" s="1">
+        <v>6</v>
+      </c>
+      <c r="F56" s="1">
         <v>5</v>
       </c>
-      <c r="F56" s="1">
-        <v>6</v>
-      </c>
       <c r="G56" s="1">
         <v>7</v>
       </c>
       <c r="H56" s="3">
-        <v>8.5</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="I56" s="3">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
@@ -4024,17 +4043,17 @@
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
       <c r="C57" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7750000000000004</v>
+        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <v>6.8</v>
       </c>
       <c r="D57" s="1">
         <v>6</v>
       </c>
       <c r="E57" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F57" s="1">
         <v>6</v>
@@ -4043,43 +4062,42 @@
         <v>7</v>
       </c>
       <c r="H57" s="3">
-        <v>7.7</v>
+        <v>8.5</v>
       </c>
       <c r="I57" s="3">
-        <v>6.8</v>
-      </c>
-      <c r="J57" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="L57" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K57" s="1"/>
-      <c r="L57" s="1"/>
-      <c r="M57" s="1"/>
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C58" s="5">
-        <f t="shared" si="1"/>
-        <v>6.75</v>
+        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <v>6.7750000000000004</v>
       </c>
       <c r="D58" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E58" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F58" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G58" s="1">
         <v>7</v>
       </c>
       <c r="H58" s="3">
-        <v>5.9</v>
+        <v>7.7</v>
       </c>
       <c r="I58" s="3">
-        <v>4.2</v>
+        <v>6.8</v>
       </c>
       <c r="J58" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4090,61 +4108,62 @@
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="C59" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7250000000000005</v>
+        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <v>6.75</v>
       </c>
       <c r="D59" s="1">
         <v>8</v>
       </c>
       <c r="E59" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F59" s="1">
         <v>7</v>
       </c>
       <c r="G59" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H59" s="3">
-        <v>7.7</v>
+        <v>5.9</v>
       </c>
       <c r="I59" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J59" s="1"/>
+        <v>4.2</v>
+      </c>
+      <c r="J59" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K59" s="1"/>
-      <c r="L59" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C60" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7</v>
+        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <v>6.7250000000000005</v>
       </c>
       <c r="D60" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E60" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F60" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G60" s="1">
         <v>6</v>
       </c>
       <c r="H60" s="3">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
       <c r="I60" s="3">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
@@ -4154,79 +4173,76 @@
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C61" s="5">
-        <f t="shared" si="1"/>
-        <v>6.55</v>
+        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <v>6.7</v>
       </c>
       <c r="D61" s="1">
         <v>5</v>
       </c>
       <c r="E61" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F61" s="1">
         <v>6</v>
       </c>
       <c r="G61" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H61" s="3">
-        <v>7</v>
+        <v>8.6</v>
       </c>
       <c r="I61" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J61" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J61" s="1"/>
+      <c r="K61" s="1"/>
+      <c r="L61" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K61" s="1"/>
-      <c r="L61" s="1"/>
-      <c r="M61" s="1"/>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="C62" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4875000000000007</v>
+        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <v>6.55</v>
       </c>
       <c r="D62" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E62" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F62" s="1">
         <v>6</v>
       </c>
       <c r="G62" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H62" s="3">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="I62" s="3">
-        <v>7.7</v>
-      </c>
-      <c r="J62" s="1"/>
-      <c r="K62" t="e" vm="2">
+        <v>5.4</v>
+      </c>
+      <c r="J62" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K62" s="1"/>
       <c r="L62" s="1"/>
-      <c r="M62" s="1" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+      <c r="M62" s="1"/>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="C63" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4</v>
+        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <v>6.4875000000000007</v>
       </c>
       <c r="D63" s="1">
         <v>6</v>
@@ -4238,46 +4254,48 @@
         <v>6</v>
       </c>
       <c r="G63" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H63" s="3">
         <v>8.1</v>
       </c>
       <c r="I63" s="3">
-        <v>6</v>
-      </c>
-      <c r="J63" t="e" vm="1">
+        <v>7.7</v>
+      </c>
+      <c r="J63" s="1"/>
+      <c r="K63" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K63" s="1"/>
       <c r="L63" s="1"/>
-      <c r="M63" s="1"/>
+      <c r="M63" s="1" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C64" s="5">
-        <f t="shared" si="1"/>
-        <v>6.3999999999999995</v>
+        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <v>6.4</v>
       </c>
       <c r="D64" s="1">
         <v>6</v>
       </c>
       <c r="E64" s="1">
+        <v>6</v>
+      </c>
+      <c r="F64" s="1">
+        <v>6</v>
+      </c>
+      <c r="G64" s="1">
         <v>5</v>
       </c>
-      <c r="F64" s="1">
-        <v>6</v>
-      </c>
-      <c r="G64" s="1">
-        <v>6</v>
-      </c>
       <c r="H64" s="3">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="I64" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="J64" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4288,66 +4306,66 @@
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C65" s="5">
-        <f t="shared" si="1"/>
-        <v>6.2250000000000005</v>
+        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D65" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E65" s="1">
         <v>5</v>
       </c>
       <c r="F65" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G65" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H65" s="3">
-        <v>8.1999999999999993</v>
+        <v>7.8</v>
       </c>
       <c r="I65" s="3">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="J65" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K65" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K65" s="1"/>
       <c r="L65" s="1"/>
       <c r="M65" s="1"/>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C66" s="5">
-        <f t="shared" si="1"/>
-        <v>6.1750000000000007</v>
+        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <v>6.2250000000000005</v>
       </c>
       <c r="D66" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E66" s="1">
         <v>5</v>
       </c>
       <c r="F66" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G66" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H66" s="3">
-        <v>6.6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I66" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="J66" s="1"/>
+        <v>6.4</v>
+      </c>
+      <c r="J66" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K66" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -4356,62 +4374,62 @@
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C72" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
-        <v>6.1624999999999996</v>
+        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <v>6.1750000000000007</v>
       </c>
       <c r="D67" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E67" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F67" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G67" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H67" s="3">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="I67" s="3">
-        <v>6.3</v>
-      </c>
-      <c r="J67" t="e" vm="1">
+        <v>6.2</v>
+      </c>
+      <c r="J67" s="1"/>
+      <c r="K67" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K67" s="1"/>
       <c r="L67" s="1"/>
       <c r="M67" s="1"/>
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="C68" s="5">
-        <f t="shared" si="2"/>
-        <v>5.9749999999999996</v>
+        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D68" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E68" s="1">
         <v>7</v>
       </c>
       <c r="F68" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G68" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H68" s="3">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="I68" s="3">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="J68" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4422,29 +4440,29 @@
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C69" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7750000000000004</v>
+        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
+        <v>5.9749999999999996</v>
       </c>
       <c r="D69" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E69" s="1">
         <v>7</v>
       </c>
       <c r="F69" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G69" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H69" s="3">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I69" s="3">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="J69" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4455,29 +4473,29 @@
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="C70" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7625000000000002</v>
+        <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
+        <v>5.7750000000000004</v>
       </c>
       <c r="D70" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E70" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F70" s="1">
+        <v>7</v>
+      </c>
+      <c r="G70" s="1">
+        <v>3</v>
+      </c>
+      <c r="H70" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I70" s="3">
         <v>5</v>
-      </c>
-      <c r="G70" s="1">
-        <v>5</v>
-      </c>
-      <c r="H70" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I70" s="3">
-        <v>4.0999999999999996</v>
       </c>
       <c r="J70" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4488,68 +4506,101 @@
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="C71" s="5">
-        <f t="shared" si="2"/>
-        <v>5.4625000000000004</v>
+        <f>AVERAGE(D71,E71,F71,F71,G71,H71,H71,I71)</f>
+        <v>5.7625000000000002</v>
       </c>
       <c r="D71" s="1">
+        <v>8</v>
+      </c>
+      <c r="E71" s="1">
+        <v>8</v>
+      </c>
+      <c r="F71" s="1">
         <v>5</v>
       </c>
-      <c r="E71" s="1">
-        <v>7</v>
-      </c>
-      <c r="F71" s="1">
-        <v>6</v>
-      </c>
       <c r="G71" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H71" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I71" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="I71" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="J71" s="1"/>
+      <c r="J71" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K71" s="1"/>
-      <c r="L71" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72" s="5">
+        <f>AVERAGE(D72,E72,F72,F72,G72,H72,H72,I72)</f>
+        <v>5.4625000000000004</v>
+      </c>
+      <c r="D72" s="1">
+        <v>5</v>
+      </c>
+      <c r="E72" s="1">
+        <v>7</v>
+      </c>
+      <c r="F72" s="1">
+        <v>6</v>
+      </c>
+      <c r="G72" s="1">
+        <v>7</v>
+      </c>
+      <c r="H72" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I72" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J72" s="1"/>
+      <c r="K72" s="1"/>
+      <c r="L72" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B73" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C72" s="5">
-        <f t="shared" si="2"/>
+      <c r="C73" s="5">
+        <f>AVERAGE(D73,E73,F73,F73,G73,H73,H73,I73)</f>
         <v>4.5874999999999995</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D73" s="1">
         <v>2</v>
       </c>
-      <c r="E72" s="1">
+      <c r="E73" s="1">
         <v>4</v>
       </c>
-      <c r="F72" s="1">
+      <c r="F73" s="1">
         <v>2</v>
       </c>
-      <c r="G72" s="1">
+      <c r="G73" s="1">
         <v>5</v>
       </c>
-      <c r="H72" s="3">
+      <c r="H73" s="3">
         <v>7.7</v>
       </c>
-      <c r="I72" s="3">
+      <c r="I73" s="3">
         <v>6.3</v>
       </c>
-      <c r="J72" t="e" vm="1">
+      <c r="J73" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K72" s="1"/>
-      <c r="L72" s="1"/>
-      <c r="M72" s="1"/>
+      <c r="K73" s="1"/>
+      <c r="L73" s="1"/>
+      <c r="M73" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4619,7 +4670,7 @@
         <v>107</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
         <v>8.9250000000000007</v>
       </c>
       <c r="D3" s="1">
@@ -4647,7 +4698,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,E4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.8625000000000007</v>
       </c>
       <c r="D4" s="1">
@@ -4675,7 +4726,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,E5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.85</v>
       </c>
       <c r="D5" s="1">
@@ -4702,7 +4753,7 @@
         <v>79</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,E6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.8375000000000004</v>
       </c>
       <c r="D6" s="1">
@@ -4729,7 +4780,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,E7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.65</v>
       </c>
       <c r="D7" s="1">
@@ -4756,7 +4807,7 @@
         <v>124</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,E8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.625</v>
       </c>
       <c r="D8" s="1">
@@ -4783,7 +4834,7 @@
         <v>121</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,E9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5250000000000004</v>
       </c>
       <c r="D9" s="1">
@@ -4810,7 +4861,7 @@
         <v>127</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,E10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D10" s="1">
@@ -4837,7 +4888,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,E11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D11" s="1">
@@ -4864,7 +4915,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,E12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D12" s="1">
@@ -4891,7 +4942,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,E13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.4375</v>
       </c>
       <c r="D13" s="1">
@@ -4918,7 +4969,7 @@
         <v>96</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,E14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.4124999999999996</v>
       </c>
       <c r="D14" s="1">
@@ -4945,7 +4996,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,E15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3999999999999986</v>
       </c>
       <c r="D15" s="1">
@@ -4972,7 +5023,7 @@
         <v>235</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,E16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.1875</v>
       </c>
       <c r="D16" s="1">
@@ -4999,7 +5050,7 @@
         <v>125</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,E17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.1750000000000007</v>
       </c>
       <c r="D17" s="1">
@@ -5026,7 +5077,7 @@
         <v>81</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,E18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.1624999999999996</v>
       </c>
       <c r="D18" s="1">
@@ -5053,7 +5104,7 @@
         <v>77</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,E19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.15</v>
       </c>
       <c r="D19" s="1">
@@ -5080,7 +5131,7 @@
         <v>54</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,E20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -5107,7 +5158,7 @@
         <v>126</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,E21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8.0750000000000011</v>
       </c>
       <c r="D21" s="1">
@@ -5134,7 +5185,7 @@
         <v>58</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,E22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>8.0625</v>
       </c>
       <c r="D22" s="1">
@@ -5161,7 +5212,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,E23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>7.9249999999999998</v>
       </c>
       <c r="D23" s="1">
@@ -5188,7 +5239,7 @@
         <v>122</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,E24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>7.9124999999999996</v>
       </c>
       <c r="D24" s="1">
@@ -5215,7 +5266,7 @@
         <v>108</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,E25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.8999999999999995</v>
       </c>
       <c r="D25" s="1">
@@ -5242,7 +5293,7 @@
         <v>78</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,E26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.875</v>
       </c>
       <c r="D26" s="1">
@@ -5269,7 +5320,7 @@
         <v>109</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,E27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D27" s="1">
@@ -5296,7 +5347,7 @@
         <v>61</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,E28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D28" s="1">
@@ -5323,7 +5374,7 @@
         <v>193</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,E29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7750000000000004</v>
       </c>
       <c r="D29" s="1">
@@ -5350,7 +5401,7 @@
         <v>60</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,E30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.7375000000000007</v>
       </c>
       <c r="D30" s="1">
@@ -5377,7 +5428,7 @@
         <v>38</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,E31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.7000000000000011</v>
       </c>
       <c r="D31" s="1">
@@ -5404,7 +5455,7 @@
         <v>63</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,E32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.6999999999999993</v>
       </c>
       <c r="D32" s="1">
@@ -5431,7 +5482,7 @@
         <v>123</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,E33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.5874999999999995</v>
       </c>
       <c r="D33" s="1">
@@ -5458,7 +5509,7 @@
         <v>37</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,E34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000011</v>
       </c>
       <c r="D34" s="1">
@@ -5485,7 +5536,7 @@
         <v>67</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
         <v>7.5750000000000002</v>
       </c>
       <c r="D35" s="1">
@@ -5512,7 +5563,7 @@
         <v>62</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,E36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D36" s="1">
@@ -5539,7 +5590,7 @@
         <v>217</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,E37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D37" s="1">
@@ -5566,7 +5617,7 @@
         <v>55</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,E38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.5624999999999991</v>
       </c>
       <c r="D38" s="1">
@@ -5593,7 +5644,7 @@
         <v>201</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,E39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.55</v>
       </c>
       <c r="D39" s="1">
@@ -5620,7 +5671,7 @@
         <v>69</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,E40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D40" s="1">
@@ -5647,7 +5698,7 @@
         <v>132</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,E41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.5125000000000002</v>
       </c>
       <c r="D41" s="1">
@@ -5674,7 +5725,7 @@
         <v>230</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,E42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.5124999999999993</v>
       </c>
       <c r="D42" s="1">
@@ -5701,7 +5752,7 @@
         <v>205</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,E43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.4875000000000007</v>
       </c>
       <c r="D43" s="1">
@@ -5728,7 +5779,7 @@
         <v>172</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,E44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.4749999999999996</v>
       </c>
       <c r="D44" s="1">
@@ -5755,7 +5806,7 @@
         <v>130</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,E45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="D45" s="1">
@@ -5782,7 +5833,7 @@
         <v>97</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,E46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.4375</v>
       </c>
       <c r="D46" s="1">
@@ -5809,7 +5860,7 @@
         <v>100</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.4249999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -5836,7 +5887,7 @@
         <v>244</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.4125000000000005</v>
       </c>
       <c r="D48" s="1">
@@ -5863,7 +5914,7 @@
         <v>131</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.4124999999999996</v>
       </c>
       <c r="D49" s="1">
@@ -5890,7 +5941,7 @@
         <v>220</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999998</v>
       </c>
       <c r="D50" s="1">
@@ -5917,7 +5968,7 @@
         <v>175</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999989</v>
       </c>
       <c r="D51" s="1">
@@ -5944,7 +5995,7 @@
         <v>52</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>7.3500000000000005</v>
       </c>
       <c r="D52" s="1">
@@ -5971,7 +6022,7 @@
         <v>165</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>7.3249999999999993</v>
       </c>
       <c r="D53" s="1">
@@ -5998,7 +6049,7 @@
         <v>224</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>7.3125</v>
       </c>
       <c r="D54" s="1">
@@ -6025,7 +6076,7 @@
         <v>111</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D55" s="1">
@@ -6052,7 +6103,7 @@
         <v>103</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D56" s="1">
@@ -6079,7 +6130,7 @@
         <v>181</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D57" s="1">
@@ -6106,7 +6157,7 @@
         <v>225</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>7.2624999999999993</v>
       </c>
       <c r="D58" s="1">
@@ -6133,7 +6184,7 @@
         <v>147</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>7.2374999999999998</v>
       </c>
       <c r="D59" s="1">
@@ -6160,7 +6211,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>7.2250000000000005</v>
       </c>
       <c r="D60" s="1">
@@ -6187,7 +6238,7 @@
         <v>65</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>7.2125000000000004</v>
       </c>
       <c r="D61" s="1">
@@ -6214,7 +6265,7 @@
         <v>146</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>7.2124999999999995</v>
       </c>
       <c r="D62" s="1">
@@ -6241,7 +6292,7 @@
         <v>94</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>7.1999999999999993</v>
       </c>
       <c r="D63" s="1">
@@ -6268,7 +6319,7 @@
         <v>53</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>7.1499999999999995</v>
       </c>
       <c r="D64" s="1">
@@ -6295,7 +6346,7 @@
         <v>104</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>7.1375000000000011</v>
       </c>
       <c r="D65" s="1">
@@ -6322,7 +6373,7 @@
         <v>40</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>7.1250000000000009</v>
       </c>
       <c r="D66" s="1">
@@ -6349,7 +6400,7 @@
         <v>39</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.125</v>
       </c>
       <c r="D67" s="1">
@@ -6376,7 +6427,7 @@
         <v>133</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D68" s="1">
@@ -6403,7 +6454,7 @@
         <v>98</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D69" s="1">
@@ -6430,7 +6481,7 @@
         <v>171</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D70" s="1">
@@ -6457,7 +6508,7 @@
         <v>110</v>
       </c>
       <c r="C71" s="5">
-        <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D71" s="1">
@@ -6484,7 +6535,7 @@
         <v>143</v>
       </c>
       <c r="C72" s="5">
-        <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D72" s="1">
@@ -6511,7 +6562,7 @@
         <v>177</v>
       </c>
       <c r="C73" s="5">
-        <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
+        <f t="shared" si="2"/>
         <v>7.0749999999999993</v>
       </c>
       <c r="D73" s="1">
@@ -6538,7 +6589,7 @@
         <v>176</v>
       </c>
       <c r="C74" s="5">
-        <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
+        <f t="shared" si="2"/>
         <v>7.05</v>
       </c>
       <c r="D74" s="1">
@@ -6565,7 +6616,7 @@
         <v>221</v>
       </c>
       <c r="C75" s="5">
-        <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
+        <f t="shared" si="2"/>
         <v>7.0250000000000004</v>
       </c>
       <c r="D75" s="1">
@@ -6592,7 +6643,7 @@
         <v>95</v>
       </c>
       <c r="C76" s="5">
-        <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
+        <f t="shared" si="2"/>
         <v>6.9375</v>
       </c>
       <c r="D76" s="1">
@@ -6619,7 +6670,7 @@
         <v>164</v>
       </c>
       <c r="C77" s="5">
-        <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
+        <f t="shared" si="2"/>
         <v>6.9124999999999996</v>
       </c>
       <c r="D77" s="1">
@@ -6646,7 +6697,7 @@
         <v>157</v>
       </c>
       <c r="C78" s="5">
-        <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
+        <f t="shared" si="2"/>
         <v>6.8999999999999995</v>
       </c>
       <c r="D78" s="1">
@@ -6673,7 +6724,7 @@
         <v>88</v>
       </c>
       <c r="C79" s="5">
-        <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D79" s="1">
@@ -6700,7 +6751,7 @@
         <v>184</v>
       </c>
       <c r="C80" s="5">
-        <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D80" s="1">
@@ -6727,7 +6778,7 @@
         <v>119</v>
       </c>
       <c r="C81" s="5">
-        <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
+        <f t="shared" si="2"/>
         <v>6.85</v>
       </c>
       <c r="D81" s="1">
@@ -6754,7 +6805,7 @@
         <v>196</v>
       </c>
       <c r="C82" s="5">
-        <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
+        <f t="shared" si="2"/>
         <v>6.7999999999999989</v>
       </c>
       <c r="D82" s="1">
@@ -6781,7 +6832,7 @@
         <v>57</v>
       </c>
       <c r="C83" s="5">
-        <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
+        <f t="shared" si="2"/>
         <v>6.6999999999999993</v>
       </c>
       <c r="D83" s="1">
@@ -6808,7 +6859,7 @@
         <v>87</v>
       </c>
       <c r="C84" s="5">
-        <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
+        <f t="shared" si="2"/>
         <v>6.6875</v>
       </c>
       <c r="D84" s="1">
@@ -6835,7 +6886,7 @@
         <v>211</v>
       </c>
       <c r="C85" s="5">
-        <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
+        <f t="shared" si="2"/>
         <v>6.6375000000000002</v>
       </c>
       <c r="D85" s="1">
@@ -6862,7 +6913,7 @@
         <v>219</v>
       </c>
       <c r="C86" s="5">
-        <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
+        <f t="shared" si="2"/>
         <v>6.6374999999999993</v>
       </c>
       <c r="D86" s="1">
@@ -6889,7 +6940,7 @@
         <v>41</v>
       </c>
       <c r="C87" s="5">
-        <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
+        <f t="shared" si="2"/>
         <v>6.6124999999999989</v>
       </c>
       <c r="D87" s="1">
@@ -6916,7 +6967,7 @@
         <v>117</v>
       </c>
       <c r="C88" s="5">
-        <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D88" s="1">
@@ -6943,7 +6994,7 @@
         <v>179</v>
       </c>
       <c r="C89" s="5">
-        <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D89" s="1">
@@ -6970,7 +7021,7 @@
         <v>215</v>
       </c>
       <c r="C90" s="5">
-        <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
+        <f t="shared" si="2"/>
         <v>6.5750000000000002</v>
       </c>
       <c r="D90" s="1">
@@ -6997,7 +7048,7 @@
         <v>168</v>
       </c>
       <c r="C91" s="5">
-        <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
+        <f t="shared" si="2"/>
         <v>6.5499999999999989</v>
       </c>
       <c r="D91" s="1">
@@ -7024,7 +7075,7 @@
         <v>197</v>
       </c>
       <c r="C92" s="5">
-        <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
+        <f t="shared" si="2"/>
         <v>6.5375000000000005</v>
       </c>
       <c r="D92" s="1">
@@ -7051,7 +7102,7 @@
         <v>202</v>
       </c>
       <c r="C93" s="5">
-        <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
+        <f t="shared" si="2"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D93" s="1">
@@ -7078,7 +7129,7 @@
         <v>183</v>
       </c>
       <c r="C94" s="5">
-        <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D94" s="1">
@@ -7105,7 +7156,7 @@
         <v>200</v>
       </c>
       <c r="C95" s="5">
-        <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
+        <f t="shared" si="2"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D95" s="1">
@@ -7132,7 +7183,7 @@
         <v>188</v>
       </c>
       <c r="C96" s="5">
-        <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D96" s="1">
@@ -7159,7 +7210,7 @@
         <v>208</v>
       </c>
       <c r="C97" s="5">
-        <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
+        <f t="shared" si="2"/>
         <v>6.35</v>
       </c>
       <c r="D97" s="1">
@@ -7186,7 +7237,7 @@
         <v>134</v>
       </c>
       <c r="C98" s="5">
-        <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
+        <f t="shared" si="2"/>
         <v>6.3125</v>
       </c>
       <c r="D98" s="1">
@@ -7213,7 +7264,7 @@
         <v>144</v>
       </c>
       <c r="C99" s="5">
-        <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
+        <f t="shared" ref="C99:C130" si="3">AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
         <v>6.2749999999999995</v>
       </c>
       <c r="D99" s="1">
@@ -7240,7 +7291,7 @@
         <v>64</v>
       </c>
       <c r="C100" s="5">
-        <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
+        <f t="shared" si="3"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D100" s="1">
@@ -7267,7 +7318,7 @@
         <v>75</v>
       </c>
       <c r="C101" s="5">
-        <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
+        <f t="shared" si="3"/>
         <v>6.2125000000000004</v>
       </c>
       <c r="D101" s="1">
@@ -7294,7 +7345,7 @@
         <v>19</v>
       </c>
       <c r="C102" s="5">
-        <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
+        <f t="shared" si="3"/>
         <v>6.2124999999999995</v>
       </c>
       <c r="D102" s="1">
@@ -7321,7 +7372,7 @@
         <v>101</v>
       </c>
       <c r="C103" s="5">
-        <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
+        <f t="shared" si="3"/>
         <v>6.15</v>
       </c>
       <c r="D103" s="1">
@@ -7348,7 +7399,7 @@
         <v>240</v>
       </c>
       <c r="C104" s="5">
-        <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
+        <f t="shared" si="3"/>
         <v>6.1250000000000009</v>
       </c>
       <c r="D104" s="1">
@@ -7375,7 +7426,7 @@
         <v>158</v>
       </c>
       <c r="C105" s="5">
-        <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
+        <f t="shared" si="3"/>
         <v>6.0874999999999995</v>
       </c>
       <c r="D105" s="1">
@@ -7402,7 +7453,7 @@
         <v>222</v>
       </c>
       <c r="C106" s="5">
-        <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
+        <f t="shared" si="3"/>
         <v>6.0625</v>
       </c>
       <c r="D106" s="1">
@@ -7429,7 +7480,7 @@
         <v>214</v>
       </c>
       <c r="C107" s="5">
-        <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
+        <f t="shared" si="3"/>
         <v>6.0500000000000007</v>
       </c>
       <c r="D107" s="1">
@@ -7456,7 +7507,7 @@
         <v>160</v>
       </c>
       <c r="C108" s="5">
-        <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D108" s="1">
@@ -7483,7 +7534,7 @@
         <v>206</v>
       </c>
       <c r="C109" s="5">
-        <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D109" s="1">
@@ -7510,7 +7561,7 @@
         <v>159</v>
       </c>
       <c r="C110" s="5">
-        <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
+        <f t="shared" si="3"/>
         <v>5.9499999999999993</v>
       </c>
       <c r="D110" s="1">
@@ -7537,7 +7588,7 @@
         <v>195</v>
       </c>
       <c r="C111" s="5">
-        <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
+        <f t="shared" si="3"/>
         <v>5.8875000000000011</v>
       </c>
       <c r="D111" s="1">
@@ -7564,7 +7615,7 @@
         <v>186</v>
       </c>
       <c r="C112" s="5">
-        <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
+        <f t="shared" si="3"/>
         <v>5.8125000000000009</v>
       </c>
       <c r="D112" s="1">
@@ -7591,7 +7642,7 @@
         <v>209</v>
       </c>
       <c r="C113" s="5">
-        <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
+        <f t="shared" si="3"/>
         <v>5.8000000000000007</v>
       </c>
       <c r="D113" s="1">
@@ -7618,7 +7669,7 @@
         <v>113</v>
       </c>
       <c r="C114" s="5">
-        <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
+        <f t="shared" si="3"/>
         <v>5.7374999999999989</v>
       </c>
       <c r="D114" s="1">
@@ -7645,7 +7696,7 @@
         <v>187</v>
       </c>
       <c r="C115" s="5">
-        <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
+        <f t="shared" si="3"/>
         <v>5.7250000000000005</v>
       </c>
       <c r="D115" s="1">
@@ -7672,7 +7723,7 @@
         <v>26</v>
       </c>
       <c r="C116" s="5">
-        <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
+        <f t="shared" si="3"/>
         <v>5.6749999999999998</v>
       </c>
       <c r="D116" s="1">
@@ -7699,7 +7750,7 @@
         <v>149</v>
       </c>
       <c r="C117" s="5">
-        <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D117" s="1">
@@ -7726,7 +7777,7 @@
         <v>156</v>
       </c>
       <c r="C118" s="5">
-        <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D118" s="1">
@@ -7753,7 +7804,7 @@
         <v>229</v>
       </c>
       <c r="C119" s="5">
-        <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
+        <f t="shared" si="3"/>
         <v>5.5375000000000005</v>
       </c>
       <c r="D119" s="1">
@@ -7780,7 +7831,7 @@
         <v>245</v>
       </c>
       <c r="C120" s="5">
-        <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
+        <f t="shared" si="3"/>
         <v>5.5125000000000011</v>
       </c>
       <c r="D120" s="1">
@@ -7807,7 +7858,7 @@
         <v>166</v>
       </c>
       <c r="C121" s="5">
-        <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D121" s="1">
@@ -7834,7 +7885,7 @@
         <v>191</v>
       </c>
       <c r="C122" s="5">
-        <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D122" s="1">
@@ -7861,7 +7912,7 @@
         <v>228</v>
       </c>
       <c r="C123" s="5">
-        <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
+        <f t="shared" si="3"/>
         <v>5.3875000000000011</v>
       </c>
       <c r="D123" s="1">
@@ -7888,7 +7939,7 @@
         <v>204</v>
       </c>
       <c r="C124" s="5">
-        <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
+        <f t="shared" si="3"/>
         <v>5.3750000000000009</v>
       </c>
       <c r="D124" s="1">
@@ -7915,7 +7966,7 @@
         <v>190</v>
       </c>
       <c r="C125" s="5">
-        <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
+        <f t="shared" si="3"/>
         <v>5.375</v>
       </c>
       <c r="D125" s="1">
@@ -7942,7 +7993,7 @@
         <v>182</v>
       </c>
       <c r="C126" s="5">
-        <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
+        <f t="shared" si="3"/>
         <v>5.2875000000000005</v>
       </c>
       <c r="D126" s="1">
@@ -7969,7 +8020,7 @@
         <v>242</v>
       </c>
       <c r="C127" s="5">
-        <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
+        <f t="shared" si="3"/>
         <v>5.25</v>
       </c>
       <c r="D127" s="1">
@@ -7996,7 +8047,7 @@
         <v>232</v>
       </c>
       <c r="C128" s="5">
-        <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
+        <f t="shared" si="3"/>
         <v>5.2</v>
       </c>
       <c r="D128" s="1">
@@ -8023,7 +8074,7 @@
         <v>74</v>
       </c>
       <c r="C129" s="5">
-        <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
+        <f t="shared" si="3"/>
         <v>5.1875</v>
       </c>
       <c r="D129" s="1">
@@ -8050,7 +8101,7 @@
         <v>145</v>
       </c>
       <c r="C130" s="5">
-        <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
+        <f t="shared" si="3"/>
         <v>5.1124999999999998</v>
       </c>
       <c r="D130" s="1">
@@ -8077,7 +8128,7 @@
         <v>223</v>
       </c>
       <c r="C131" s="5">
-        <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
+        <f t="shared" ref="C131:C162" si="4">AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
         <v>5.0750000000000002</v>
       </c>
       <c r="D131" s="1">
@@ -8104,7 +8155,7 @@
         <v>21</v>
       </c>
       <c r="C132" s="5">
-        <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
+        <f t="shared" si="4"/>
         <v>5.05</v>
       </c>
       <c r="D132" s="1">
@@ -8131,7 +8182,7 @@
         <v>203</v>
       </c>
       <c r="C133" s="5">
-        <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
+        <f t="shared" si="4"/>
         <v>4.9875000000000007</v>
       </c>
       <c r="D133" s="1">
@@ -8158,7 +8209,7 @@
         <v>169</v>
       </c>
       <c r="C134" s="5">
-        <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
+        <f t="shared" si="4"/>
         <v>4.9874999999999998</v>
       </c>
       <c r="D134" s="1">
@@ -8185,7 +8236,7 @@
         <v>241</v>
       </c>
       <c r="C135" s="5">
-        <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
+        <f t="shared" si="4"/>
         <v>4.9249999999999998</v>
       </c>
       <c r="D135" s="1">
@@ -8212,7 +8263,7 @@
         <v>163</v>
       </c>
       <c r="C136" s="5">
-        <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
+        <f t="shared" si="4"/>
         <v>4.8499999999999996</v>
       </c>
       <c r="D136" s="1">
@@ -8239,7 +8290,7 @@
         <v>162</v>
       </c>
       <c r="C137" s="5">
-        <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
+        <f t="shared" si="4"/>
         <v>4.7875000000000005</v>
       </c>
       <c r="D137" s="1">
@@ -8266,7 +8317,7 @@
         <v>213</v>
       </c>
       <c r="C138" s="5">
-        <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
+        <f t="shared" si="4"/>
         <v>4.6124999999999998</v>
       </c>
       <c r="D138" s="1">
@@ -8293,7 +8344,7 @@
         <v>154</v>
       </c>
       <c r="C139" s="5">
-        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <f t="shared" si="4"/>
         <v>4.5999999999999996</v>
       </c>
       <c r="D139" s="1">
@@ -8320,7 +8371,7 @@
         <v>135</v>
       </c>
       <c r="C140" s="5">
-        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <f t="shared" si="4"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D140" s="1">
@@ -8347,7 +8398,7 @@
         <v>243</v>
       </c>
       <c r="C141" s="5">
-        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <f t="shared" si="4"/>
         <v>4.5</v>
       </c>
       <c r="D141" s="1">
@@ -8374,7 +8425,7 @@
         <v>161</v>
       </c>
       <c r="C142" s="5">
-        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <f t="shared" si="4"/>
         <v>4.4249999999999998</v>
       </c>
       <c r="D142" s="1">
@@ -8401,7 +8452,7 @@
         <v>114</v>
       </c>
       <c r="C143" s="5">
-        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <f t="shared" si="4"/>
         <v>4.4124999999999996</v>
       </c>
       <c r="D143" s="1">
@@ -8428,7 +8479,7 @@
         <v>207</v>
       </c>
       <c r="C144" s="5">
-        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <f t="shared" si="4"/>
         <v>4.3375000000000004</v>
       </c>
       <c r="D144" s="1">
@@ -8455,7 +8506,7 @@
         <v>150</v>
       </c>
       <c r="C145" s="5">
-        <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
+        <f t="shared" si="4"/>
         <v>4.3374999999999995</v>
       </c>
       <c r="D145" s="1">
@@ -8482,7 +8533,7 @@
         <v>173</v>
       </c>
       <c r="C146" s="5">
-        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <f t="shared" si="4"/>
         <v>4.3125</v>
       </c>
       <c r="D146" s="1">
@@ -8509,7 +8560,7 @@
         <v>212</v>
       </c>
       <c r="C147" s="5">
-        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <f t="shared" si="4"/>
         <v>4.3</v>
       </c>
       <c r="D147" s="1">
@@ -8536,7 +8587,7 @@
         <v>167</v>
       </c>
       <c r="C148" s="5">
-        <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
+        <f t="shared" si="4"/>
         <v>4.2749999999999995</v>
       </c>
       <c r="D148" s="1">
@@ -8563,7 +8614,7 @@
         <v>236</v>
       </c>
       <c r="C149" s="5">
-        <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
+        <f t="shared" si="4"/>
         <v>4.1749999999999998</v>
       </c>
       <c r="D149" s="1">
@@ -8590,7 +8641,7 @@
         <v>233</v>
       </c>
       <c r="C150" s="5">
-        <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
+        <f t="shared" si="4"/>
         <v>4.1625000000000005</v>
       </c>
       <c r="D150" s="1">
@@ -8617,7 +8668,7 @@
         <v>68</v>
       </c>
       <c r="C151" s="5">
-        <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
+        <f t="shared" si="4"/>
         <v>4.1124999999999998</v>
       </c>
       <c r="D151" s="1">
@@ -8644,7 +8695,7 @@
         <v>218</v>
       </c>
       <c r="C152" s="5">
-        <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
+        <f t="shared" si="4"/>
         <v>3.9499999999999997</v>
       </c>
       <c r="D152" s="1">
@@ -8671,7 +8722,7 @@
         <v>199</v>
       </c>
       <c r="C153" s="5">
-        <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
+        <f t="shared" si="4"/>
         <v>3.7375000000000003</v>
       </c>
       <c r="D153" s="1">
@@ -8694,11 +8745,11 @@
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B154" s="9" t="s">
+      <c r="B154" s="2" t="s">
         <v>246</v>
       </c>
       <c r="C154" s="5">
-        <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
+        <f t="shared" si="4"/>
         <v>3.5749999999999997</v>
       </c>
       <c r="D154" s="1">
@@ -8725,7 +8776,7 @@
         <v>180</v>
       </c>
       <c r="C155" s="5">
-        <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
+        <f t="shared" si="4"/>
         <v>3.5625000000000004</v>
       </c>
       <c r="D155" s="1">
@@ -8752,7 +8803,7 @@
         <v>216</v>
       </c>
       <c r="C156" s="5">
-        <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
+        <f t="shared" si="4"/>
         <v>3.5375000000000005</v>
       </c>
       <c r="D156" s="1">
@@ -8779,7 +8830,7 @@
         <v>189</v>
       </c>
       <c r="C157" s="5">
-        <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
+        <f t="shared" si="4"/>
         <v>3.3250000000000002</v>
       </c>
       <c r="D157" s="1">
@@ -8806,7 +8857,7 @@
         <v>194</v>
       </c>
       <c r="C158" s="5">
-        <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
+        <f t="shared" si="4"/>
         <v>3.2749999999999995</v>
       </c>
       <c r="D158" s="1">
@@ -8833,7 +8884,7 @@
         <v>155</v>
       </c>
       <c r="C159" s="5">
-        <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
+        <f t="shared" si="4"/>
         <v>2.9124999999999996</v>
       </c>
       <c r="D159" s="1">
@@ -8860,7 +8911,7 @@
         <v>237</v>
       </c>
       <c r="C160" s="5">
-        <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
+        <f t="shared" si="4"/>
         <v>2.8125</v>
       </c>
       <c r="D160" s="1">
@@ -8887,7 +8938,7 @@
         <v>239</v>
       </c>
       <c r="C161" s="5">
-        <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
+        <f t="shared" si="4"/>
         <v>2.7625000000000002</v>
       </c>
       <c r="D161" s="1">
@@ -8914,7 +8965,7 @@
         <v>174</v>
       </c>
       <c r="C162" s="5">
-        <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
+        <f t="shared" si="4"/>
         <v>2.6375000000000002</v>
       </c>
       <c r="D162" s="1">
@@ -8941,7 +8992,7 @@
         <v>226</v>
       </c>
       <c r="C163" s="5">
-        <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
+        <f t="shared" ref="C163:C194" si="5">AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
         <v>2.5125000000000002</v>
       </c>
       <c r="D163" s="1">

</xml_diff>

<commit_message>
V. 144 "The Creator" & "Abuela Tremenda"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14805AAD-8F54-4796-9DCA-CCC3EDC639AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3775E77-DB00-455E-84A2-2C022F2D96D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -621,7 +621,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="250">
   <si>
     <t>Película</t>
   </si>
@@ -1365,6 +1365,12 @@
   </si>
   <si>
     <t>Muertos S.L.</t>
+  </si>
+  <si>
+    <t>Abuela tremenda</t>
+  </si>
+  <si>
+    <t>The Creator</t>
   </si>
 </sst>
 </file>
@@ -1374,7 +1380,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1410,12 +1416,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1459,7 +1459,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1474,14 +1474,17 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1489,6 +1492,45 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1529,45 +1571,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1694,48 +1697,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M73" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M73" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="B2:M73" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M73">
     <sortCondition descending="1" ref="C2:C73"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I163" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I163" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I163">
-    <sortCondition descending="1" ref="C2:C163"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I165" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="B2:I165" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I165">
+    <sortCondition descending="1" ref="C2:C165"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2237,7 +2240,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="6" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2246,7 +2249,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2273,14 +2276,14 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="8"/>
+      <c r="O3" s="6"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2313,7 +2316,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2340,7 +2343,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="8" t="s">
+      <c r="O5" s="6" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2349,7 +2352,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2378,14 +2381,14 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="8"/>
+      <c r="O6" s="6"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2412,14 +2415,14 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="8"/>
+      <c r="O7" s="6"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2452,7 +2455,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2485,7 +2488,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2518,7 +2521,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2551,7 +2554,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2586,7 +2589,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2621,7 +2624,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2654,7 +2657,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2687,7 +2690,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2722,7 +2725,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2755,7 +2758,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2788,7 +2791,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2821,7 +2824,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2852,7 +2855,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2885,7 +2888,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2918,7 +2921,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2951,7 +2954,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2984,7 +2987,7 @@
         <v>238</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.8874999999999993</v>
       </c>
       <c r="D25" s="1">
@@ -3017,7 +3020,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.8750000000000009</v>
       </c>
       <c r="D26" s="1">
@@ -3050,7 +3053,7 @@
         <v>43</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.8125000000000009</v>
       </c>
       <c r="D27" s="1">
@@ -3083,7 +3086,7 @@
         <v>138</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.8125</v>
       </c>
       <c r="D28" s="1">
@@ -3116,7 +3119,7 @@
         <v>82</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7874999999999996</v>
       </c>
       <c r="D29" s="1">
@@ -3149,7 +3152,7 @@
         <v>73</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.7250000000000005</v>
       </c>
       <c r="D30" s="1">
@@ -3184,7 +3187,7 @@
         <v>142</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3217,7 +3220,7 @@
         <v>192</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.6624999999999996</v>
       </c>
       <c r="D32" s="1">
@@ -3250,7 +3253,7 @@
         <v>47</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.6000000000000005</v>
       </c>
       <c r="D33" s="1">
@@ -3283,7 +3286,7 @@
         <v>198</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5625</v>
       </c>
       <c r="D34" s="1">
@@ -3316,7 +3319,7 @@
         <v>15</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
@@ -3352,7 +3355,7 @@
         <v>210</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D36" s="1">
@@ -3385,7 +3388,7 @@
         <v>105</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
@@ -3420,7 +3423,7 @@
         <v>141</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.5249999999999995</v>
       </c>
       <c r="D38" s="1">
@@ -3453,7 +3456,7 @@
         <v>16</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.4874999999999989</v>
       </c>
       <c r="D39" s="1">
@@ -3485,7 +3488,7 @@
         <v>247</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="D40" s="1">
@@ -3518,7 +3521,7 @@
         <v>50</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.35</v>
       </c>
       <c r="D41" s="1">
@@ -3550,7 +3553,7 @@
         <v>185</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D42" s="1">
@@ -3583,7 +3586,7 @@
         <v>80</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.2500000000000009</v>
       </c>
       <c r="D43" s="1">
@@ -3616,7 +3619,7 @@
         <v>115</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.25</v>
       </c>
       <c r="D44" s="1">
@@ -3649,7 +3652,7 @@
         <v>29</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.2</v>
       </c>
       <c r="D45" s="1">
@@ -3684,7 +3687,7 @@
         <v>22</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.2</v>
       </c>
       <c r="D46" s="1">
@@ -3716,7 +3719,7 @@
         <v>140</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.1875000000000009</v>
       </c>
       <c r="D47" s="1">
@@ -3749,7 +3752,7 @@
         <v>45</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.1875</v>
       </c>
       <c r="D48" s="1">
@@ -3782,7 +3785,7 @@
         <v>27</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.1749999999999998</v>
       </c>
       <c r="D49" s="1">
@@ -3816,7 +3819,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.1749999999999998</v>
       </c>
       <c r="D50" s="1">
@@ -3849,7 +3852,7 @@
         <v>234</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>7.1000000000000005</v>
       </c>
       <c r="D51" s="1">
@@ -3882,7 +3885,7 @@
         <v>227</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D52" s="1">
@@ -3915,7 +3918,7 @@
         <v>231</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D53" s="1">
@@ -3946,7 +3949,7 @@
         <v>71</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>6.9750000000000005</v>
       </c>
       <c r="D54" s="1">
@@ -3981,7 +3984,7 @@
         <v>76</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>6.9</v>
       </c>
       <c r="D55" s="1">
@@ -4014,7 +4017,7 @@
         <v>44</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>6.8750000000000009</v>
       </c>
       <c r="D56" s="1">
@@ -4046,7 +4049,7 @@
         <v>48</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>6.8</v>
       </c>
       <c r="D57" s="1">
@@ -4078,7 +4081,7 @@
         <v>148</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>6.7750000000000004</v>
       </c>
       <c r="D58" s="1">
@@ -4111,7 +4114,7 @@
         <v>153</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>6.75</v>
       </c>
       <c r="D59" s="1">
@@ -4144,7 +4147,7 @@
         <v>17</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>6.7250000000000005</v>
       </c>
       <c r="D60" s="1">
@@ -4176,7 +4179,7 @@
         <v>18</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>6.7</v>
       </c>
       <c r="D61" s="1">
@@ -4208,7 +4211,7 @@
         <v>9</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>6.55</v>
       </c>
       <c r="D62" s="1">
@@ -4241,7 +4244,7 @@
         <v>106</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>6.4875000000000007</v>
       </c>
       <c r="D63" s="1">
@@ -4276,7 +4279,7 @@
         <v>30</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>6.4</v>
       </c>
       <c r="D64" s="1">
@@ -4309,7 +4312,7 @@
         <v>13</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D65" s="1">
@@ -4342,7 +4345,7 @@
         <v>32</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>6.2250000000000005</v>
       </c>
       <c r="D66" s="1">
@@ -4377,7 +4380,7 @@
         <v>42</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>6.1750000000000007</v>
       </c>
       <c r="D67" s="1">
@@ -4410,7 +4413,7 @@
         <v>11</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>6.1624999999999996</v>
       </c>
       <c r="D68" s="1">
@@ -4443,7 +4446,7 @@
         <v>89</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>5.9749999999999996</v>
       </c>
       <c r="D69" s="1">
@@ -4476,7 +4479,7 @@
         <v>99</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>5.7750000000000004</v>
       </c>
       <c r="D70" s="1">
@@ -4509,7 +4512,7 @@
         <v>180</v>
       </c>
       <c r="C71" s="5">
-        <f>AVERAGE(D71,E71,F71,F71,G71,H71,H71,I71)</f>
+        <f t="shared" si="2"/>
         <v>5.7625000000000002</v>
       </c>
       <c r="D71" s="1">
@@ -4542,7 +4545,7 @@
         <v>91</v>
       </c>
       <c r="C72" s="5">
-        <f>AVERAGE(D72,E72,F72,F72,G72,H72,H72,I72)</f>
+        <f t="shared" si="2"/>
         <v>5.4625000000000004</v>
       </c>
       <c r="D72" s="1">
@@ -4574,7 +4577,7 @@
         <v>36</v>
       </c>
       <c r="C73" s="5">
-        <f>AVERAGE(D73,E73,F73,F73,G73,H73,H73,I73)</f>
+        <f t="shared" si="2"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D73" s="1">
@@ -4623,7 +4626,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K163"/>
+  <dimension ref="B2:K165"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4661,7 +4664,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="7" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4670,7 +4673,7 @@
         <v>107</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
+        <f>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
         <v>8.9250000000000007</v>
       </c>
       <c r="D3" s="1">
@@ -4691,14 +4694,14 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="7"/>
+      <c r="K3" s="8"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>66</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D4,E4,E4,F4,G4,H4,H4,I4)</f>
         <v>8.8625000000000007</v>
       </c>
       <c r="D4" s="1">
@@ -4719,14 +4722,14 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="7"/>
+      <c r="K4" s="8"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C5" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D5,E5,E5,F5,G5,H5,H5,I5)</f>
         <v>8.85</v>
       </c>
       <c r="D5" s="1">
@@ -4753,7 +4756,7 @@
         <v>79</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D6,E6,E6,F6,G6,H6,H6,I6)</f>
         <v>8.8375000000000004</v>
       </c>
       <c r="D6" s="1">
@@ -4780,7 +4783,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D7,E7,E7,F7,G7,H7,H7,I7)</f>
         <v>8.65</v>
       </c>
       <c r="D7" s="1">
@@ -4807,7 +4810,7 @@
         <v>124</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D8,E8,E8,F8,G8,H8,H8,I8)</f>
         <v>8.625</v>
       </c>
       <c r="D8" s="1">
@@ -4834,7 +4837,7 @@
         <v>121</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D9,E9,E9,F9,G9,H9,H9,I9)</f>
         <v>8.5250000000000004</v>
       </c>
       <c r="D9" s="1">
@@ -4861,7 +4864,7 @@
         <v>127</v>
       </c>
       <c r="C10" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D10,E10,E10,F10,G10,H10,H10,I10)</f>
         <v>8.5</v>
       </c>
       <c r="D10" s="1">
@@ -4888,7 +4891,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D11,E11,E11,F11,G11,H11,H11,I11)</f>
         <v>8.5</v>
       </c>
       <c r="D11" s="1">
@@ -4915,7 +4918,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D12,E12,E12,F12,G12,H12,H12,I12)</f>
         <v>8.5</v>
       </c>
       <c r="D12" s="1">
@@ -4942,7 +4945,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D13,E13,E13,F13,G13,H13,H13,I13)</f>
         <v>8.4375</v>
       </c>
       <c r="D13" s="1">
@@ -4969,7 +4972,7 @@
         <v>96</v>
       </c>
       <c r="C14" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D14,E14,E14,F14,G14,H14,H14,I14)</f>
         <v>8.4124999999999996</v>
       </c>
       <c r="D14" s="1">
@@ -4996,7 +4999,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D15,E15,E15,F15,G15,H15,H15,I15)</f>
         <v>8.3999999999999986</v>
       </c>
       <c r="D15" s="1">
@@ -5023,7 +5026,7 @@
         <v>235</v>
       </c>
       <c r="C16" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D16,E16,E16,F16,G16,H16,H16,I16)</f>
         <v>8.1875</v>
       </c>
       <c r="D16" s="1">
@@ -5050,7 +5053,7 @@
         <v>125</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D17,E17,E17,F17,G17,H17,H17,I17)</f>
         <v>8.1750000000000007</v>
       </c>
       <c r="D17" s="1">
@@ -5077,7 +5080,7 @@
         <v>81</v>
       </c>
       <c r="C18" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D18,E18,E18,F18,G18,H18,H18,I18)</f>
         <v>8.1624999999999996</v>
       </c>
       <c r="D18" s="1">
@@ -5104,7 +5107,7 @@
         <v>77</v>
       </c>
       <c r="C19" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D19,E19,E19,F19,G19,H19,H19,I19)</f>
         <v>8.15</v>
       </c>
       <c r="D19" s="1">
@@ -5131,7 +5134,7 @@
         <v>54</v>
       </c>
       <c r="C20" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D20,E20,E20,F20,G20,H20,H20,I20)</f>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -5158,7 +5161,7 @@
         <v>126</v>
       </c>
       <c r="C21" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D21,E21,E21,F21,G21,H21,H21,I21)</f>
         <v>8.0750000000000011</v>
       </c>
       <c r="D21" s="1">
@@ -5185,7 +5188,7 @@
         <v>58</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D22,E22,E22,F22,G22,H22,H22,I22)</f>
         <v>8.0625</v>
       </c>
       <c r="D22" s="1">
@@ -5212,7 +5215,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D23,E23,E23,F23,G23,H23,H23,I23)</f>
         <v>7.9249999999999998</v>
       </c>
       <c r="D23" s="1">
@@ -5239,7 +5242,7 @@
         <v>122</v>
       </c>
       <c r="C24" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D24,E24,E24,F24,G24,H24,H24,I24)</f>
         <v>7.9124999999999996</v>
       </c>
       <c r="D24" s="1">
@@ -5266,7 +5269,7 @@
         <v>108</v>
       </c>
       <c r="C25" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D25,E25,E25,F25,G25,H25,H25,I25)</f>
         <v>7.8999999999999995</v>
       </c>
       <c r="D25" s="1">
@@ -5293,7 +5296,7 @@
         <v>78</v>
       </c>
       <c r="C26" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D26,E26,E26,F26,G26,H26,H26,I26)</f>
         <v>7.875</v>
       </c>
       <c r="D26" s="1">
@@ -5320,7 +5323,7 @@
         <v>109</v>
       </c>
       <c r="C27" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D27,E27,E27,F27,G27,H27,H27,I27)</f>
         <v>7.7875000000000005</v>
       </c>
       <c r="D27" s="1">
@@ -5347,7 +5350,7 @@
         <v>61</v>
       </c>
       <c r="C28" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D28,E28,E28,F28,G28,H28,H28,I28)</f>
         <v>7.7875000000000005</v>
       </c>
       <c r="D28" s="1">
@@ -5374,7 +5377,7 @@
         <v>193</v>
       </c>
       <c r="C29" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D29,E29,E29,F29,G29,H29,H29,I29)</f>
         <v>7.7750000000000004</v>
       </c>
       <c r="D29" s="1">
@@ -5401,7 +5404,7 @@
         <v>60</v>
       </c>
       <c r="C30" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D30,E30,E30,F30,G30,H30,H30,I30)</f>
         <v>7.7375000000000007</v>
       </c>
       <c r="D30" s="1">
@@ -5428,7 +5431,7 @@
         <v>38</v>
       </c>
       <c r="C31" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D31,E31,E31,F31,G31,H31,H31,I31)</f>
         <v>7.7000000000000011</v>
       </c>
       <c r="D31" s="1">
@@ -5455,7 +5458,7 @@
         <v>63</v>
       </c>
       <c r="C32" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D32,E32,E32,F32,G32,H32,H32,I32)</f>
         <v>7.6999999999999993</v>
       </c>
       <c r="D32" s="1">
@@ -5482,7 +5485,7 @@
         <v>123</v>
       </c>
       <c r="C33" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D33,E33,E33,F33,G33,H33,H33,I33)</f>
         <v>7.5874999999999995</v>
       </c>
       <c r="D33" s="1">
@@ -5509,7 +5512,7 @@
         <v>37</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D34,E34,E34,F34,G34,H34,H34,I34)</f>
         <v>7.5750000000000011</v>
       </c>
       <c r="D34" s="1">
@@ -5536,7 +5539,7 @@
         <v>67</v>
       </c>
       <c r="C35" s="5">
-        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
+        <f>AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
         <v>7.5750000000000002</v>
       </c>
       <c r="D35" s="1">
@@ -5563,7 +5566,7 @@
         <v>62</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D36,E36,E36,F36,G36,H36,H36,I36)</f>
         <v>7.5625</v>
       </c>
       <c r="D36" s="1">
@@ -5590,7 +5593,7 @@
         <v>217</v>
       </c>
       <c r="C37" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D37,E37,E37,F37,G37,H37,H37,I37)</f>
         <v>7.5625</v>
       </c>
       <c r="D37" s="1">
@@ -5617,7 +5620,7 @@
         <v>55</v>
       </c>
       <c r="C38" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D38,E38,E38,F38,G38,H38,H38,I38)</f>
         <v>7.5624999999999991</v>
       </c>
       <c r="D38" s="1">
@@ -5644,7 +5647,7 @@
         <v>201</v>
       </c>
       <c r="C39" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D39,E39,E39,F39,G39,H39,H39,I39)</f>
         <v>7.55</v>
       </c>
       <c r="D39" s="1">
@@ -5671,7 +5674,7 @@
         <v>69</v>
       </c>
       <c r="C40" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D40,E40,E40,F40,G40,H40,H40,I40)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D40" s="1">
@@ -5698,7 +5701,7 @@
         <v>132</v>
       </c>
       <c r="C41" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D41,E41,E41,F41,G41,H41,H41,I41)</f>
         <v>7.5125000000000002</v>
       </c>
       <c r="D41" s="1">
@@ -5725,7 +5728,7 @@
         <v>230</v>
       </c>
       <c r="C42" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D42,E42,E42,F42,G42,H42,H42,I42)</f>
         <v>7.5124999999999993</v>
       </c>
       <c r="D42" s="1">
@@ -5752,7 +5755,7 @@
         <v>205</v>
       </c>
       <c r="C43" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D43,E43,E43,F43,G43,H43,H43,I43)</f>
         <v>7.4875000000000007</v>
       </c>
       <c r="D43" s="1">
@@ -5779,7 +5782,7 @@
         <v>172</v>
       </c>
       <c r="C44" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D44,E44,E44,F44,G44,H44,H44,I44)</f>
         <v>7.4749999999999996</v>
       </c>
       <c r="D44" s="1">
@@ -5806,7 +5809,7 @@
         <v>130</v>
       </c>
       <c r="C45" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D45,E45,E45,F45,G45,H45,H45,I45)</f>
         <v>7.4625000000000004</v>
       </c>
       <c r="D45" s="1">
@@ -5833,7 +5836,7 @@
         <v>97</v>
       </c>
       <c r="C46" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D46,E46,E46,F46,G46,H46,H46,I46)</f>
         <v>7.4375</v>
       </c>
       <c r="D46" s="1">
@@ -5860,7 +5863,7 @@
         <v>100</v>
       </c>
       <c r="C47" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
         <v>7.4249999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -5887,7 +5890,7 @@
         <v>244</v>
       </c>
       <c r="C48" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
         <v>7.4125000000000005</v>
       </c>
       <c r="D48" s="1">
@@ -5914,7 +5917,7 @@
         <v>131</v>
       </c>
       <c r="C49" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
         <v>7.4124999999999996</v>
       </c>
       <c r="D49" s="1">
@@ -5941,7 +5944,7 @@
         <v>220</v>
       </c>
       <c r="C50" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
         <v>7.3624999999999998</v>
       </c>
       <c r="D50" s="1">
@@ -5968,7 +5971,7 @@
         <v>175</v>
       </c>
       <c r="C51" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
         <v>7.3624999999999989</v>
       </c>
       <c r="D51" s="1">
@@ -5995,7 +5998,7 @@
         <v>52</v>
       </c>
       <c r="C52" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
         <v>7.3500000000000005</v>
       </c>
       <c r="D52" s="1">
@@ -6022,7 +6025,7 @@
         <v>165</v>
       </c>
       <c r="C53" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
         <v>7.3249999999999993</v>
       </c>
       <c r="D53" s="1">
@@ -6049,7 +6052,7 @@
         <v>224</v>
       </c>
       <c r="C54" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
         <v>7.3125</v>
       </c>
       <c r="D54" s="1">
@@ -6076,7 +6079,7 @@
         <v>111</v>
       </c>
       <c r="C55" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
         <v>7.3</v>
       </c>
       <c r="D55" s="1">
@@ -6103,7 +6106,7 @@
         <v>103</v>
       </c>
       <c r="C56" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D56" s="1">
@@ -6130,7 +6133,7 @@
         <v>181</v>
       </c>
       <c r="C57" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D57" s="1">
@@ -6157,7 +6160,7 @@
         <v>225</v>
       </c>
       <c r="C58" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
         <v>7.2624999999999993</v>
       </c>
       <c r="D58" s="1">
@@ -6184,7 +6187,7 @@
         <v>147</v>
       </c>
       <c r="C59" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
         <v>7.2374999999999998</v>
       </c>
       <c r="D59" s="1">
@@ -6211,7 +6214,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
         <v>7.2250000000000005</v>
       </c>
       <c r="D60" s="1">
@@ -6238,7 +6241,7 @@
         <v>65</v>
       </c>
       <c r="C61" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
         <v>7.2125000000000004</v>
       </c>
       <c r="D61" s="1">
@@ -6265,7 +6268,7 @@
         <v>146</v>
       </c>
       <c r="C62" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
         <v>7.2124999999999995</v>
       </c>
       <c r="D62" s="1">
@@ -6292,7 +6295,7 @@
         <v>94</v>
       </c>
       <c r="C63" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
         <v>7.1999999999999993</v>
       </c>
       <c r="D63" s="1">
@@ -6319,7 +6322,7 @@
         <v>53</v>
       </c>
       <c r="C64" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
         <v>7.1499999999999995</v>
       </c>
       <c r="D64" s="1">
@@ -6346,7 +6349,7 @@
         <v>104</v>
       </c>
       <c r="C65" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
         <v>7.1375000000000011</v>
       </c>
       <c r="D65" s="1">
@@ -6373,7 +6376,7 @@
         <v>40</v>
       </c>
       <c r="C66" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
         <v>7.1250000000000009</v>
       </c>
       <c r="D66" s="1">
@@ -6400,7 +6403,7 @@
         <v>39</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
+        <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.125</v>
       </c>
       <c r="D67" s="1">
@@ -6427,7 +6430,7 @@
         <v>133</v>
       </c>
       <c r="C68" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
         <v>7.0875000000000004</v>
       </c>
       <c r="D68" s="1">
@@ -6454,7 +6457,7 @@
         <v>98</v>
       </c>
       <c r="C69" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D69" s="1">
@@ -6481,7 +6484,7 @@
         <v>171</v>
       </c>
       <c r="C70" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D70" s="1">
@@ -6508,7 +6511,7 @@
         <v>110</v>
       </c>
       <c r="C71" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D71" s="1">
@@ -6535,7 +6538,7 @@
         <v>143</v>
       </c>
       <c r="C72" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D72" s="1">
@@ -6562,7 +6565,7 @@
         <v>177</v>
       </c>
       <c r="C73" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
         <v>7.0749999999999993</v>
       </c>
       <c r="D73" s="1">
@@ -6589,7 +6592,7 @@
         <v>176</v>
       </c>
       <c r="C74" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
         <v>7.05</v>
       </c>
       <c r="D74" s="1">
@@ -6616,7 +6619,7 @@
         <v>221</v>
       </c>
       <c r="C75" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
         <v>7.0250000000000004</v>
       </c>
       <c r="D75" s="1">
@@ -6643,7 +6646,7 @@
         <v>95</v>
       </c>
       <c r="C76" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
         <v>6.9375</v>
       </c>
       <c r="D76" s="1">
@@ -6670,7 +6673,7 @@
         <v>164</v>
       </c>
       <c r="C77" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
         <v>6.9124999999999996</v>
       </c>
       <c r="D77" s="1">
@@ -6697,7 +6700,7 @@
         <v>157</v>
       </c>
       <c r="C78" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
         <v>6.8999999999999995</v>
       </c>
       <c r="D78" s="1">
@@ -6724,7 +6727,7 @@
         <v>88</v>
       </c>
       <c r="C79" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
         <v>6.8624999999999989</v>
       </c>
       <c r="D79" s="1">
@@ -6751,7 +6754,7 @@
         <v>184</v>
       </c>
       <c r="C80" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
         <v>6.8624999999999989</v>
       </c>
       <c r="D80" s="1">
@@ -6778,7 +6781,7 @@
         <v>119</v>
       </c>
       <c r="C81" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
         <v>6.85</v>
       </c>
       <c r="D81" s="1">
@@ -6805,7 +6808,7 @@
         <v>196</v>
       </c>
       <c r="C82" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
         <v>6.7999999999999989</v>
       </c>
       <c r="D82" s="1">
@@ -6832,7 +6835,7 @@
         <v>57</v>
       </c>
       <c r="C83" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
         <v>6.6999999999999993</v>
       </c>
       <c r="D83" s="1">
@@ -6859,7 +6862,7 @@
         <v>87</v>
       </c>
       <c r="C84" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
         <v>6.6875</v>
       </c>
       <c r="D84" s="1">
@@ -6886,7 +6889,7 @@
         <v>211</v>
       </c>
       <c r="C85" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
         <v>6.6375000000000002</v>
       </c>
       <c r="D85" s="1">
@@ -6913,7 +6916,7 @@
         <v>219</v>
       </c>
       <c r="C86" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
         <v>6.6374999999999993</v>
       </c>
       <c r="D86" s="1">
@@ -6940,7 +6943,7 @@
         <v>41</v>
       </c>
       <c r="C87" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
         <v>6.6124999999999989</v>
       </c>
       <c r="D87" s="1">
@@ -6967,7 +6970,7 @@
         <v>117</v>
       </c>
       <c r="C88" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D88" s="1">
@@ -6994,7 +6997,7 @@
         <v>179</v>
       </c>
       <c r="C89" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D89" s="1">
@@ -7021,7 +7024,7 @@
         <v>215</v>
       </c>
       <c r="C90" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
         <v>6.5750000000000002</v>
       </c>
       <c r="D90" s="1">
@@ -7044,12 +7047,12 @@
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B91" s="2" t="s">
-        <v>168</v>
+      <c r="B91" s="9" t="s">
+        <v>249</v>
       </c>
       <c r="C91" s="5">
-        <f t="shared" si="2"/>
-        <v>6.5499999999999989</v>
+        <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
+        <v>6.5625</v>
       </c>
       <c r="D91" s="1">
         <v>8</v>
@@ -7061,79 +7064,79 @@
         <v>7</v>
       </c>
       <c r="G91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H91" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I91" s="3">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C92" s="5">
-        <f t="shared" si="2"/>
-        <v>6.5375000000000005</v>
+        <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D92" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E92" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" s="1">
         <v>7</v>
       </c>
       <c r="G92" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H92" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I92" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C93" s="5">
-        <f t="shared" si="2"/>
-        <v>6.3999999999999995</v>
+        <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D93" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E93" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F93" s="1">
         <v>7</v>
       </c>
       <c r="G93" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H93" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I93" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="C94" s="5">
-        <f t="shared" si="2"/>
-        <v>6.3624999999999998</v>
+        <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D94" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E94" s="1">
         <v>6</v>
@@ -7145,25 +7148,25 @@
         <v>7</v>
       </c>
       <c r="H94" s="3">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="I94" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C95" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D95" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E95" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" s="1">
         <v>7</v>
@@ -7172,79 +7175,79 @@
         <v>7</v>
       </c>
       <c r="H95" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I95" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C96" s="5">
-        <f t="shared" si="2"/>
-        <v>6.35</v>
+        <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D96" s="1">
         <v>7</v>
       </c>
       <c r="E96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F96" s="1">
         <v>7</v>
       </c>
       <c r="G96" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H96" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I96" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C97" s="5">
-        <f t="shared" si="2"/>
+        <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
         <v>6.35</v>
       </c>
       <c r="D97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E97" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G97" s="1">
         <v>6</v>
       </c>
       <c r="H97" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I97" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C98" s="5">
-        <f t="shared" si="2"/>
-        <v>6.3125</v>
+        <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
+        <v>6.35</v>
       </c>
       <c r="D98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F98" s="1">
         <v>6</v>
@@ -7253,184 +7256,184 @@
         <v>6</v>
       </c>
       <c r="H98" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I98" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C99" s="5">
-        <f t="shared" ref="C99:C130" si="3">AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.2749999999999995</v>
+        <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
+        <v>6.3125</v>
       </c>
       <c r="D99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E99" s="1">
         <v>6</v>
       </c>
       <c r="F99" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G99" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H99" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I99" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C100" s="5">
-        <f t="shared" si="3"/>
+        <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
         <v>6.2749999999999995</v>
       </c>
       <c r="D100" s="1">
         <v>6</v>
       </c>
       <c r="E100" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H100" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I100" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="C101" s="5">
-        <f t="shared" si="3"/>
-        <v>6.2125000000000004</v>
+        <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D101" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F101" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G101" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H101" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.4</v>
       </c>
       <c r="I101" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C102" s="5">
-        <f t="shared" si="3"/>
-        <v>6.2124999999999995</v>
+        <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D102" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E102" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F102" s="1">
         <v>8</v>
       </c>
       <c r="G102" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H102" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I102" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C103" s="5">
-        <f t="shared" si="3"/>
-        <v>6.15</v>
+        <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D103" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E103" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F103" s="1">
         <v>8</v>
       </c>
       <c r="G103" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H103" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I103" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>240</v>
+        <v>101</v>
       </c>
       <c r="C104" s="5">
-        <f t="shared" si="3"/>
-        <v>6.1250000000000009</v>
+        <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
+        <v>6.15</v>
       </c>
       <c r="D104" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E104" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F104" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G104" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H104" s="3">
-        <v>6.7</v>
+        <v>5</v>
       </c>
       <c r="I104" s="3">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>158</v>
+        <v>240</v>
       </c>
       <c r="C105" s="5">
-        <f t="shared" si="3"/>
-        <v>6.0874999999999995</v>
+        <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D105" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E105" s="1">
         <v>7</v>
@@ -7442,46 +7445,46 @@
         <v>7</v>
       </c>
       <c r="H105" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I105" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C106" s="5">
-        <f t="shared" si="3"/>
-        <v>6.0625</v>
+        <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
       </c>
       <c r="E106" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F106" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G106" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H106" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I106" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C107" s="5">
-        <f t="shared" si="3"/>
-        <v>6.0500000000000007</v>
+        <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
+        <v>6.0625</v>
       </c>
       <c r="D107" s="1">
         <v>7</v>
@@ -7490,25 +7493,25 @@
         <v>6</v>
       </c>
       <c r="F107" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G107" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H107" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I107" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C108" s="5">
-        <f t="shared" si="3"/>
-        <v>6.05</v>
+        <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D108" s="1">
         <v>7</v>
@@ -7520,49 +7523,49 @@
         <v>7</v>
       </c>
       <c r="G108" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H108" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I108" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C109" s="5">
-        <f t="shared" si="3"/>
+        <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
         <v>6.05</v>
       </c>
       <c r="D109" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E109" s="1">
         <v>6</v>
       </c>
       <c r="F109" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G109" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H109" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I109" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C110" s="5">
-        <f t="shared" si="3"/>
-        <v>5.9499999999999993</v>
+        <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
+        <v>6.05</v>
       </c>
       <c r="D110" s="1">
         <v>6</v>
@@ -7571,133 +7574,133 @@
         <v>6</v>
       </c>
       <c r="F110" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G110" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H110" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I110" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C111" s="5">
-        <f t="shared" si="3"/>
-        <v>5.8875000000000011</v>
+        <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D111" s="1">
         <v>6</v>
       </c>
       <c r="E111" s="1">
+        <v>6</v>
+      </c>
+      <c r="F111" s="1">
+        <v>8</v>
+      </c>
+      <c r="G111" s="1">
         <v>5</v>
       </c>
-      <c r="F111" s="1">
-        <v>6</v>
-      </c>
-      <c r="G111" s="1">
-        <v>6</v>
-      </c>
       <c r="H111" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I111" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C112" s="5">
-        <f t="shared" si="3"/>
-        <v>5.8125000000000009</v>
+        <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D112" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E112" s="1">
         <v>5</v>
       </c>
       <c r="F112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G112" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H112" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I112" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C113" s="5">
-        <f t="shared" si="3"/>
-        <v>5.8000000000000007</v>
+        <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D113" s="1">
         <v>7</v>
       </c>
       <c r="E113" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F113" s="1">
         <v>5</v>
       </c>
       <c r="G113" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H113" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I113" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C114" s="5">
-        <f t="shared" si="3"/>
-        <v>5.7374999999999989</v>
+        <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D114" s="1">
         <v>7</v>
       </c>
       <c r="E114" s="1">
+        <v>6</v>
+      </c>
+      <c r="F114" s="1">
         <v>5</v>
       </c>
-      <c r="F114" s="1">
-        <v>4</v>
-      </c>
       <c r="G114" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H114" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I114" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C115" s="5">
-        <f t="shared" si="3"/>
-        <v>5.7250000000000005</v>
+        <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D115" s="1">
         <v>7</v>
@@ -7709,37 +7712,37 @@
         <v>4</v>
       </c>
       <c r="G115" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H115" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I115" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="C116" s="5">
-        <f t="shared" si="3"/>
-        <v>5.6749999999999998</v>
+        <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D116" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E116" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F116" s="1">
+        <v>4</v>
+      </c>
+      <c r="G116" s="1">
         <v>5</v>
       </c>
-      <c r="G116" s="1">
-        <v>6</v>
-      </c>
       <c r="H116" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I116" s="3">
         <v>6.4</v>
@@ -7747,50 +7750,50 @@
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C117" s="5">
-        <f t="shared" si="3"/>
-        <v>5.5624999999999991</v>
+        <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D117" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E117" s="1">
+        <v>3</v>
+      </c>
+      <c r="F117" s="1">
         <v>5</v>
       </c>
-      <c r="F117" s="1">
-        <v>6</v>
-      </c>
       <c r="G117" s="1">
         <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I117" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C118" s="5">
-        <f t="shared" si="3"/>
+        <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D118" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E118" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F118" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G118" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H118" s="3">
         <v>5.8</v>
@@ -7801,26 +7804,26 @@
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>229</v>
+        <v>156</v>
       </c>
       <c r="C119" s="5">
-        <f t="shared" si="3"/>
-        <v>5.5375000000000005</v>
+        <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D119" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E119" s="1">
+        <v>6</v>
+      </c>
+      <c r="F119" s="1">
+        <v>8</v>
+      </c>
+      <c r="G119" s="1">
         <v>5</v>
       </c>
-      <c r="F119" s="1">
-        <v>6</v>
-      </c>
-      <c r="G119" s="1">
-        <v>6</v>
-      </c>
       <c r="H119" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I119" s="3">
         <v>4.9000000000000004</v>
@@ -7828,11 +7831,11 @@
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="C120" s="5">
-        <f t="shared" si="3"/>
-        <v>5.5125000000000011</v>
+        <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D120" s="1">
         <v>6</v>
@@ -7850,22 +7853,22 @@
         <v>5.7</v>
       </c>
       <c r="I120" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>166</v>
+        <v>245</v>
       </c>
       <c r="C121" s="5">
-        <f t="shared" si="3"/>
-        <v>5.4874999999999989</v>
+        <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D121" s="1">
         <v>6</v>
       </c>
       <c r="E121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F121" s="1">
         <v>6</v>
@@ -7874,349 +7877,349 @@
         <v>6</v>
       </c>
       <c r="H121" s="3">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="I121" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C122" s="5">
-        <f t="shared" si="3"/>
+        <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D122" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E122" s="1">
         <v>6</v>
       </c>
       <c r="F122" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G122" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H122" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I122" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>228</v>
+        <v>191</v>
       </c>
       <c r="C123" s="5">
-        <f t="shared" si="3"/>
-        <v>5.3875000000000011</v>
+        <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D123" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E123" s="1">
         <v>6</v>
       </c>
       <c r="F123" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G123" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H123" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I123" s="3">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="C124" s="5">
-        <f t="shared" si="3"/>
-        <v>5.3750000000000009</v>
+        <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D124" s="1">
         <v>6</v>
       </c>
       <c r="E124" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F124" s="1">
         <v>6</v>
       </c>
       <c r="G124" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H124" s="3">
         <v>4.7</v>
       </c>
       <c r="I124" s="3">
-        <v>4.5999999999999996</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C125" s="5">
-        <f t="shared" si="3"/>
-        <v>5.375</v>
+        <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D125" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E125" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F125" s="1">
         <v>6</v>
       </c>
       <c r="G125" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H125" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I125" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C126" s="5">
-        <f t="shared" si="3"/>
-        <v>5.2875000000000005</v>
+        <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
+        <v>5.375</v>
       </c>
       <c r="D126" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E126" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F126" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G126" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H126" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I126" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>242</v>
+        <v>182</v>
       </c>
       <c r="C127" s="5">
-        <f t="shared" si="3"/>
-        <v>5.25</v>
+        <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D127" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E127" s="1">
         <v>5</v>
       </c>
       <c r="F127" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G127" s="1">
         <v>5</v>
       </c>
       <c r="H127" s="3">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="I127" s="3">
-        <v>5.6</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C128" s="5">
-        <f t="shared" si="3"/>
-        <v>5.2</v>
+        <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
+        <v>5.25</v>
       </c>
       <c r="D128" s="1">
         <v>6</v>
       </c>
       <c r="E128" s="1">
+        <v>5</v>
+      </c>
+      <c r="F128" s="1">
         <v>4</v>
-      </c>
-      <c r="F128" s="1">
-        <v>2</v>
       </c>
       <c r="G128" s="1">
         <v>5</v>
       </c>
       <c r="H128" s="3">
-        <v>7.1</v>
+        <v>5.7</v>
       </c>
       <c r="I128" s="3">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>74</v>
+        <v>232</v>
       </c>
       <c r="C129" s="5">
-        <f t="shared" si="3"/>
-        <v>5.1875</v>
+        <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
+        <v>5.2</v>
       </c>
       <c r="D129" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E129" s="1">
+        <v>4</v>
+      </c>
+      <c r="F129" s="1">
+        <v>2</v>
+      </c>
+      <c r="G129" s="1">
         <v>5</v>
       </c>
-      <c r="F129" s="1">
-        <v>6</v>
-      </c>
-      <c r="G129" s="1">
-        <v>6</v>
-      </c>
       <c r="H129" s="3">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="I129" s="3">
-        <v>3.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C130" s="5">
-        <f t="shared" si="3"/>
-        <v>5.1124999999999998</v>
+        <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
+        <v>5.1875</v>
       </c>
       <c r="D130" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E130" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F130" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G130" s="1">
         <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I130" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C131" s="5">
-        <f t="shared" ref="C131:C162" si="4">AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>5.0750000000000002</v>
+        <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E131" s="1">
         <v>4</v>
       </c>
       <c r="F131" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H131" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I131" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C132" s="5">
-        <f t="shared" si="4"/>
-        <v>5.05</v>
+        <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D132" s="1">
         <v>5</v>
       </c>
       <c r="E132" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F132" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G132" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H132" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I132" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C133" s="5">
-        <f t="shared" si="4"/>
-        <v>4.9875000000000007</v>
+        <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
+        <v>5.05</v>
       </c>
       <c r="D133" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E133" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F133" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G133" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H133" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I133" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C134" s="5">
-        <f t="shared" si="4"/>
-        <v>4.9874999999999998</v>
+        <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D134" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E134" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F134" s="1">
         <v>5</v>
@@ -8225,25 +8228,25 @@
         <v>6</v>
       </c>
       <c r="H134" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I134" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>241</v>
+        <v>169</v>
       </c>
       <c r="C135" s="5">
-        <f t="shared" si="4"/>
-        <v>4.9249999999999998</v>
+        <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D135" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E135" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F135" s="1">
         <v>5</v>
@@ -8252,154 +8255,154 @@
         <v>6</v>
       </c>
       <c r="H135" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I135" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>163</v>
+        <v>241</v>
       </c>
       <c r="C136" s="5">
-        <f t="shared" si="4"/>
-        <v>4.8499999999999996</v>
+        <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D136" s="1">
         <v>5</v>
       </c>
       <c r="E136" s="1">
+        <v>4</v>
+      </c>
+      <c r="F136" s="1">
         <v>5</v>
       </c>
-      <c r="F136" s="1">
-        <v>3</v>
-      </c>
       <c r="G136" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H136" s="3">
         <v>5.5</v>
       </c>
       <c r="I136" s="3">
-        <v>4.8</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C137" s="5">
-        <f t="shared" si="4"/>
-        <v>4.7875000000000005</v>
+        <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D137" s="1">
         <v>5</v>
       </c>
       <c r="E137" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F137" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G137" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H137" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I137" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I137" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C138" s="5">
-        <f t="shared" si="4"/>
-        <v>4.6124999999999998</v>
+        <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D138" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E138" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F138" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G138" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H138" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I138" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C139" s="5">
-        <f t="shared" si="4"/>
-        <v>4.5999999999999996</v>
+        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D139" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E139" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F139" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G139" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H139" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I139" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C140" s="5">
-        <f t="shared" si="4"/>
-        <v>4.5874999999999995</v>
+        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D140" s="1">
         <v>5</v>
       </c>
       <c r="E140" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F140" s="1">
         <v>5</v>
       </c>
       <c r="G140" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H140" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I140" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>243</v>
+        <v>135</v>
       </c>
       <c r="C141" s="5">
-        <f t="shared" si="4"/>
-        <v>4.5</v>
+        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D141" s="1">
         <v>5</v>
@@ -8408,322 +8411,322 @@
         <v>4</v>
       </c>
       <c r="F141" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G141" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H141" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I141" s="3">
-        <v>5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>161</v>
+        <v>243</v>
       </c>
       <c r="C142" s="5">
-        <f t="shared" si="4"/>
-        <v>4.4249999999999998</v>
+        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <v>4.5</v>
       </c>
       <c r="D142" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E142" s="1">
         <v>4</v>
       </c>
       <c r="F142" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G142" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H142" s="3">
         <v>5.5</v>
       </c>
       <c r="I142" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C143" s="5">
-        <f t="shared" si="4"/>
-        <v>4.4124999999999996</v>
+        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D143" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E143" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F143" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G143" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H143" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I143" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C144" s="5">
-        <f t="shared" si="4"/>
-        <v>4.3375000000000004</v>
+        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D144" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E144" s="1">
+        <v>0</v>
+      </c>
+      <c r="F144" s="1">
         <v>2</v>
       </c>
-      <c r="F144" s="1">
-        <v>4</v>
-      </c>
       <c r="G144" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H144" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I144" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C145" s="5">
-        <f t="shared" si="4"/>
-        <v>4.3374999999999995</v>
+        <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D145" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E145" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F145" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G145" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H145" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I145" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C146" s="5">
-        <f t="shared" si="4"/>
-        <v>4.3125</v>
+        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D146" s="1">
+        <v>5</v>
+      </c>
+      <c r="E146" s="1">
         <v>3</v>
       </c>
-      <c r="E146" s="1">
-        <v>4</v>
-      </c>
       <c r="F146" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G146" s="1">
         <v>4</v>
       </c>
       <c r="H146" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I146" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>212</v>
+        <v>173</v>
       </c>
       <c r="C147" s="5">
-        <f t="shared" si="4"/>
-        <v>4.3</v>
+        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <v>4.3125</v>
       </c>
       <c r="D147" s="1">
+        <v>3</v>
+      </c>
+      <c r="E147" s="1">
         <v>4</v>
       </c>
-      <c r="E147" s="1">
-        <v>3</v>
-      </c>
       <c r="F147" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G147" s="1">
         <v>4</v>
       </c>
       <c r="H147" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="I147" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C148" s="5">
-        <f t="shared" si="4"/>
-        <v>4.2749999999999995</v>
+        <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
+        <v>4.3</v>
       </c>
       <c r="D148" s="1">
         <v>4</v>
       </c>
       <c r="E148" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F148" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G148" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H148" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I148" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="C149" s="5">
-        <f t="shared" si="4"/>
-        <v>4.1749999999999998</v>
+        <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D149" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E149" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F149" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G149" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H149" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I149" s="3">
-        <v>3.6</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C150" s="5">
-        <f t="shared" si="4"/>
-        <v>4.1625000000000005</v>
+        <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D150" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E150" s="1">
         <v>3</v>
       </c>
       <c r="F150" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G150" s="1">
         <v>4</v>
       </c>
       <c r="H150" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I150" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C151" s="5">
-        <f t="shared" si="4"/>
-        <v>4.1124999999999998</v>
+        <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D151" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E151" s="1">
+        <v>3</v>
+      </c>
+      <c r="F151" s="1">
+        <v>3</v>
+      </c>
+      <c r="G151" s="1">
         <v>4</v>
       </c>
-      <c r="F151" s="1">
-        <v>2</v>
-      </c>
-      <c r="G151" s="1">
-        <v>5</v>
-      </c>
       <c r="H151" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I151" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C152" s="5">
-        <f t="shared" si="4"/>
-        <v>3.9499999999999997</v>
+        <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D152" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E152" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F152" s="1">
         <v>2</v>
       </c>
       <c r="G152" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H152" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I152" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C153" s="5">
-        <f t="shared" si="4"/>
-        <v>3.7375000000000003</v>
+        <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D153" s="1">
         <v>3</v>
@@ -8732,187 +8735,187 @@
         <v>3</v>
       </c>
       <c r="F153" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G153" s="1">
         <v>4</v>
       </c>
       <c r="H153" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I153" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I153" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C154" s="5">
+        <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
+        <v>3.7375000000000003</v>
+      </c>
+      <c r="D154" s="1">
+        <v>3</v>
+      </c>
+      <c r="E154" s="1">
+        <v>3</v>
+      </c>
+      <c r="F154" s="1">
+        <v>3</v>
+      </c>
+      <c r="G154" s="1">
+        <v>4</v>
+      </c>
+      <c r="H154" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="I154" s="3">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="155" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B155" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C154" s="5">
-        <f t="shared" si="4"/>
+      <c r="C155" s="5">
+        <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
         <v>3.5749999999999997</v>
       </c>
-      <c r="D154" s="1">
+      <c r="D155" s="1">
         <v>5</v>
       </c>
-      <c r="E154" s="1">
+      <c r="E155" s="1">
         <v>2</v>
       </c>
-      <c r="F154" s="1">
+      <c r="F155" s="1">
         <v>0</v>
       </c>
-      <c r="G154" s="1">
+      <c r="G155" s="1">
         <v>2</v>
       </c>
-      <c r="H154" s="3">
+      <c r="H155" s="3">
         <v>6.2</v>
       </c>
-      <c r="I154" s="3">
+      <c r="I155" s="3">
         <v>5.2</v>
       </c>
     </row>
-    <row r="155" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B155" s="2">
+    <row r="156" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B156" s="2">
         <v>180</v>
       </c>
-      <c r="C155" s="5">
-        <f t="shared" si="4"/>
+      <c r="C156" s="5">
+        <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
         <v>3.5625000000000004</v>
       </c>
-      <c r="D155" s="1">
+      <c r="D156" s="1">
         <v>3</v>
       </c>
-      <c r="E155" s="1">
+      <c r="E156" s="1">
         <v>3</v>
       </c>
-      <c r="F155" s="1">
+      <c r="F156" s="1">
         <v>3</v>
-      </c>
-      <c r="G155" s="1">
-        <v>3</v>
-      </c>
-      <c r="H155" s="3">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="I155" s="3">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="156" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B156" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C156" s="5">
-        <f t="shared" si="4"/>
-        <v>3.5375000000000005</v>
-      </c>
-      <c r="D156" s="1">
-        <v>5</v>
-      </c>
-      <c r="E156" s="1">
-        <v>2</v>
-      </c>
-      <c r="F156" s="1">
-        <v>2</v>
       </c>
       <c r="G156" s="1">
         <v>3</v>
       </c>
       <c r="H156" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I156" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>189</v>
+        <v>216</v>
       </c>
       <c r="C157" s="5">
-        <f t="shared" si="4"/>
-        <v>3.3250000000000002</v>
+        <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D157" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E157" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F157" s="1">
         <v>2</v>
       </c>
       <c r="G157" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H157" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I157" s="3">
-        <v>5</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B158" s="2" t="s">
-        <v>194</v>
+      <c r="B158" s="9" t="s">
+        <v>248</v>
       </c>
       <c r="C158" s="5">
-        <f t="shared" si="4"/>
-        <v>3.2749999999999995</v>
+        <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
+        <v>3.3375000000000004</v>
       </c>
       <c r="D158" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E158" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F158" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G158" s="1">
         <v>3</v>
       </c>
       <c r="H158" s="3">
-        <v>5.4</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I158" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="C159" s="5">
-        <f t="shared" si="4"/>
-        <v>2.9124999999999996</v>
+        <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D159" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E159" s="1">
         <v>1</v>
       </c>
       <c r="F159" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G159" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H159" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I159" s="3">
-        <v>5.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>237</v>
+        <v>194</v>
       </c>
       <c r="C160" s="5">
-        <f t="shared" si="4"/>
-        <v>2.8125</v>
+        <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D160" s="1">
         <v>2</v>
@@ -8921,79 +8924,79 @@
         <v>2</v>
       </c>
       <c r="F160" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G160" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H160" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="I160" s="3">
-        <v>5.5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>239</v>
+        <v>155</v>
       </c>
       <c r="C161" s="5">
-        <f t="shared" si="4"/>
-        <v>2.7625000000000002</v>
+        <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D161" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E161" s="1">
         <v>1</v>
       </c>
       <c r="F161" s="1">
+        <v>0</v>
+      </c>
+      <c r="G161" s="1">
         <v>1</v>
       </c>
-      <c r="G161" s="1">
-        <v>2</v>
-      </c>
       <c r="H161" s="3">
-        <v>5.5</v>
+        <v>6.7</v>
       </c>
       <c r="I161" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>174</v>
+        <v>237</v>
       </c>
       <c r="C162" s="5">
-        <f t="shared" si="4"/>
-        <v>2.6375000000000002</v>
+        <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
+        <v>2.8125</v>
       </c>
       <c r="D162" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E162" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F162" s="1">
         <v>0</v>
       </c>
       <c r="G162" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H162" s="3">
-        <v>7.6</v>
+        <v>4.5</v>
       </c>
       <c r="I162" s="3">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C163" s="5">
-        <f t="shared" ref="C163:C194" si="5">AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>2.5125000000000002</v>
+        <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D163" s="1">
         <v>2</v>
@@ -9002,15 +9005,69 @@
         <v>1</v>
       </c>
       <c r="F163" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G163" s="1">
         <v>2</v>
       </c>
       <c r="H163" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I163" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="164" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B164" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C164" s="5">
+        <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D164" s="1">
+        <v>0</v>
+      </c>
+      <c r="E164" s="1">
+        <v>0</v>
+      </c>
+      <c r="F164" s="1">
+        <v>0</v>
+      </c>
+      <c r="G164" s="1">
+        <v>0</v>
+      </c>
+      <c r="H164" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I164" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="165" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B165" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C165" s="5">
+        <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
+        <v>2.5125000000000002</v>
+      </c>
+      <c r="D165" s="1">
+        <v>2</v>
+      </c>
+      <c r="E165" s="1">
+        <v>1</v>
+      </c>
+      <c r="F165" s="1">
+        <v>2</v>
+      </c>
+      <c r="G165" s="1">
+        <v>2</v>
+      </c>
+      <c r="H165" s="3">
         <v>4.3</v>
       </c>
-      <c r="I163" s="3">
+      <c r="I165" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 145 "72 horas"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3775E77-DB00-455E-84A2-2C022F2D96D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBD4969-7DFA-4937-9EA6-2E0DDE5F2505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -621,7 +621,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="251">
   <si>
     <t>Película</t>
   </si>
@@ -1371,6 +1371,9 @@
   </si>
   <si>
     <t>The Creator</t>
+  </si>
+  <si>
+    <t>72 horas</t>
   </si>
 </sst>
 </file>
@@ -1474,13 +1477,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1492,45 +1495,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1571,6 +1535,45 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1697,48 +1700,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M73" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M73" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:M73" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M73">
     <sortCondition descending="1" ref="C2:C73"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I165" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I165" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I165">
-    <sortCondition descending="1" ref="C2:C165"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I166" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I166" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I166">
+    <sortCondition descending="1" ref="C2:C166"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2240,7 +2243,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2276,7 +2279,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -2343,7 +2346,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2381,7 +2384,7 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="6"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -2415,7 +2418,7 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="6"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -4380,7 +4383,7 @@
         <v>42</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C73" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>6.1750000000000007</v>
       </c>
       <c r="D67" s="1">
@@ -4626,7 +4629,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K165"/>
+  <dimension ref="B2:K166"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4664,7 +4667,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4694,7 +4697,7 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -4722,7 +4725,7 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -7047,7 +7050,7 @@
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B91" s="9" t="s">
+      <c r="B91" s="2" t="s">
         <v>249</v>
       </c>
       <c r="C91" s="5">
@@ -8775,299 +8778,326 @@
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B155" s="2" t="s">
-        <v>246</v>
+      <c r="B155" s="9" t="s">
+        <v>250</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>3.5749999999999997</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="D155" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E155" s="1">
         <v>2</v>
       </c>
       <c r="F155" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G155" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H155" s="3">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="I155" s="3">
-        <v>5.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B156" s="2">
-        <v>180</v>
+      <c r="B156" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>3.5625000000000004</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D156" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E156" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F156" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G156" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H156" s="3">
-        <v>4.5999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I156" s="3">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B157" s="2" t="s">
-        <v>216</v>
+      <c r="B157" s="2">
+        <v>180</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D157" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E157" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F157" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G157" s="1">
         <v>3</v>
       </c>
       <c r="H157" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I157" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B158" s="9" t="s">
-        <v>248</v>
+      <c r="B158" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>3.3375000000000004</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D158" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E158" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F158" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G158" s="1">
         <v>3</v>
       </c>
       <c r="H158" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="I158" s="3">
         <v>4.0999999999999996</v>
-      </c>
-      <c r="I158" s="3">
-        <v>3.5</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>3.3250000000000002</v>
+        <v>3.3375000000000004</v>
       </c>
       <c r="D159" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E159" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F159" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G159" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H159" s="3">
-        <v>5.8</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I159" s="3">
-        <v>5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D160" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E160" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F160" s="1">
         <v>2</v>
       </c>
       <c r="G160" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H160" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I160" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D161" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E161" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F161" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G161" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H161" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I161" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D162" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E162" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F162" s="1">
         <v>0</v>
       </c>
       <c r="G162" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H162" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I162" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C163" s="5">
         <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D163" s="1">
         <v>2</v>
       </c>
       <c r="E163" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F163" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G163" s="1">
         <v>2</v>
       </c>
       <c r="H163" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I163" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I163" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="164" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B164" s="2" t="s">
-        <v>174</v>
+        <v>239</v>
       </c>
       <c r="C164" s="5">
         <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
-        <v>2.6375000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D164" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E164" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F164" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G164" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H164" s="3">
-        <v>7.6</v>
+        <v>5.5</v>
       </c>
       <c r="I164" s="3">
-        <v>5.9</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="165" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B165" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C165" s="5">
         <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D165" s="1">
+        <v>0</v>
+      </c>
+      <c r="E165" s="1">
+        <v>0</v>
+      </c>
+      <c r="F165" s="1">
+        <v>0</v>
+      </c>
+      <c r="G165" s="1">
+        <v>0</v>
+      </c>
+      <c r="H165" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I165" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="166" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B166" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C166" s="5">
+        <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D165" s="1">
+      <c r="D166" s="1">
         <v>2</v>
       </c>
-      <c r="E165" s="1">
+      <c r="E166" s="1">
         <v>1</v>
       </c>
-      <c r="F165" s="1">
+      <c r="F166" s="1">
         <v>2</v>
       </c>
-      <c r="G165" s="1">
+      <c r="G166" s="1">
         <v>2</v>
       </c>
-      <c r="H165" s="3">
+      <c r="H166" s="3">
         <v>4.3</v>
       </c>
-      <c r="I165" s="3">
+      <c r="I166" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 146 Muchas películas y una serie nuevas
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DBD4969-7DFA-4937-9EA6-2E0DDE5F2505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B166403E-503B-45A9-AE83-A1706ECC4E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,6 +80,7 @@
     <author>tc={3E762906-7E78-4A82-82BD-91226BEEE65F}</author>
     <author>tc={A836A830-A167-47D8-ADFF-FC6A88D1B4AF}</author>
     <author>tc={153818FB-95E4-42BD-AB45-ADAC7CCB6F82}</author>
+    <author>tc={FAC69656-4B66-464B-9367-1002FA156B8A}</author>
     <author>tc={25130372-4D49-4F87-AE9D-9CE5F4E681C1}</author>
     <author>tc={83190950-04EC-4A0B-AFCD-A5040D1110EE}</author>
     <author>tc={05CBDE97-3245-4537-8EC3-A451CBCFADDC}</author>
@@ -426,7 +427,15 @@
     14 temporadas</t>
       </text>
     </comment>
-    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+    <comment ref="B51" authorId="41" shapeId="0" xr:uid="{FAC69656-4B66-464B-9367-1002FA156B8A}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    4 temporadas</t>
+      </text>
+    </comment>
+    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -434,7 +443,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B52" authorId="42" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -442,7 +451,7 @@
     5 temporadas</t>
       </text>
     </comment>
-    <comment ref="B53" authorId="43" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+    <comment ref="B54" authorId="44" shapeId="0" xr:uid="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -450,7 +459,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B54" authorId="44" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+    <comment ref="B55" authorId="45" shapeId="0" xr:uid="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -458,7 +467,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B55" authorId="45" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+    <comment ref="B56" authorId="46" shapeId="0" xr:uid="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -466,7 +475,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B58" authorId="46" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -474,7 +483,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B59" authorId="47" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{96839C2B-31B6-4DC0-88B7-37E650032258}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -482,7 +491,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B60" authorId="48" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+    <comment ref="B61" authorId="49" shapeId="0" xr:uid="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -490,7 +499,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B61" authorId="49" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+    <comment ref="B62" authorId="50" shapeId="0" xr:uid="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -498,7 +507,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B62" authorId="50" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+    <comment ref="B63" authorId="51" shapeId="0" xr:uid="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -506,7 +515,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B68" authorId="51" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -514,7 +523,7 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B69" authorId="52" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -522,7 +531,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -530,7 +539,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -538,7 +547,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+    <comment ref="B73" authorId="56" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -546,7 +555,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B73" authorId="56" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+    <comment ref="B74" authorId="57" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -621,7 +630,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="259">
   <si>
     <t>Película</t>
   </si>
@@ -1374,6 +1383,30 @@
   </si>
   <si>
     <t>72 horas</t>
+  </si>
+  <si>
+    <t>No le digas a mamá que la niñera ha muerto</t>
+  </si>
+  <si>
+    <t>The Amazing Spider-Man</t>
+  </si>
+  <si>
+    <t>Madagascar 2: Escape de África</t>
+  </si>
+  <si>
+    <t>No se desea buena suerte</t>
+  </si>
+  <si>
+    <t>Mamma Mia!</t>
+  </si>
+  <si>
+    <t>The Amazing Spider-Man 2: Rise of Electro</t>
+  </si>
+  <si>
+    <t>El cobrador de deudas</t>
+  </si>
+  <si>
+    <t>Cuerpos especiales (The Heat)</t>
   </si>
 </sst>
 </file>
@@ -1383,7 +1416,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1419,6 +1452,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1700,10 +1739,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M73" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="B2:M73" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M73">
-    <sortCondition descending="1" ref="C2:C73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M74" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="B2:M74" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M74">
+    <sortCondition descending="1" ref="C2:C74"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
@@ -1726,10 +1765,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I166" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I166" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I166">
-    <sortCondition descending="1" ref="C2:C166"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I174" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I174" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I174">
+    <sortCondition descending="1" ref="C2:C174"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -2133,52 +2172,55 @@
   <threadedComment ref="B49" dT="2024-07-08T19:07:51.37" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{153818FB-95E4-42BD-AB45-ADAC7CCB6F82}">
     <text>14 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B51" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
+  <threadedComment ref="B51" dT="2026-08-28T20:56:41.78" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{FAC69656-4B66-464B-9367-1002FA156B8A}">
+    <text>4 temporadas</text>
+  </threadedComment>
+  <threadedComment ref="B52" dT="2026-06-02T15:23:20.11" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25130372-4D49-4F87-AE9D-9CE5F4E681C1}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B52" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
+  <threadedComment ref="B53" dT="2026-05-11T14:15:50.68" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{83190950-04EC-4A0B-AFCD-A5040D1110EE}">
     <text>5 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B53" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
+  <threadedComment ref="B54" dT="2026-05-26T11:52:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{05CBDE97-3245-4537-8EC3-A451CBCFADDC}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B54" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
+  <threadedComment ref="B55" dT="2024-07-08T19:08:59.55" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3D8C30B1-4F7A-4A97-801E-73E85EF747E6}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B55" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
+  <threadedComment ref="B56" dT="2024-07-08T19:09:15.09" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{008FAA73-DE5D-4913-AE22-80AE836D5D61}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B58" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
+  <threadedComment ref="B59" dT="2025-06-14T16:15:11.96" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{5698F250-EDD4-45DE-B2E5-000AD058A767}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B59" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
+  <threadedComment ref="B60" dT="2025-07-02T22:08:33.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{96839C2B-31B6-4DC0-88B7-37E650032258}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B60" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
+  <threadedComment ref="B61" dT="2024-07-08T19:09:40.48" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{AC20EAA3-2085-4F9E-9888-5F2AB1B2897A}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B61" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
+  <threadedComment ref="B62" dT="2024-07-08T19:10:11.66" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{6FEDD623-6837-47F8-9B55-96EB3415266F}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B62" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
+  <threadedComment ref="B63" dT="2024-07-08T19:08:34.89" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B68" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
+  <threadedComment ref="B69" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B69" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+  <threadedComment ref="B70" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B70" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+  <threadedComment ref="B71" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B71" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+  <threadedComment ref="B72" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B72" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+  <threadedComment ref="B73" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B73" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+  <threadedComment ref="B74" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
     <text>4 temporadas</text>
   </threadedComment>
 </ThreadedComments>
@@ -2190,7 +2232,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O73"/>
+  <dimension ref="B2:O74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.140625" customWidth="1"/>
@@ -2252,7 +2294,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
+        <f>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</f>
         <v>9.5250000000000004</v>
       </c>
       <c r="D3" s="1">
@@ -2286,7 +2328,7 @@
         <v>118</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D4,E4,F4,F4,G4,H4,H4,I4)</f>
         <v>8.9749999999999996</v>
       </c>
       <c r="D4" s="1">
@@ -2319,7 +2361,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D5,E5,F5,F5,G5,H5,H5,I5)</f>
         <v>8.6062500000000011</v>
       </c>
       <c r="D5" s="1">
@@ -2355,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D6,E6,F6,F6,G6,H6,H6,I6)</f>
         <v>8.5874999999999986</v>
       </c>
       <c r="D6" s="1">
@@ -2391,7 +2433,7 @@
         <v>112</v>
       </c>
       <c r="C7" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D7,E7,F7,F7,G7,H7,H7,I7)</f>
         <v>8.5750000000000011</v>
       </c>
       <c r="D7" s="1">
@@ -2425,7 +2467,7 @@
         <v>83</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D8,E8,F8,F8,G8,H8,H8,I8)</f>
         <v>8.5125000000000011</v>
       </c>
       <c r="D8" s="1">
@@ -2458,7 +2500,7 @@
         <v>178</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D9,E9,F9,F9,G9,H9,H9,I9)</f>
         <v>8.5124999999999993</v>
       </c>
       <c r="D9" s="1">
@@ -2491,7 +2533,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D10,E10,F10,F10,G10,H10,H10,I10)</f>
         <v>8.4875000000000007</v>
       </c>
       <c r="D10" s="1">
@@ -2524,7 +2566,7 @@
         <v>93</v>
       </c>
       <c r="C11" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D11,E11,F11,F11,G11,H11,H11,I11)</f>
         <v>8.4</v>
       </c>
       <c r="D11" s="1">
@@ -2557,7 +2599,7 @@
         <v>8</v>
       </c>
       <c r="C12" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D12,E12,F12,F12,G12,H12,H12,I12)</f>
         <v>8.3875000000000011</v>
       </c>
       <c r="D12" s="1">
@@ -2592,7 +2634,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D13,E13,F13,F13,G13,H13,H13,I13)</f>
         <v>8.3625000000000007</v>
       </c>
       <c r="D13" s="1">
@@ -2627,7 +2669,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D14,E14,F14,F14,G14,H14,H14,I14)</f>
         <v>8.3624999999999989</v>
       </c>
       <c r="D14" s="1">
@@ -2660,7 +2702,7 @@
         <v>137</v>
       </c>
       <c r="C15" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D15,E15,F15,F15,G15,H15,H15,I15)</f>
         <v>8.3125</v>
       </c>
       <c r="D15" s="1">
@@ -2693,7 +2735,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D16,E16,F16,F16,G16,H16,H16,I16)</f>
         <v>8.2875000000000014</v>
       </c>
       <c r="D16" s="1">
@@ -2728,7 +2770,7 @@
         <v>139</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D17,E17,F17,F17,G17,H17,H17,I17)</f>
         <v>8.2874999999999996</v>
       </c>
       <c r="D17" s="1">
@@ -2761,7 +2803,7 @@
         <v>46</v>
       </c>
       <c r="C18" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D18,E18,F18,F18,G18,H18,H18,I18)</f>
         <v>8.1375000000000011</v>
       </c>
       <c r="D18" s="1">
@@ -2794,7 +2836,7 @@
         <v>136</v>
       </c>
       <c r="C19" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D19,E19,F19,F19,G19,H19,H19,I19)</f>
         <v>8.125</v>
       </c>
       <c r="D19" s="1">
@@ -2827,7 +2869,7 @@
         <v>70</v>
       </c>
       <c r="C20" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D20,E20,F20,F20,G20,H20,H20,I20)</f>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -2858,7 +2900,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D21,E21,F21,F21,G21,H21,H21,I21)</f>
         <v>8</v>
       </c>
       <c r="D21" s="1">
@@ -2891,7 +2933,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D22,E22,F22,F22,G22,H22,H22,I22)</f>
         <v>8</v>
       </c>
       <c r="D22" s="1">
@@ -2924,7 +2966,7 @@
         <v>120</v>
       </c>
       <c r="C23" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D23,E23,F23,F23,G23,H23,H23,I23)</f>
         <v>8</v>
       </c>
       <c r="D23" s="1">
@@ -2957,7 +2999,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D24,E24,F24,F24,G24,H24,H24,I24)</f>
         <v>8</v>
       </c>
       <c r="D24" s="1">
@@ -2990,7 +3032,7 @@
         <v>238</v>
       </c>
       <c r="C25" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D25,E25,F25,F25,G25,H25,H25,I25)</f>
         <v>7.8874999999999993</v>
       </c>
       <c r="D25" s="1">
@@ -3023,7 +3065,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D26,E26,F26,F26,G26,H26,H26,I26)</f>
         <v>7.8750000000000009</v>
       </c>
       <c r="D26" s="1">
@@ -3056,7 +3098,7 @@
         <v>43</v>
       </c>
       <c r="C27" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D27,E27,F27,F27,G27,H27,H27,I27)</f>
         <v>7.8125000000000009</v>
       </c>
       <c r="D27" s="1">
@@ -3089,7 +3131,7 @@
         <v>138</v>
       </c>
       <c r="C28" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D28,E28,F28,F28,G28,H28,H28,I28)</f>
         <v>7.8125</v>
       </c>
       <c r="D28" s="1">
@@ -3122,7 +3164,7 @@
         <v>82</v>
       </c>
       <c r="C29" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D29,E29,F29,F29,G29,H29,H29,I29)</f>
         <v>7.7874999999999996</v>
       </c>
       <c r="D29" s="1">
@@ -3155,7 +3197,7 @@
         <v>73</v>
       </c>
       <c r="C30" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D30,E30,F30,F30,G30,H30,H30,I30)</f>
         <v>7.7250000000000005</v>
       </c>
       <c r="D30" s="1">
@@ -3190,7 +3232,7 @@
         <v>142</v>
       </c>
       <c r="C31" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D31,E31,F31,F31,G31,H31,H31,I31)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D31" s="1">
@@ -3223,7 +3265,7 @@
         <v>192</v>
       </c>
       <c r="C32" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D32,E32,F32,F32,G32,H32,H32,I32)</f>
         <v>7.6624999999999996</v>
       </c>
       <c r="D32" s="1">
@@ -3256,7 +3298,7 @@
         <v>47</v>
       </c>
       <c r="C33" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D33,E33,F33,F33,G33,H33,H33,I33)</f>
         <v>7.6000000000000005</v>
       </c>
       <c r="D33" s="1">
@@ -3289,7 +3331,7 @@
         <v>198</v>
       </c>
       <c r="C34" s="5">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(D34,E34,F34,F34,G34,H34,H34,I34)</f>
         <v>7.5625</v>
       </c>
       <c r="D34" s="1">
@@ -3322,7 +3364,7 @@
         <v>15</v>
       </c>
       <c r="C35" s="5">
-        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
+        <f>AVERAGE(D35,E35,F35,F35,G35,H35,H35,I35)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D35" s="1">
@@ -3358,7 +3400,7 @@
         <v>210</v>
       </c>
       <c r="C36" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D36,E36,F36,F36,G36,H36,H36,I36)</f>
         <v>7.5250000000000004</v>
       </c>
       <c r="D36" s="1">
@@ -3391,7 +3433,7 @@
         <v>105</v>
       </c>
       <c r="C37" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D37,E37,F37,F37,G37,H37,H37,I37)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D37" s="1">
@@ -3426,7 +3468,7 @@
         <v>141</v>
       </c>
       <c r="C38" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D38,E38,F38,F38,G38,H38,H38,I38)</f>
         <v>7.5249999999999995</v>
       </c>
       <c r="D38" s="1">
@@ -3459,7 +3501,7 @@
         <v>16</v>
       </c>
       <c r="C39" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D39,E39,F39,F39,G39,H39,H39,I39)</f>
         <v>7.4874999999999989</v>
       </c>
       <c r="D39" s="1">
@@ -3491,7 +3533,7 @@
         <v>247</v>
       </c>
       <c r="C40" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D40,E40,F40,F40,G40,H40,H40,I40)</f>
         <v>7.4625000000000004</v>
       </c>
       <c r="D40" s="1">
@@ -3524,7 +3566,7 @@
         <v>50</v>
       </c>
       <c r="C41" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D41,E41,F41,F41,G41,H41,H41,I41)</f>
         <v>7.35</v>
       </c>
       <c r="D41" s="1">
@@ -3556,7 +3598,7 @@
         <v>185</v>
       </c>
       <c r="C42" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D42,E42,F42,F42,G42,H42,H42,I42)</f>
         <v>7.3</v>
       </c>
       <c r="D42" s="1">
@@ -3589,7 +3631,7 @@
         <v>80</v>
       </c>
       <c r="C43" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D43,E43,F43,F43,G43,H43,H43,I43)</f>
         <v>7.2500000000000009</v>
       </c>
       <c r="D43" s="1">
@@ -3622,7 +3664,7 @@
         <v>115</v>
       </c>
       <c r="C44" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D44,E44,F44,F44,G44,H44,H44,I44)</f>
         <v>7.25</v>
       </c>
       <c r="D44" s="1">
@@ -3655,7 +3697,7 @@
         <v>29</v>
       </c>
       <c r="C45" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D45,E45,F45,F45,G45,H45,H45,I45)</f>
         <v>7.2</v>
       </c>
       <c r="D45" s="1">
@@ -3690,7 +3732,7 @@
         <v>22</v>
       </c>
       <c r="C46" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D46,E46,F46,F46,G46,H46,H46,I46)</f>
         <v>7.2</v>
       </c>
       <c r="D46" s="1">
@@ -3722,7 +3764,7 @@
         <v>140</v>
       </c>
       <c r="C47" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D47,E47,F47,F47,G47,H47,H47,I47)</f>
         <v>7.1875000000000009</v>
       </c>
       <c r="D47" s="1">
@@ -3755,7 +3797,7 @@
         <v>45</v>
       </c>
       <c r="C48" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D48,E48,F48,F48,G48,H48,H48,I48)</f>
         <v>7.1875</v>
       </c>
       <c r="D48" s="1">
@@ -3788,7 +3830,7 @@
         <v>27</v>
       </c>
       <c r="C49" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D49,E49,F49,F49,G49,H49,H49,I49)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D49" s="1">
@@ -3822,7 +3864,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D50,E50,F50,F50,G50,H50,H50,I50)</f>
         <v>7.1749999999999998</v>
       </c>
       <c r="D50" s="1">
@@ -3852,17 +3894,17 @@
     </row>
     <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C51" s="5">
-        <f t="shared" si="1"/>
-        <v>7.1000000000000005</v>
+        <f>AVERAGE(D51,E51,F51,F51,G51,H51,H51,I51)</f>
+        <v>7.1125000000000007</v>
       </c>
       <c r="D51" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E51" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" s="1">
         <v>8</v>
@@ -3871,10 +3913,10 @@
         <v>5</v>
       </c>
       <c r="H51" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I51" s="3">
         <v>6.7</v>
-      </c>
-      <c r="I51" s="3">
-        <v>5.4</v>
       </c>
       <c r="J51" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3885,29 +3927,29 @@
     </row>
     <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C52" s="5">
-        <f t="shared" si="1"/>
-        <v>7.0875000000000004</v>
+        <f>AVERAGE(D52,E52,F52,F52,G52,H52,H52,I52)</f>
+        <v>7.1000000000000005</v>
       </c>
       <c r="D52" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E52" s="1">
         <v>8</v>
       </c>
       <c r="F52" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G52" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H52" s="3">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="I52" s="3">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="J52" t="e" vm="1">
         <v>#VALUE!</v>
@@ -3918,14 +3960,14 @@
     </row>
     <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C53" s="5">
-        <f t="shared" si="1"/>
+        <f>AVERAGE(D53,E53,F53,F53,G53,H53,H53,I53)</f>
         <v>7.0875000000000004</v>
       </c>
       <c r="D53" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E53" s="1">
         <v>8</v>
@@ -3934,144 +3976,145 @@
         <v>7</v>
       </c>
       <c r="G53" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H53" s="3">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="I53" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="J53" s="1"/>
+        <v>6.3</v>
+      </c>
+      <c r="J53" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
     </row>
     <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>71</v>
+        <v>231</v>
       </c>
       <c r="C54" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9750000000000005</v>
+        <f>AVERAGE(D54,E54,F54,F54,G54,H54,H54,I54)</f>
+        <v>7.0875000000000004</v>
       </c>
       <c r="D54" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E54" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F54" s="1">
         <v>7</v>
       </c>
       <c r="G54" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H54" s="3">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="I54" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J54" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="K54" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+        <v>5.5</v>
+      </c>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
     </row>
     <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C55" s="5">
-        <f t="shared" si="1"/>
-        <v>6.9</v>
+        <f>AVERAGE(D55,E55,F55,F55,G55,H55,H55,I55)</f>
+        <v>6.9750000000000005</v>
       </c>
       <c r="D55" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E55" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F55" s="1">
         <v>7</v>
       </c>
       <c r="G55" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H55" s="3">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="I55" s="3">
-        <v>7.2</v>
+        <v>6.4</v>
       </c>
       <c r="J55" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K55" s="1"/>
+      <c r="K55" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
     </row>
     <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="C56" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8750000000000009</v>
+        <f>AVERAGE(D56,E56,F56,F56,G56,H56,H56,I56)</f>
+        <v>6.9</v>
       </c>
       <c r="D56" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E56" s="1">
         <v>6</v>
       </c>
       <c r="F56" s="1">
+        <v>7</v>
+      </c>
+      <c r="G56" s="1">
         <v>5</v>
       </c>
-      <c r="G56" s="1">
-        <v>7</v>
-      </c>
       <c r="H56" s="3">
-        <v>8.6999999999999993</v>
+        <v>8</v>
       </c>
       <c r="I56" s="3">
-        <v>8.6</v>
-      </c>
-      <c r="J56" s="1"/>
+        <v>7.2</v>
+      </c>
+      <c r="J56" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K56" s="1"/>
-      <c r="L56" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
     </row>
     <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C57" s="5">
-        <f t="shared" si="1"/>
-        <v>6.8</v>
+        <f>AVERAGE(D57,E57,F57,F57,G57,H57,H57,I57)</f>
+        <v>6.8750000000000009</v>
       </c>
       <c r="D57" s="1">
         <v>6</v>
       </c>
       <c r="E57" s="1">
+        <v>6</v>
+      </c>
+      <c r="F57" s="1">
         <v>5</v>
       </c>
-      <c r="F57" s="1">
-        <v>6</v>
-      </c>
       <c r="G57" s="1">
         <v>7</v>
       </c>
       <c r="H57" s="3">
-        <v>8.5</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="I57" s="3">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
@@ -4081,17 +4124,17 @@
     </row>
     <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
       <c r="C58" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7750000000000004</v>
+        <f>AVERAGE(D58,E58,F58,F58,G58,H58,H58,I58)</f>
+        <v>6.8</v>
       </c>
       <c r="D58" s="1">
         <v>6</v>
       </c>
       <c r="E58" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F58" s="1">
         <v>6</v>
@@ -4100,43 +4143,42 @@
         <v>7</v>
       </c>
       <c r="H58" s="3">
-        <v>7.7</v>
+        <v>8.5</v>
       </c>
       <c r="I58" s="3">
-        <v>6.8</v>
-      </c>
-      <c r="J58" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K58" s="1"/>
-      <c r="L58" s="1"/>
-      <c r="M58" s="1"/>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C59" s="5">
-        <f t="shared" si="1"/>
-        <v>6.75</v>
+        <f>AVERAGE(D59,E59,F59,F59,G59,H59,H59,I59)</f>
+        <v>6.7750000000000004</v>
       </c>
       <c r="D59" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E59" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F59" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G59" s="1">
         <v>7</v>
       </c>
       <c r="H59" s="3">
-        <v>5.9</v>
+        <v>7.7</v>
       </c>
       <c r="I59" s="3">
-        <v>4.2</v>
+        <v>6.8</v>
       </c>
       <c r="J59" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4147,61 +4189,62 @@
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="2" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="C60" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7250000000000005</v>
+        <f>AVERAGE(D60,E60,F60,F60,G60,H60,H60,I60)</f>
+        <v>6.75</v>
       </c>
       <c r="D60" s="1">
         <v>8</v>
       </c>
       <c r="E60" s="1">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F60" s="1">
         <v>7</v>
       </c>
       <c r="G60" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H60" s="3">
-        <v>7.7</v>
+        <v>5.9</v>
       </c>
       <c r="I60" s="3">
-        <v>6.4</v>
-      </c>
-      <c r="J60" s="1"/>
+        <v>4.2</v>
+      </c>
+      <c r="J60" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K60" s="1"/>
-      <c r="L60" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C61" s="5">
-        <f t="shared" si="1"/>
-        <v>6.7</v>
+        <f>AVERAGE(D61,E61,F61,F61,G61,H61,H61,I61)</f>
+        <v>6.7250000000000005</v>
       </c>
       <c r="D61" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E61" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F61" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G61" s="1">
         <v>6</v>
       </c>
       <c r="H61" s="3">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
       <c r="I61" s="3">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
@@ -4211,79 +4254,76 @@
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C62" s="5">
-        <f t="shared" si="1"/>
-        <v>6.55</v>
+        <f>AVERAGE(D62,E62,F62,F62,G62,H62,H62,I62)</f>
+        <v>6.7</v>
       </c>
       <c r="D62" s="1">
         <v>5</v>
       </c>
       <c r="E62" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F62" s="1">
         <v>6</v>
       </c>
       <c r="G62" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H62" s="3">
-        <v>7</v>
+        <v>8.6</v>
       </c>
       <c r="I62" s="3">
-        <v>5.4</v>
-      </c>
-      <c r="J62" t="e" vm="1">
+        <v>7.4</v>
+      </c>
+      <c r="J62" s="1"/>
+      <c r="K62" s="1"/>
+      <c r="L62" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="K62" s="1"/>
-      <c r="L62" s="1"/>
-      <c r="M62" s="1"/>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="C63" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4875000000000007</v>
+        <f>AVERAGE(D63,E63,F63,F63,G63,H63,H63,I63)</f>
+        <v>6.55</v>
       </c>
       <c r="D63" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E63" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F63" s="1">
         <v>6</v>
       </c>
       <c r="G63" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H63" s="3">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="I63" s="3">
-        <v>7.7</v>
-      </c>
-      <c r="J63" s="1"/>
-      <c r="K63" t="e" vm="2">
+        <v>5.4</v>
+      </c>
+      <c r="J63" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="K63" s="1"/>
       <c r="L63" s="1"/>
-      <c r="M63" s="1" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+      <c r="M63" s="1"/>
     </row>
     <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="C64" s="5">
-        <f t="shared" si="1"/>
-        <v>6.4</v>
+        <f>AVERAGE(D64,E64,F64,F64,G64,H64,H64,I64)</f>
+        <v>6.4875000000000007</v>
       </c>
       <c r="D64" s="1">
         <v>6</v>
@@ -4295,46 +4335,48 @@
         <v>6</v>
       </c>
       <c r="G64" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H64" s="3">
         <v>8.1</v>
       </c>
       <c r="I64" s="3">
-        <v>6</v>
-      </c>
-      <c r="J64" t="e" vm="1">
+        <v>7.7</v>
+      </c>
+      <c r="J64" s="1"/>
+      <c r="K64" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K64" s="1"/>
       <c r="L64" s="1"/>
-      <c r="M64" s="1"/>
+      <c r="M64" s="1" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C65" s="5">
-        <f t="shared" si="1"/>
-        <v>6.3999999999999995</v>
+        <f>AVERAGE(D65,E65,F65,F65,G65,H65,H65,I65)</f>
+        <v>6.4</v>
       </c>
       <c r="D65" s="1">
         <v>6</v>
       </c>
       <c r="E65" s="1">
+        <v>6</v>
+      </c>
+      <c r="F65" s="1">
+        <v>6</v>
+      </c>
+      <c r="G65" s="1">
         <v>5</v>
       </c>
-      <c r="F65" s="1">
-        <v>6</v>
-      </c>
-      <c r="G65" s="1">
-        <v>6</v>
-      </c>
       <c r="H65" s="3">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="I65" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="J65" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4345,66 +4387,66 @@
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C66" s="5">
-        <f t="shared" si="1"/>
-        <v>6.2250000000000005</v>
+        <f>AVERAGE(D66,E66,F66,F66,G66,H66,H66,I66)</f>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D66" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E66" s="1">
         <v>5</v>
       </c>
       <c r="F66" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G66" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H66" s="3">
-        <v>8.1999999999999993</v>
+        <v>7.8</v>
       </c>
       <c r="I66" s="3">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="J66" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K66" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="K66" s="1"/>
       <c r="L66" s="1"/>
       <c r="M66" s="1"/>
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C73" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
-        <v>6.1750000000000007</v>
+        <f>AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <v>6.2250000000000005</v>
       </c>
       <c r="D67" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E67" s="1">
         <v>5</v>
       </c>
       <c r="F67" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G67" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H67" s="3">
-        <v>6.6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I67" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="J67" s="1"/>
+        <v>6.4</v>
+      </c>
+      <c r="J67" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K67" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -4413,62 +4455,62 @@
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C68" s="5">
-        <f t="shared" si="2"/>
-        <v>6.1624999999999996</v>
+        <f>AVERAGE(D68,E68,F68,F68,G68,H68,H68,I68)</f>
+        <v>6.1750000000000007</v>
       </c>
       <c r="D68" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E68" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F68" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G68" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H68" s="3">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="I68" s="3">
-        <v>6.3</v>
-      </c>
-      <c r="J68" t="e" vm="1">
+        <v>6.2</v>
+      </c>
+      <c r="J68" s="1"/>
+      <c r="K68" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="K68" s="1"/>
       <c r="L68" s="1"/>
       <c r="M68" s="1"/>
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="2" t="s">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="C69" s="5">
-        <f t="shared" si="2"/>
-        <v>5.9749999999999996</v>
+        <f>AVERAGE(D69,E69,F69,F69,G69,H69,H69,I69)</f>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D69" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E69" s="1">
         <v>7</v>
       </c>
       <c r="F69" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G69" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H69" s="3">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="I69" s="3">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="J69" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4479,29 +4521,29 @@
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C70" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7750000000000004</v>
+        <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
+        <v>5.9749999999999996</v>
       </c>
       <c r="D70" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E70" s="1">
         <v>7</v>
       </c>
       <c r="F70" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G70" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H70" s="3">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I70" s="3">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="J70" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4512,29 +4554,29 @@
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="C71" s="5">
-        <f t="shared" si="2"/>
-        <v>5.7625000000000002</v>
+        <f>AVERAGE(D71,E71,F71,F71,G71,H71,H71,I71)</f>
+        <v>5.7750000000000004</v>
       </c>
       <c r="D71" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E71" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" s="1">
+        <v>7</v>
+      </c>
+      <c r="G71" s="1">
+        <v>3</v>
+      </c>
+      <c r="H71" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I71" s="3">
         <v>5</v>
-      </c>
-      <c r="G71" s="1">
-        <v>5</v>
-      </c>
-      <c r="H71" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I71" s="3">
-        <v>4.0999999999999996</v>
       </c>
       <c r="J71" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4545,68 +4587,101 @@
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="C72" s="5">
-        <f t="shared" si="2"/>
-        <v>5.4625000000000004</v>
+        <f>AVERAGE(D72,E72,F72,F72,G72,H72,H72,I72)</f>
+        <v>5.7625000000000002</v>
       </c>
       <c r="D72" s="1">
+        <v>8</v>
+      </c>
+      <c r="E72" s="1">
+        <v>8</v>
+      </c>
+      <c r="F72" s="1">
         <v>5</v>
       </c>
-      <c r="E72" s="1">
-        <v>7</v>
-      </c>
-      <c r="F72" s="1">
-        <v>6</v>
-      </c>
       <c r="G72" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H72" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I72" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="I72" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="J72" s="1"/>
+      <c r="J72" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K72" s="1"/>
-      <c r="L72" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L72" s="1"/>
+      <c r="M72" s="1"/>
     </row>
     <row r="73" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C73" s="5">
+        <f>AVERAGE(D73,E73,F73,F73,G73,H73,H73,I73)</f>
+        <v>5.4625000000000004</v>
+      </c>
+      <c r="D73" s="1">
+        <v>5</v>
+      </c>
+      <c r="E73" s="1">
+        <v>7</v>
+      </c>
+      <c r="F73" s="1">
+        <v>6</v>
+      </c>
+      <c r="G73" s="1">
+        <v>7</v>
+      </c>
+      <c r="H73" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I73" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J73" s="1"/>
+      <c r="K73" s="1"/>
+      <c r="L73" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B74" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C73" s="5">
-        <f t="shared" si="2"/>
+      <c r="C74" s="5">
+        <f>AVERAGE(D74,E74,F74,F74,G74,H74,H74,I74)</f>
         <v>4.5874999999999995</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D74" s="1">
         <v>2</v>
       </c>
-      <c r="E73" s="1">
+      <c r="E74" s="1">
         <v>4</v>
       </c>
-      <c r="F73" s="1">
+      <c r="F74" s="1">
         <v>2</v>
       </c>
-      <c r="G73" s="1">
+      <c r="G74" s="1">
         <v>5</v>
       </c>
-      <c r="H73" s="3">
+      <c r="H74" s="3">
         <v>7.7</v>
       </c>
-      <c r="I73" s="3">
+      <c r="I74" s="3">
         <v>6.3</v>
       </c>
-      <c r="J73" t="e" vm="1">
+      <c r="J74" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K73" s="1"/>
-      <c r="L73" s="1"/>
-      <c r="M73" s="1"/>
+      <c r="K74" s="1"/>
+      <c r="L74" s="1"/>
+      <c r="M74" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4629,7 +4704,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K166"/>
+  <dimension ref="B2:K174"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -6942,147 +7017,147 @@
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B87" s="2" t="s">
-        <v>41</v>
+      <c r="B87" s="9" t="s">
+        <v>255</v>
       </c>
       <c r="C87" s="5">
         <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6124999999999998</v>
       </c>
       <c r="D87" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E87" s="1">
         <v>6</v>
       </c>
       <c r="F87" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G87" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H87" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I87" s="3">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C88" s="5">
         <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D88" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E88" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G88" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H88" s="3">
         <v>6.3</v>
       </c>
       <c r="I88" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
         <v>6.5874999999999995</v>
       </c>
       <c r="D89" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F89" s="1">
         <v>7</v>
       </c>
       <c r="G89" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H89" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I89" s="3">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D90" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E90" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" s="1">
         <v>7</v>
       </c>
       <c r="G90" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H90" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I90" s="3">
-        <v>5.6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>249</v>
+        <v>215</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
-        <v>6.5625</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D91" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F91" s="1">
         <v>7</v>
       </c>
       <c r="G91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H91" s="3">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="I91" s="3">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="2" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C92" s="5">
         <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5625</v>
       </c>
       <c r="D92" s="1">
         <v>8</v>
@@ -7094,79 +7169,79 @@
         <v>7</v>
       </c>
       <c r="G92" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H92" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I92" s="3">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D93" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E93" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" s="1">
         <v>7</v>
       </c>
       <c r="G93" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H93" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I93" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
-        <v>6.3999999999999995</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D94" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F94" s="1">
         <v>7</v>
       </c>
       <c r="G94" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H94" s="3">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="I94" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B95" s="2" t="s">
-        <v>183</v>
+      <c r="B95" s="9" t="s">
+        <v>252</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.3624999999999998</v>
+        <v>6.4749999999999996</v>
       </c>
       <c r="D95" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E95" s="1">
         <v>6</v>
@@ -7178,49 +7253,49 @@
         <v>7</v>
       </c>
       <c r="H95" s="3">
-        <v>5.9</v>
+        <v>7</v>
       </c>
       <c r="I95" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B96" s="2" t="s">
-        <v>200</v>
+      <c r="B96" s="9" t="s">
+        <v>254</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
-        <v>6.3624999999999998</v>
+        <v>6.4124999999999996</v>
       </c>
       <c r="D96" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E96" s="1">
         <v>7</v>
       </c>
       <c r="F96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G96" s="1">
         <v>7</v>
       </c>
       <c r="H96" s="3">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
       <c r="I96" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.35</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D97" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E97" s="1">
         <v>6</v>
@@ -7229,82 +7304,82 @@
         <v>7</v>
       </c>
       <c r="G97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H97" s="3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I97" s="3">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B98" s="2" t="s">
-        <v>208</v>
+      <c r="B98" s="9" t="s">
+        <v>256</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.35</v>
+        <v>6.3625000000000007</v>
       </c>
       <c r="D98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" s="1">
         <v>6</v>
       </c>
       <c r="G98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H98" s="3">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="I98" s="3">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>134</v>
+        <v>183</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.3125</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D99" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E99" s="1">
         <v>6</v>
       </c>
       <c r="F99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H99" s="3">
-        <v>6.9</v>
+        <v>5.9</v>
       </c>
       <c r="I99" s="3">
-        <v>5.7</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F100" s="1">
         <v>7</v>
@@ -7313,208 +7388,208 @@
         <v>7</v>
       </c>
       <c r="H100" s="3">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="I100" s="3">
-        <v>5.6</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>64</v>
+        <v>188</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>6.2749999999999995</v>
+        <v>6.35</v>
       </c>
       <c r="D101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E101" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F101" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G101" s="1">
         <v>6</v>
       </c>
       <c r="H101" s="3">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="I101" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>75</v>
+        <v>208</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
-        <v>6.2125000000000004</v>
+        <v>6.35</v>
       </c>
       <c r="D102" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E102" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F102" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G102" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H102" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.3</v>
       </c>
       <c r="I102" s="3">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>19</v>
+        <v>134</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>6.2124999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D103" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E103" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F103" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G103" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H103" s="3">
-        <v>4.3</v>
+        <v>6.9</v>
       </c>
       <c r="I103" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>101</v>
+        <v>144</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
-        <v>6.15</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D104" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E104" s="1">
         <v>6</v>
       </c>
       <c r="F104" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G104" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H104" s="3">
-        <v>5</v>
+        <v>6.3</v>
       </c>
       <c r="I104" s="3">
-        <v>4.2</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>240</v>
+        <v>64</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>6.1250000000000009</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D105" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E105" s="1">
         <v>7</v>
       </c>
       <c r="F105" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G105" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H105" s="3">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
       <c r="I105" s="3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>158</v>
+        <v>75</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>6.0874999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D106" s="1">
         <v>7</v>
       </c>
       <c r="E106" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F106" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G106" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H106" s="3">
-        <v>4.8</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I106" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>222</v>
+        <v>19</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>6.0625</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D107" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F107" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H107" s="3">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
       <c r="I107" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>214</v>
+        <v>101</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>6.0500000000000007</v>
+        <v>6.15</v>
       </c>
       <c r="D108" s="1">
         <v>7</v>
@@ -7523,13 +7598,13 @@
         <v>6</v>
       </c>
       <c r="F108" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G108" s="1">
         <v>8</v>
       </c>
       <c r="H108" s="3">
-        <v>5.0999999999999996</v>
+        <v>5</v>
       </c>
       <c r="I108" s="3">
         <v>4.2</v>
@@ -7537,17 +7612,17 @@
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>160</v>
+        <v>240</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>6.05</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D109" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E109" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F109" s="1">
         <v>7</v>
@@ -7556,403 +7631,403 @@
         <v>7</v>
       </c>
       <c r="H109" s="3">
-        <v>5.4</v>
+        <v>6.7</v>
       </c>
       <c r="I109" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>206</v>
+        <v>158</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>6.05</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D110" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E110" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F110" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G110" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H110" s="3">
-        <v>6.5</v>
+        <v>4.8</v>
       </c>
       <c r="I110" s="3">
-        <v>5.4</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>159</v>
+        <v>222</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>5.9499999999999993</v>
+        <v>6.0625</v>
       </c>
       <c r="D111" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E111" s="1">
         <v>6</v>
       </c>
       <c r="F111" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G111" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H111" s="3">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="I111" s="3">
-        <v>5</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>5.8875000000000011</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E112" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G112" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H112" s="3">
-        <v>6.7</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I112" s="3">
-        <v>5.7</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>5.8125000000000009</v>
+        <v>6.05</v>
       </c>
       <c r="D113" s="1">
         <v>7</v>
       </c>
       <c r="E113" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F113" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G113" s="1">
         <v>7</v>
       </c>
       <c r="H113" s="3">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="I113" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>5.8000000000000007</v>
+        <v>6.05</v>
       </c>
       <c r="D114" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E114" s="1">
         <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G114" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H114" s="3">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="I114" s="3">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>113</v>
+        <v>159</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>5.7374999999999989</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D115" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E115" s="1">
+        <v>6</v>
+      </c>
+      <c r="F115" s="1">
+        <v>8</v>
+      </c>
+      <c r="G115" s="1">
         <v>5</v>
       </c>
-      <c r="F115" s="1">
-        <v>4</v>
-      </c>
-      <c r="G115" s="1">
-        <v>6</v>
-      </c>
       <c r="H115" s="3">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="I115" s="3">
-        <v>5.3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B116" s="2" t="s">
-        <v>187</v>
+      <c r="B116" s="9" t="s">
+        <v>257</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.7250000000000005</v>
+        <v>5.9250000000000007</v>
       </c>
       <c r="D116" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F116" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116" s="3">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
       <c r="I116" s="3">
-        <v>6.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>26</v>
+        <v>195</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.6749999999999998</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D117" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E117" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
         <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I117" s="3">
-        <v>6.4</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>149</v>
+        <v>186</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.5624999999999991</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E118" s="1">
         <v>5</v>
       </c>
       <c r="F118" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H118" s="3">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="I118" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>156</v>
+        <v>209</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.5624999999999991</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D119" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E119" s="1">
         <v>6</v>
       </c>
       <c r="F119" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G119" s="1">
         <v>5</v>
       </c>
       <c r="H119" s="3">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="I119" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>229</v>
+        <v>113</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.5375000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D120" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E120" s="1">
         <v>5</v>
       </c>
       <c r="F120" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G120" s="1">
         <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>5.7</v>
+        <v>6.8</v>
       </c>
       <c r="I120" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>245</v>
+        <v>187</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.5125000000000011</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D121" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E121" s="1">
         <v>5</v>
       </c>
       <c r="F121" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H121" s="3">
-        <v>5.7</v>
+        <v>6.7</v>
       </c>
       <c r="I121" s="3">
-        <v>4.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B122" s="2" t="s">
-        <v>166</v>
+      <c r="B122" s="9" t="s">
+        <v>253</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.4874999999999989</v>
+        <v>5.6875000000000009</v>
       </c>
       <c r="D122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E122" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G122" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H122" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I122" s="3">
-        <v>4.3</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>191</v>
+        <v>26</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.4874999999999989</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D123" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E123" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F123" s="1">
         <v>5</v>
       </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I123" s="3">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>228</v>
+        <v>149</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.3875000000000011</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D124" s="1">
         <v>6</v>
       </c>
       <c r="E124" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F124" s="1">
         <v>6</v>
@@ -7961,52 +8036,52 @@
         <v>6</v>
       </c>
       <c r="H124" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I124" s="3">
-        <v>3.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>204</v>
+        <v>156</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.3750000000000009</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D125" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E125" s="1">
+        <v>6</v>
+      </c>
+      <c r="F125" s="1">
+        <v>8</v>
+      </c>
+      <c r="G125" s="1">
         <v>5</v>
       </c>
-      <c r="F125" s="1">
-        <v>6</v>
-      </c>
-      <c r="G125" s="1">
-        <v>7</v>
-      </c>
       <c r="H125" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I125" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>190</v>
+        <v>229</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>5.375</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D126" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E126" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
         <v>6</v>
@@ -8015,106 +8090,106 @@
         <v>6</v>
       </c>
       <c r="H126" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="I126" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>182</v>
+        <v>245</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>5.2875000000000005</v>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D127" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E127" s="1">
         <v>5</v>
       </c>
       <c r="F127" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G127" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H127" s="3">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="I127" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>242</v>
+        <v>166</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.25</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D128" s="1">
         <v>6</v>
       </c>
       <c r="E128" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F128" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G128" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H128" s="3">
-        <v>5.7</v>
+        <v>4.8</v>
       </c>
       <c r="I128" s="3">
-        <v>5.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>5.2</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D129" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E129" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F129" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G129" s="1">
         <v>5</v>
       </c>
       <c r="H129" s="3">
-        <v>7.1</v>
+        <v>5.8</v>
       </c>
       <c r="I129" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>74</v>
+        <v>228</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>5.1875</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D130" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E130" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F130" s="1">
         <v>6</v>
@@ -8123,265 +8198,265 @@
         <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="I130" s="3">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>145</v>
+        <v>204</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>5.1124999999999998</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D131" s="1">
         <v>6</v>
       </c>
       <c r="E131" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F131" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H131" s="3">
-        <v>5.9</v>
+        <v>4.7</v>
       </c>
       <c r="I131" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>223</v>
+        <v>190</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>5.0750000000000002</v>
+        <v>5.375</v>
       </c>
       <c r="D132" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E132" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F132" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G132" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H132" s="3">
-        <v>6.3</v>
+        <v>5.6</v>
       </c>
       <c r="I132" s="3">
-        <v>5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>21</v>
+        <v>182</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>5.05</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D133" s="1">
         <v>5</v>
       </c>
       <c r="E133" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F133" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G133" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H133" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I133" s="3">
-        <v>5.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>203</v>
+        <v>242</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>4.9875000000000007</v>
+        <v>5.25</v>
       </c>
       <c r="D134" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E134" s="1">
         <v>5</v>
       </c>
       <c r="F134" s="1">
+        <v>4</v>
+      </c>
+      <c r="G134" s="1">
         <v>5</v>
       </c>
-      <c r="G134" s="1">
-        <v>6</v>
-      </c>
       <c r="H134" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.7</v>
       </c>
       <c r="I134" s="3">
-        <v>3.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>169</v>
+        <v>232</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>4.9874999999999998</v>
+        <v>5.2</v>
       </c>
       <c r="D135" s="1">
         <v>6</v>
       </c>
       <c r="E135" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F135" s="1">
+        <v>2</v>
+      </c>
+      <c r="G135" s="1">
         <v>5</v>
       </c>
-      <c r="G135" s="1">
-        <v>6</v>
-      </c>
       <c r="H135" s="3">
-        <v>6</v>
+        <v>7.1</v>
       </c>
       <c r="I135" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>241</v>
+        <v>74</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>4.9249999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D136" s="1">
+        <v>7</v>
+      </c>
+      <c r="E136" s="1">
         <v>5</v>
       </c>
-      <c r="E136" s="1">
-        <v>4</v>
-      </c>
       <c r="F136" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G136" s="1">
         <v>6</v>
       </c>
       <c r="H136" s="3">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="I136" s="3">
-        <v>4.4000000000000004</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>4.8499999999999996</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E137" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F137" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H137" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I137" s="3">
-        <v>4.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>162</v>
+        <v>223</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>4.7875000000000005</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D138" s="1">
         <v>5</v>
       </c>
       <c r="E138" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F138" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G138" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H138" s="3">
-        <v>4.8</v>
+        <v>6.3</v>
       </c>
       <c r="I138" s="3">
-        <v>3.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>213</v>
+        <v>21</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>4.6124999999999998</v>
+        <v>5.05</v>
       </c>
       <c r="D139" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E139" s="1">
         <v>3</v>
       </c>
       <c r="F139" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G139" s="1">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H139" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I139" s="3">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>154</v>
+        <v>203</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>4.5999999999999996</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D140" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E140" s="1">
         <v>5</v>
@@ -8390,49 +8465,49 @@
         <v>5</v>
       </c>
       <c r="G140" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H140" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I140" s="3">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.5874999999999995</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D141" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E141" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F141" s="1">
         <v>5</v>
       </c>
       <c r="G141" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H141" s="3">
+        <v>6</v>
+      </c>
+      <c r="I141" s="3">
         <v>4.9000000000000004</v>
-      </c>
-      <c r="I141" s="3">
-        <v>3.9</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.5</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D142" s="1">
         <v>5</v>
@@ -8441,34 +8516,34 @@
         <v>4</v>
       </c>
       <c r="F142" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G142" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H142" s="3">
         <v>5.5</v>
       </c>
       <c r="I142" s="3">
-        <v>5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.4249999999999998</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D143" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E143" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F143" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G143" s="1">
         <v>5</v>
@@ -8477,130 +8552,130 @@
         <v>5.5</v>
       </c>
       <c r="I143" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.4124999999999996</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D144" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E144" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F144" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G144" s="1">
         <v>2</v>
       </c>
       <c r="H144" s="3">
-        <v>8.1999999999999993</v>
+        <v>4.8</v>
       </c>
       <c r="I144" s="3">
-        <v>7.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.3375000000000004</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D145" s="1">
+        <v>4</v>
+      </c>
+      <c r="E145" s="1">
         <v>3</v>
-      </c>
-      <c r="E145" s="1">
-        <v>2</v>
       </c>
       <c r="F145" s="1">
         <v>4</v>
       </c>
       <c r="G145" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H145" s="3">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="I145" s="3">
-        <v>4.7</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.3374999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D146" s="1">
         <v>5</v>
       </c>
       <c r="E146" s="1">
+        <v>5</v>
+      </c>
+      <c r="F146" s="1">
+        <v>5</v>
+      </c>
+      <c r="G146" s="1">
         <v>3</v>
       </c>
-      <c r="F146" s="1">
-        <v>3</v>
-      </c>
-      <c r="G146" s="1">
+      <c r="H146" s="3">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I146" s="3">
         <v>4</v>
-      </c>
-      <c r="H146" s="3">
-        <v>5.9</v>
-      </c>
-      <c r="I146" s="3">
-        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>173</v>
+        <v>135</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>4.3125</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D147" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E147" s="1">
         <v>4</v>
       </c>
       <c r="F147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H147" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I147" s="3">
-        <v>4.7</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>212</v>
+        <v>243</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="D148" s="1">
+        <v>5</v>
+      </c>
+      <c r="E148" s="1">
         <v>4</v>
-      </c>
-      <c r="E148" s="1">
-        <v>3</v>
       </c>
       <c r="F148" s="1">
         <v>3</v>
@@ -8609,34 +8684,34 @@
         <v>4</v>
       </c>
       <c r="H148" s="3">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="I148" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>4.2749999999999995</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D149" s="1">
+        <v>1</v>
+      </c>
+      <c r="E149" s="1">
         <v>4</v>
       </c>
-      <c r="E149" s="1">
-        <v>2</v>
-      </c>
       <c r="F149" s="1">
         <v>6</v>
       </c>
       <c r="G149" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H149" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.5</v>
       </c>
       <c r="I149" s="3">
         <v>4.4000000000000004</v>
@@ -8644,53 +8719,53 @@
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>236</v>
+        <v>114</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>4.1749999999999998</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D150" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E150" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F150" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G150" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H150" s="3">
-        <v>5.4</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I150" s="3">
-        <v>3.6</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>233</v>
+        <v>207</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>4.1625000000000005</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D151" s="1">
+        <v>3</v>
+      </c>
+      <c r="E151" s="1">
+        <v>2</v>
+      </c>
+      <c r="F151" s="1">
         <v>4</v>
       </c>
-      <c r="E151" s="1">
-        <v>3</v>
-      </c>
-      <c r="F151" s="1">
-        <v>3</v>
-      </c>
       <c r="G151" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H151" s="3">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="I151" s="3">
         <v>4.7</v>
@@ -8698,98 +8773,98 @@
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>68</v>
+        <v>150</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>4.1124999999999998</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D152" s="1">
         <v>5</v>
       </c>
       <c r="E152" s="1">
+        <v>3</v>
+      </c>
+      <c r="F152" s="1">
+        <v>3</v>
+      </c>
+      <c r="G152" s="1">
         <v>4</v>
       </c>
-      <c r="F152" s="1">
-        <v>2</v>
-      </c>
-      <c r="G152" s="1">
-        <v>5</v>
-      </c>
       <c r="H152" s="3">
-        <v>4.5</v>
+        <v>5.9</v>
       </c>
       <c r="I152" s="3">
-        <v>3.9</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>218</v>
+        <v>173</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>3.9499999999999997</v>
+        <v>4.3125</v>
       </c>
       <c r="D153" s="1">
         <v>3</v>
       </c>
       <c r="E153" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F153" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G153" s="1">
         <v>4</v>
       </c>
       <c r="H153" s="3">
-        <v>5.9</v>
+        <v>5.4</v>
       </c>
       <c r="I153" s="3">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B154" s="2" t="s">
-        <v>199</v>
+      <c r="B154" s="9" t="s">
+        <v>258</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>3.7375000000000003</v>
+        <v>4.3000000000000007</v>
       </c>
       <c r="D154" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E154" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F154" s="1">
         <v>3</v>
       </c>
       <c r="G154" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H154" s="3">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
       <c r="I154" s="3">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B155" s="9" t="s">
-        <v>250</v>
+      <c r="B155" s="2" t="s">
+        <v>212</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>3.6624999999999996</v>
+        <v>4.3</v>
       </c>
       <c r="D155" s="1">
+        <v>4</v>
+      </c>
+      <c r="E155" s="1">
         <v>3</v>
-      </c>
-      <c r="E155" s="1">
-        <v>2</v>
       </c>
       <c r="F155" s="1">
         <v>3</v>
@@ -8798,211 +8873,211 @@
         <v>4</v>
       </c>
       <c r="H155" s="3">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="I155" s="3">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>246</v>
+        <v>167</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>3.5749999999999997</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D156" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E156" s="1">
         <v>2</v>
       </c>
       <c r="F156" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G156" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H156" s="3">
-        <v>6.2</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I156" s="3">
-        <v>5.2</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B157" s="2">
-        <v>180</v>
+      <c r="B157" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>3.5625000000000004</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D157" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E157" s="1">
         <v>3</v>
       </c>
       <c r="F157" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G157" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H157" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.4</v>
       </c>
       <c r="I157" s="3">
-        <v>4.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>3.5375000000000005</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D158" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E158" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F158" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G158" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H158" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.8</v>
       </c>
       <c r="I158" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>248</v>
+        <v>68</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>3.3375000000000004</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D159" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E159" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F159" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G159" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H159" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="I159" s="3">
-        <v>3.5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>189</v>
+        <v>218</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>3.3250000000000002</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D160" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E160" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F160" s="1">
         <v>2</v>
       </c>
       <c r="G160" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H160" s="3">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="I160" s="3">
-        <v>5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>3.2749999999999995</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D161" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E161" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F161" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G161" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H161" s="3">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="I161" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>155</v>
+        <v>250</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
-        <v>2.9124999999999996</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="D162" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E162" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F162" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G162" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H162" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I162" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C163" s="5">
         <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>2.8125</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D163" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E163" s="1">
         <v>2</v>
@@ -9014,90 +9089,306 @@
         <v>2</v>
       </c>
       <c r="H163" s="3">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
       <c r="I163" s="3">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="164" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B164" s="2" t="s">
-        <v>239</v>
+      <c r="B164" s="2">
+        <v>180</v>
       </c>
       <c r="C164" s="5">
         <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
-        <v>2.7625000000000002</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D164" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E164" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F164" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G164" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H164" s="3">
-        <v>5.5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I164" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="165" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B165" s="2" t="s">
-        <v>174</v>
+        <v>216</v>
       </c>
       <c r="C165" s="5">
         <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
-        <v>2.6375000000000002</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D165" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E165" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F165" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G165" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H165" s="3">
-        <v>7.6</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I165" s="3">
-        <v>5.9</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="166" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B166" s="2" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
       <c r="C166" s="5">
         <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
+        <v>3.3375000000000004</v>
+      </c>
+      <c r="D166" s="1">
+        <v>3</v>
+      </c>
+      <c r="E166" s="1">
+        <v>3</v>
+      </c>
+      <c r="F166" s="1">
+        <v>3</v>
+      </c>
+      <c r="G166" s="1">
+        <v>3</v>
+      </c>
+      <c r="H166" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I166" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="167" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B167" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C167" s="5">
+        <f>AVERAGE(D167,E167,E167,F167,G167,H167,H167,I167)</f>
+        <v>3.3250000000000002</v>
+      </c>
+      <c r="D167" s="1">
+        <v>4</v>
+      </c>
+      <c r="E167" s="1">
+        <v>1</v>
+      </c>
+      <c r="F167" s="1">
+        <v>2</v>
+      </c>
+      <c r="G167" s="1">
+        <v>2</v>
+      </c>
+      <c r="H167" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="I167" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="168" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B168" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C168" s="5">
+        <f>AVERAGE(D168,E168,E168,F168,G168,H168,H168,I168)</f>
+        <v>3.2749999999999995</v>
+      </c>
+      <c r="D168" s="1">
+        <v>2</v>
+      </c>
+      <c r="E168" s="1">
+        <v>2</v>
+      </c>
+      <c r="F168" s="1">
+        <v>2</v>
+      </c>
+      <c r="G168" s="1">
+        <v>3</v>
+      </c>
+      <c r="H168" s="3">
+        <v>5.4</v>
+      </c>
+      <c r="I168" s="3">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="169" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B169" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C169" s="5">
+        <f>AVERAGE(D169,E169,E169,F169,G169,H169,H169,I169)</f>
+        <v>2.9124999999999996</v>
+      </c>
+      <c r="D169" s="1">
+        <v>1</v>
+      </c>
+      <c r="E169" s="1">
+        <v>1</v>
+      </c>
+      <c r="F169" s="1">
+        <v>0</v>
+      </c>
+      <c r="G169" s="1">
+        <v>1</v>
+      </c>
+      <c r="H169" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I169" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="170" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B170" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C170" s="5">
+        <f>AVERAGE(D170,E170,E170,F170,G170,H170,H170,I170)</f>
+        <v>2.8125</v>
+      </c>
+      <c r="D170" s="1">
+        <v>2</v>
+      </c>
+      <c r="E170" s="1">
+        <v>2</v>
+      </c>
+      <c r="F170" s="1">
+        <v>0</v>
+      </c>
+      <c r="G170" s="1">
+        <v>2</v>
+      </c>
+      <c r="H170" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I170" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="171" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B171" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C171" s="5">
+        <f>AVERAGE(D171,E171,E171,F171,G171,H171,H171,I171)</f>
+        <v>2.7625000000000002</v>
+      </c>
+      <c r="D171" s="1">
+        <v>2</v>
+      </c>
+      <c r="E171" s="1">
+        <v>1</v>
+      </c>
+      <c r="F171" s="1">
+        <v>1</v>
+      </c>
+      <c r="G171" s="1">
+        <v>2</v>
+      </c>
+      <c r="H171" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I171" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="172" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B172" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="C172" s="5">
+        <f>AVERAGE(D172,E172,E172,F172,G172,H172,H172,I172)</f>
+        <v>2.65</v>
+      </c>
+      <c r="D172" s="1">
+        <v>3</v>
+      </c>
+      <c r="E172" s="1">
+        <v>1</v>
+      </c>
+      <c r="F172" s="1">
+        <v>2</v>
+      </c>
+      <c r="G172" s="1">
+        <v>2</v>
+      </c>
+      <c r="H172" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="I172" s="3">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="173" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B173" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C173" s="5">
+        <f>AVERAGE(D173,E173,E173,F173,G173,H173,H173,I173)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D173" s="1">
+        <v>0</v>
+      </c>
+      <c r="E173" s="1">
+        <v>0</v>
+      </c>
+      <c r="F173" s="1">
+        <v>0</v>
+      </c>
+      <c r="G173" s="1">
+        <v>0</v>
+      </c>
+      <c r="H173" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I173" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="174" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B174" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C174" s="5">
+        <f>AVERAGE(D174,E174,E174,F174,G174,H174,H174,I174)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D166" s="1">
+      <c r="D174" s="1">
         <v>2</v>
       </c>
-      <c r="E166" s="1">
+      <c r="E174" s="1">
         <v>1</v>
       </c>
-      <c r="F166" s="1">
+      <c r="F174" s="1">
         <v>2</v>
       </c>
-      <c r="G166" s="1">
+      <c r="G174" s="1">
         <v>2</v>
       </c>
-      <c r="H166" s="3">
+      <c r="H174" s="3">
         <v>4.3</v>
       </c>
-      <c r="I166" s="3">
+      <c r="I174" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 147 "I Will Find You"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B166403E-503B-45A9-AE83-A1706ECC4E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51770A0F-8CCB-41B3-9CB0-11135367D985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -92,6 +92,7 @@
     <author>tc={6FEDD623-6837-47F8-9B55-96EB3415266F}</author>
     <author>tc={B9AA30C0-3BCC-4842-ABCD-15892A9A17A4}</author>
     <author>tc={ED84D32D-B87E-494D-BC5A-D963B24A65B4}</author>
+    <author>tc={3F7F4075-15C7-4FE0-888B-70BAAFC86B7F}</author>
     <author>tc={25B82680-662E-4149-A9D4-D7D343B29E09}</author>
     <author>tc={8D955452-5474-4D7F-9EFB-C317CB8E77C7}</author>
     <author>tc={3955FC3A-5089-4113-A6FF-7CA6DD36C98F}</author>
@@ -523,7 +524,15 @@
     7 temporadas</t>
       </text>
     </comment>
-    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+    <comment ref="B70" authorId="53" shapeId="0" xr:uid="{3F7F4075-15C7-4FE0-888B-70BAAFC86B7F}">
+      <text>
+        <t>[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+    1 temporada</t>
+      </text>
+    </comment>
+    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{25B82680-662E-4149-A9D4-D7D343B29E09}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -531,7 +540,7 @@
     3 temporadas</t>
       </text>
     </comment>
-    <comment ref="B71" authorId="54" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -539,7 +548,7 @@
     4 temporadas</t>
       </text>
     </comment>
-    <comment ref="B72" authorId="55" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+    <comment ref="B73" authorId="56" shapeId="0" xr:uid="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -547,7 +556,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B73" authorId="56" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+    <comment ref="B74" authorId="57" shapeId="0" xr:uid="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -555,7 +564,7 @@
     1 temporada</t>
       </text>
     </comment>
-    <comment ref="B74" authorId="57" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+    <comment ref="B75" authorId="58" shapeId="0" xr:uid="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -630,7 +639,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="260">
   <si>
     <t>Película</t>
   </si>
@@ -1407,6 +1416,9 @@
   </si>
   <si>
     <t>Cuerpos especiales (The Heat)</t>
+  </si>
+  <si>
+    <t>I Will Find You</t>
   </si>
 </sst>
 </file>
@@ -1457,7 +1469,7 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1501,7 +1513,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1524,9 +1536,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1739,10 +1748,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M74" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="B2:M74" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M74">
-    <sortCondition descending="1" ref="C2:C74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M75" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="B2:M75" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M75">
+    <sortCondition descending="1" ref="C2:C75"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
@@ -2208,19 +2217,22 @@
   <threadedComment ref="B69" dT="2024-07-08T19:10:27.18" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{ED84D32D-B87E-494D-BC5A-D963B24A65B4}">
     <text>7 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B70" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
+  <threadedComment ref="B70" dT="2026-08-30T16:24:36.80" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3F7F4075-15C7-4FE0-888B-70BAAFC86B7F}">
+    <text>1 temporada</text>
+  </threadedComment>
+  <threadedComment ref="B71" dT="2024-07-08T18:58:56.17" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{25B82680-662E-4149-A9D4-D7D343B29E09}">
     <text>3 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B71" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
+  <threadedComment ref="B72" dT="2024-10-02T22:28:33.03" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{8D955452-5474-4D7F-9EFB-C317CB8E77C7}">
     <text>4 temporadas</text>
   </threadedComment>
-  <threadedComment ref="B72" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
+  <threadedComment ref="B73" dT="2025-10-07T18:49:36.71" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{3955FC3A-5089-4113-A6FF-7CA6DD36C98F}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B73" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
+  <threadedComment ref="B74" dT="2024-07-09T17:54:39.57" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{C6F778D8-6F01-47AB-B632-8939C5C0B507}">
     <text>1 temporada</text>
   </threadedComment>
-  <threadedComment ref="B74" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
+  <threadedComment ref="B75" dT="2024-07-08T19:10:55.56" personId="{2E232528-F057-4355-8D9E-53D77C4311A2}" id="{B1297543-A2F2-4625-BBB2-C2604CA16AED}">
     <text>4 temporadas</text>
   </threadedComment>
 </ThreadedComments>
@@ -2232,7 +2244,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:O74"/>
+  <dimension ref="B2:O75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.140625" customWidth="1"/>
@@ -4521,29 +4533,29 @@
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>89</v>
+        <v>259</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,F70,F70,G70,H70,H70,I70)</f>
-        <v>5.9749999999999996</v>
+        <v>6.15</v>
       </c>
       <c r="D70" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E70" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F70" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G70" s="1">
         <v>6</v>
       </c>
       <c r="H70" s="3">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="I70" s="3">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="J70" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4554,29 +4566,29 @@
     </row>
     <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,F71,F71,G71,H71,H71,I71)</f>
-        <v>5.7750000000000004</v>
+        <v>5.9749999999999996</v>
       </c>
       <c r="D71" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E71" s="1">
         <v>7</v>
       </c>
       <c r="F71" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G71" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H71" s="3">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="I71" s="3">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="J71" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4587,29 +4599,29 @@
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>180</v>
+        <v>99</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,F72,F72,G72,H72,H72,I72)</f>
-        <v>5.7625000000000002</v>
+        <v>5.7750000000000004</v>
       </c>
       <c r="D72" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E72" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F72" s="1">
+        <v>7</v>
+      </c>
+      <c r="G72" s="1">
+        <v>3</v>
+      </c>
+      <c r="H72" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="I72" s="3">
         <v>5</v>
-      </c>
-      <c r="G72" s="1">
-        <v>5</v>
-      </c>
-      <c r="H72" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I72" s="3">
-        <v>4.0999999999999996</v>
       </c>
       <c r="J72" t="e" vm="1">
         <v>#VALUE!</v>
@@ -4620,68 +4632,101 @@
     </row>
     <row r="73" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,F73,F73,G73,H73,H73,I73)</f>
-        <v>5.4625000000000004</v>
+        <v>5.7625000000000002</v>
       </c>
       <c r="D73" s="1">
+        <v>8</v>
+      </c>
+      <c r="E73" s="1">
+        <v>8</v>
+      </c>
+      <c r="F73" s="1">
         <v>5</v>
       </c>
-      <c r="E73" s="1">
-        <v>7</v>
-      </c>
-      <c r="F73" s="1">
-        <v>6</v>
-      </c>
       <c r="G73" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H73" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I73" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="I73" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="J73" s="1"/>
+      <c r="J73" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="K73" s="1"/>
-      <c r="L73" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="L73" s="1"/>
+      <c r="M73" s="1"/>
     </row>
     <row r="74" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
-        <v>36</v>
+        <v>91</v>
       </c>
       <c r="C74" s="5">
         <f>AVERAGE(D74,E74,F74,F74,G74,H74,H74,I74)</f>
+        <v>5.4625000000000004</v>
+      </c>
+      <c r="D74" s="1">
+        <v>5</v>
+      </c>
+      <c r="E74" s="1">
+        <v>7</v>
+      </c>
+      <c r="F74" s="1">
+        <v>6</v>
+      </c>
+      <c r="G74" s="1">
+        <v>7</v>
+      </c>
+      <c r="H74" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="I74" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J74" s="1"/>
+      <c r="K74" s="1"/>
+      <c r="L74" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B75" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C75" s="5">
+        <f>AVERAGE(D75,E75,F75,F75,G75,H75,H75,I75)</f>
         <v>4.5874999999999995</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D75" s="1">
         <v>2</v>
       </c>
-      <c r="E74" s="1">
+      <c r="E75" s="1">
         <v>4</v>
       </c>
-      <c r="F74" s="1">
+      <c r="F75" s="1">
         <v>2</v>
       </c>
-      <c r="G74" s="1">
+      <c r="G75" s="1">
         <v>5</v>
       </c>
-      <c r="H74" s="3">
+      <c r="H75" s="3">
         <v>7.7</v>
       </c>
-      <c r="I74" s="3">
+      <c r="I75" s="3">
         <v>6.3</v>
       </c>
-      <c r="J74" t="e" vm="1">
+      <c r="J75" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="K74" s="1"/>
-      <c r="L74" s="1"/>
-      <c r="M74" s="1"/>
+      <c r="K75" s="1"/>
+      <c r="L75" s="1"/>
+      <c r="M75" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4751,7 +4796,7 @@
         <v>107</v>
       </c>
       <c r="C3" s="5">
-        <f>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
+        <f t="shared" ref="C3:C34" si="0">AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</f>
         <v>8.9250000000000007</v>
       </c>
       <c r="D3" s="1">
@@ -4779,7 +4824,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="5">
-        <f>AVERAGE(D4,E4,E4,F4,G4,H4,H4,I4)</f>
+        <f t="shared" si="0"/>
         <v>8.8625000000000007</v>
       </c>
       <c r="D4" s="1">
@@ -4807,7 +4852,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="5">
-        <f>AVERAGE(D5,E5,E5,F5,G5,H5,H5,I5)</f>
+        <f t="shared" si="0"/>
         <v>8.85</v>
       </c>
       <c r="D5" s="1">
@@ -4834,7 +4879,7 @@
         <v>79</v>
       </c>
       <c r="C6" s="5">
-        <f>AVERAGE(D6,E6,E6,F6,G6,H6,H6,I6)</f>
+        <f t="shared" si="0"/>
         <v>8.8375000000000004</v>
       </c>
       <c r="D6" s="1">
@@ -4861,7 +4906,7 @@
         <v>128</v>
       </c>
       <c r="C7" s="5">
-        <f>AVERAGE(D7,E7,E7,F7,G7,H7,H7,I7)</f>
+        <f t="shared" si="0"/>
         <v>8.65</v>
       </c>
       <c r="D7" s="1">
@@ -4888,7 +4933,7 @@
         <v>124</v>
       </c>
       <c r="C8" s="5">
-        <f>AVERAGE(D8,E8,E8,F8,G8,H8,H8,I8)</f>
+        <f t="shared" si="0"/>
         <v>8.625</v>
       </c>
       <c r="D8" s="1">
@@ -4915,7 +4960,7 @@
         <v>121</v>
       </c>
       <c r="C9" s="5">
-        <f>AVERAGE(D9,E9,E9,F9,G9,H9,H9,I9)</f>
+        <f t="shared" si="0"/>
         <v>8.5250000000000004</v>
       </c>
       <c r="D9" s="1">
@@ -4942,7 +4987,7 @@
         <v>127</v>
       </c>
       <c r="C10" s="5">
-        <f>AVERAGE(D10,E10,E10,F10,G10,H10,H10,I10)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D10" s="1">
@@ -4969,7 +5014,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="5">
-        <f>AVERAGE(D11,E11,E11,F11,G11,H11,H11,I11)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D11" s="1">
@@ -4996,7 +5041,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="5">
-        <f>AVERAGE(D12,E12,E12,F12,G12,H12,H12,I12)</f>
+        <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="D12" s="1">
@@ -5023,7 +5068,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5">
-        <f>AVERAGE(D13,E13,E13,F13,G13,H13,H13,I13)</f>
+        <f t="shared" si="0"/>
         <v>8.4375</v>
       </c>
       <c r="D13" s="1">
@@ -5050,7 +5095,7 @@
         <v>96</v>
       </c>
       <c r="C14" s="5">
-        <f>AVERAGE(D14,E14,E14,F14,G14,H14,H14,I14)</f>
+        <f t="shared" si="0"/>
         <v>8.4124999999999996</v>
       </c>
       <c r="D14" s="1">
@@ -5077,7 +5122,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="5">
-        <f>AVERAGE(D15,E15,E15,F15,G15,H15,H15,I15)</f>
+        <f t="shared" si="0"/>
         <v>8.3999999999999986</v>
       </c>
       <c r="D15" s="1">
@@ -5104,7 +5149,7 @@
         <v>235</v>
       </c>
       <c r="C16" s="5">
-        <f>AVERAGE(D16,E16,E16,F16,G16,H16,H16,I16)</f>
+        <f t="shared" si="0"/>
         <v>8.1875</v>
       </c>
       <c r="D16" s="1">
@@ -5131,7 +5176,7 @@
         <v>125</v>
       </c>
       <c r="C17" s="5">
-        <f>AVERAGE(D17,E17,E17,F17,G17,H17,H17,I17)</f>
+        <f t="shared" si="0"/>
         <v>8.1750000000000007</v>
       </c>
       <c r="D17" s="1">
@@ -5158,7 +5203,7 @@
         <v>81</v>
       </c>
       <c r="C18" s="5">
-        <f>AVERAGE(D18,E18,E18,F18,G18,H18,H18,I18)</f>
+        <f t="shared" si="0"/>
         <v>8.1624999999999996</v>
       </c>
       <c r="D18" s="1">
@@ -5185,7 +5230,7 @@
         <v>77</v>
       </c>
       <c r="C19" s="5">
-        <f>AVERAGE(D19,E19,E19,F19,G19,H19,H19,I19)</f>
+        <f t="shared" si="0"/>
         <v>8.15</v>
       </c>
       <c r="D19" s="1">
@@ -5212,7 +5257,7 @@
         <v>54</v>
       </c>
       <c r="C20" s="5">
-        <f>AVERAGE(D20,E20,E20,F20,G20,H20,H20,I20)</f>
+        <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
       <c r="D20" s="1">
@@ -5239,7 +5284,7 @@
         <v>126</v>
       </c>
       <c r="C21" s="5">
-        <f>AVERAGE(D21,E21,E21,F21,G21,H21,H21,I21)</f>
+        <f t="shared" si="0"/>
         <v>8.0750000000000011</v>
       </c>
       <c r="D21" s="1">
@@ -5266,7 +5311,7 @@
         <v>58</v>
       </c>
       <c r="C22" s="5">
-        <f>AVERAGE(D22,E22,E22,F22,G22,H22,H22,I22)</f>
+        <f t="shared" si="0"/>
         <v>8.0625</v>
       </c>
       <c r="D22" s="1">
@@ -5293,7 +5338,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="5">
-        <f>AVERAGE(D23,E23,E23,F23,G23,H23,H23,I23)</f>
+        <f t="shared" si="0"/>
         <v>7.9249999999999998</v>
       </c>
       <c r="D23" s="1">
@@ -5320,7 +5365,7 @@
         <v>122</v>
       </c>
       <c r="C24" s="5">
-        <f>AVERAGE(D24,E24,E24,F24,G24,H24,H24,I24)</f>
+        <f t="shared" si="0"/>
         <v>7.9124999999999996</v>
       </c>
       <c r="D24" s="1">
@@ -5347,7 +5392,7 @@
         <v>108</v>
       </c>
       <c r="C25" s="5">
-        <f>AVERAGE(D25,E25,E25,F25,G25,H25,H25,I25)</f>
+        <f t="shared" si="0"/>
         <v>7.8999999999999995</v>
       </c>
       <c r="D25" s="1">
@@ -5374,7 +5419,7 @@
         <v>78</v>
       </c>
       <c r="C26" s="5">
-        <f>AVERAGE(D26,E26,E26,F26,G26,H26,H26,I26)</f>
+        <f t="shared" si="0"/>
         <v>7.875</v>
       </c>
       <c r="D26" s="1">
@@ -5401,7 +5446,7 @@
         <v>109</v>
       </c>
       <c r="C27" s="5">
-        <f>AVERAGE(D27,E27,E27,F27,G27,H27,H27,I27)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D27" s="1">
@@ -5428,7 +5473,7 @@
         <v>61</v>
       </c>
       <c r="C28" s="5">
-        <f>AVERAGE(D28,E28,E28,F28,G28,H28,H28,I28)</f>
+        <f t="shared" si="0"/>
         <v>7.7875000000000005</v>
       </c>
       <c r="D28" s="1">
@@ -5455,7 +5500,7 @@
         <v>193</v>
       </c>
       <c r="C29" s="5">
-        <f>AVERAGE(D29,E29,E29,F29,G29,H29,H29,I29)</f>
+        <f t="shared" si="0"/>
         <v>7.7750000000000004</v>
       </c>
       <c r="D29" s="1">
@@ -5482,7 +5527,7 @@
         <v>60</v>
       </c>
       <c r="C30" s="5">
-        <f>AVERAGE(D30,E30,E30,F30,G30,H30,H30,I30)</f>
+        <f t="shared" si="0"/>
         <v>7.7375000000000007</v>
       </c>
       <c r="D30" s="1">
@@ -5509,7 +5554,7 @@
         <v>38</v>
       </c>
       <c r="C31" s="5">
-        <f>AVERAGE(D31,E31,E31,F31,G31,H31,H31,I31)</f>
+        <f t="shared" si="0"/>
         <v>7.7000000000000011</v>
       </c>
       <c r="D31" s="1">
@@ -5536,7 +5581,7 @@
         <v>63</v>
       </c>
       <c r="C32" s="5">
-        <f>AVERAGE(D32,E32,E32,F32,G32,H32,H32,I32)</f>
+        <f t="shared" si="0"/>
         <v>7.6999999999999993</v>
       </c>
       <c r="D32" s="1">
@@ -5563,7 +5608,7 @@
         <v>123</v>
       </c>
       <c r="C33" s="5">
-        <f>AVERAGE(D33,E33,E33,F33,G33,H33,H33,I33)</f>
+        <f t="shared" si="0"/>
         <v>7.5874999999999995</v>
       </c>
       <c r="D33" s="1">
@@ -5590,7 +5635,7 @@
         <v>37</v>
       </c>
       <c r="C34" s="5">
-        <f>AVERAGE(D34,E34,E34,F34,G34,H34,H34,I34)</f>
+        <f t="shared" si="0"/>
         <v>7.5750000000000011</v>
       </c>
       <c r="D34" s="1">
@@ -5617,7 +5662,7 @@
         <v>67</v>
       </c>
       <c r="C35" s="5">
-        <f>AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
+        <f t="shared" ref="C35:C66" si="1">AVERAGE(D35,E35,E35,F35,G35,H35,H35,I35)</f>
         <v>7.5750000000000002</v>
       </c>
       <c r="D35" s="1">
@@ -5644,7 +5689,7 @@
         <v>62</v>
       </c>
       <c r="C36" s="5">
-        <f>AVERAGE(D36,E36,E36,F36,G36,H36,H36,I36)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D36" s="1">
@@ -5671,7 +5716,7 @@
         <v>217</v>
       </c>
       <c r="C37" s="5">
-        <f>AVERAGE(D37,E37,E37,F37,G37,H37,H37,I37)</f>
+        <f t="shared" si="1"/>
         <v>7.5625</v>
       </c>
       <c r="D37" s="1">
@@ -5698,7 +5743,7 @@
         <v>55</v>
       </c>
       <c r="C38" s="5">
-        <f>AVERAGE(D38,E38,E38,F38,G38,H38,H38,I38)</f>
+        <f t="shared" si="1"/>
         <v>7.5624999999999991</v>
       </c>
       <c r="D38" s="1">
@@ -5725,7 +5770,7 @@
         <v>201</v>
       </c>
       <c r="C39" s="5">
-        <f>AVERAGE(D39,E39,E39,F39,G39,H39,H39,I39)</f>
+        <f t="shared" si="1"/>
         <v>7.55</v>
       </c>
       <c r="D39" s="1">
@@ -5752,7 +5797,7 @@
         <v>69</v>
       </c>
       <c r="C40" s="5">
-        <f>AVERAGE(D40,E40,E40,F40,G40,H40,H40,I40)</f>
+        <f t="shared" si="1"/>
         <v>7.5250000000000004</v>
       </c>
       <c r="D40" s="1">
@@ -5779,7 +5824,7 @@
         <v>132</v>
       </c>
       <c r="C41" s="5">
-        <f>AVERAGE(D41,E41,E41,F41,G41,H41,H41,I41)</f>
+        <f t="shared" si="1"/>
         <v>7.5125000000000002</v>
       </c>
       <c r="D41" s="1">
@@ -5806,7 +5851,7 @@
         <v>230</v>
       </c>
       <c r="C42" s="5">
-        <f>AVERAGE(D42,E42,E42,F42,G42,H42,H42,I42)</f>
+        <f t="shared" si="1"/>
         <v>7.5124999999999993</v>
       </c>
       <c r="D42" s="1">
@@ -5833,7 +5878,7 @@
         <v>205</v>
       </c>
       <c r="C43" s="5">
-        <f>AVERAGE(D43,E43,E43,F43,G43,H43,H43,I43)</f>
+        <f t="shared" si="1"/>
         <v>7.4875000000000007</v>
       </c>
       <c r="D43" s="1">
@@ -5860,7 +5905,7 @@
         <v>172</v>
       </c>
       <c r="C44" s="5">
-        <f>AVERAGE(D44,E44,E44,F44,G44,H44,H44,I44)</f>
+        <f t="shared" si="1"/>
         <v>7.4749999999999996</v>
       </c>
       <c r="D44" s="1">
@@ -5887,7 +5932,7 @@
         <v>130</v>
       </c>
       <c r="C45" s="5">
-        <f>AVERAGE(D45,E45,E45,F45,G45,H45,H45,I45)</f>
+        <f t="shared" si="1"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="D45" s="1">
@@ -5914,7 +5959,7 @@
         <v>97</v>
       </c>
       <c r="C46" s="5">
-        <f>AVERAGE(D46,E46,E46,F46,G46,H46,H46,I46)</f>
+        <f t="shared" si="1"/>
         <v>7.4375</v>
       </c>
       <c r="D46" s="1">
@@ -5941,7 +5986,7 @@
         <v>100</v>
       </c>
       <c r="C47" s="5">
-        <f>AVERAGE(D47,E47,E47,F47,G47,H47,H47,I47)</f>
+        <f t="shared" si="1"/>
         <v>7.4249999999999998</v>
       </c>
       <c r="D47" s="1">
@@ -5968,7 +6013,7 @@
         <v>244</v>
       </c>
       <c r="C48" s="5">
-        <f>AVERAGE(D48,E48,E48,F48,G48,H48,H48,I48)</f>
+        <f t="shared" si="1"/>
         <v>7.4125000000000005</v>
       </c>
       <c r="D48" s="1">
@@ -5995,7 +6040,7 @@
         <v>131</v>
       </c>
       <c r="C49" s="5">
-        <f>AVERAGE(D49,E49,E49,F49,G49,H49,H49,I49)</f>
+        <f t="shared" si="1"/>
         <v>7.4124999999999996</v>
       </c>
       <c r="D49" s="1">
@@ -6022,7 +6067,7 @@
         <v>220</v>
       </c>
       <c r="C50" s="5">
-        <f>AVERAGE(D50,E50,E50,F50,G50,H50,H50,I50)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999998</v>
       </c>
       <c r="D50" s="1">
@@ -6049,7 +6094,7 @@
         <v>175</v>
       </c>
       <c r="C51" s="5">
-        <f>AVERAGE(D51,E51,E51,F51,G51,H51,H51,I51)</f>
+        <f t="shared" si="1"/>
         <v>7.3624999999999989</v>
       </c>
       <c r="D51" s="1">
@@ -6076,7 +6121,7 @@
         <v>52</v>
       </c>
       <c r="C52" s="5">
-        <f>AVERAGE(D52,E52,E52,F52,G52,H52,H52,I52)</f>
+        <f t="shared" si="1"/>
         <v>7.3500000000000005</v>
       </c>
       <c r="D52" s="1">
@@ -6103,7 +6148,7 @@
         <v>165</v>
       </c>
       <c r="C53" s="5">
-        <f>AVERAGE(D53,E53,E53,F53,G53,H53,H53,I53)</f>
+        <f t="shared" si="1"/>
         <v>7.3249999999999993</v>
       </c>
       <c r="D53" s="1">
@@ -6130,7 +6175,7 @@
         <v>224</v>
       </c>
       <c r="C54" s="5">
-        <f>AVERAGE(D54,E54,E54,F54,G54,H54,H54,I54)</f>
+        <f t="shared" si="1"/>
         <v>7.3125</v>
       </c>
       <c r="D54" s="1">
@@ -6157,7 +6202,7 @@
         <v>111</v>
       </c>
       <c r="C55" s="5">
-        <f>AVERAGE(D55,E55,E55,F55,G55,H55,H55,I55)</f>
+        <f t="shared" si="1"/>
         <v>7.3</v>
       </c>
       <c r="D55" s="1">
@@ -6184,7 +6229,7 @@
         <v>103</v>
       </c>
       <c r="C56" s="5">
-        <f>AVERAGE(D56,E56,E56,F56,G56,H56,H56,I56)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D56" s="1">
@@ -6211,7 +6256,7 @@
         <v>181</v>
       </c>
       <c r="C57" s="5">
-        <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
+        <f t="shared" si="1"/>
         <v>7.2750000000000004</v>
       </c>
       <c r="D57" s="1">
@@ -6238,7 +6283,7 @@
         <v>225</v>
       </c>
       <c r="C58" s="5">
-        <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
+        <f t="shared" si="1"/>
         <v>7.2624999999999993</v>
       </c>
       <c r="D58" s="1">
@@ -6265,7 +6310,7 @@
         <v>147</v>
       </c>
       <c r="C59" s="5">
-        <f>AVERAGE(D59,E59,E59,F59,G59,H59,H59,I59)</f>
+        <f t="shared" si="1"/>
         <v>7.2374999999999998</v>
       </c>
       <c r="D59" s="1">
@@ -6292,7 +6337,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="5">
-        <f>AVERAGE(D60,E60,E60,F60,G60,H60,H60,I60)</f>
+        <f t="shared" si="1"/>
         <v>7.2250000000000005</v>
       </c>
       <c r="D60" s="1">
@@ -6319,7 +6364,7 @@
         <v>65</v>
       </c>
       <c r="C61" s="5">
-        <f>AVERAGE(D61,E61,E61,F61,G61,H61,H61,I61)</f>
+        <f t="shared" si="1"/>
         <v>7.2125000000000004</v>
       </c>
       <c r="D61" s="1">
@@ -6346,7 +6391,7 @@
         <v>146</v>
       </c>
       <c r="C62" s="5">
-        <f>AVERAGE(D62,E62,E62,F62,G62,H62,H62,I62)</f>
+        <f t="shared" si="1"/>
         <v>7.2124999999999995</v>
       </c>
       <c r="D62" s="1">
@@ -6373,7 +6418,7 @@
         <v>94</v>
       </c>
       <c r="C63" s="5">
-        <f>AVERAGE(D63,E63,E63,F63,G63,H63,H63,I63)</f>
+        <f t="shared" si="1"/>
         <v>7.1999999999999993</v>
       </c>
       <c r="D63" s="1">
@@ -6400,7 +6445,7 @@
         <v>53</v>
       </c>
       <c r="C64" s="5">
-        <f>AVERAGE(D64,E64,E64,F64,G64,H64,H64,I64)</f>
+        <f t="shared" si="1"/>
         <v>7.1499999999999995</v>
       </c>
       <c r="D64" s="1">
@@ -6427,7 +6472,7 @@
         <v>104</v>
       </c>
       <c r="C65" s="5">
-        <f>AVERAGE(D65,E65,E65,F65,G65,H65,H65,I65)</f>
+        <f t="shared" si="1"/>
         <v>7.1375000000000011</v>
       </c>
       <c r="D65" s="1">
@@ -6454,7 +6499,7 @@
         <v>40</v>
       </c>
       <c r="C66" s="5">
-        <f>AVERAGE(D66,E66,E66,F66,G66,H66,H66,I66)</f>
+        <f t="shared" si="1"/>
         <v>7.1250000000000009</v>
       </c>
       <c r="D66" s="1">
@@ -6481,7 +6526,7 @@
         <v>39</v>
       </c>
       <c r="C67" s="5">
-        <f>AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,E67,F67,G67,H67,H67,I67)</f>
         <v>7.125</v>
       </c>
       <c r="D67" s="1">
@@ -6508,7 +6553,7 @@
         <v>133</v>
       </c>
       <c r="C68" s="5">
-        <f>AVERAGE(D68,E68,E68,F68,G68,H68,H68,I68)</f>
+        <f t="shared" si="2"/>
         <v>7.0875000000000004</v>
       </c>
       <c r="D68" s="1">
@@ -6535,7 +6580,7 @@
         <v>98</v>
       </c>
       <c r="C69" s="5">
-        <f>AVERAGE(D69,E69,E69,F69,G69,H69,H69,I69)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D69" s="1">
@@ -6562,7 +6607,7 @@
         <v>171</v>
       </c>
       <c r="C70" s="5">
-        <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000011</v>
       </c>
       <c r="D70" s="1">
@@ -6589,7 +6634,7 @@
         <v>110</v>
       </c>
       <c r="C71" s="5">
-        <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D71" s="1">
@@ -6616,7 +6661,7 @@
         <v>143</v>
       </c>
       <c r="C72" s="5">
-        <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
+        <f t="shared" si="2"/>
         <v>7.0750000000000002</v>
       </c>
       <c r="D72" s="1">
@@ -6643,7 +6688,7 @@
         <v>177</v>
       </c>
       <c r="C73" s="5">
-        <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
+        <f t="shared" si="2"/>
         <v>7.0749999999999993</v>
       </c>
       <c r="D73" s="1">
@@ -6670,7 +6715,7 @@
         <v>176</v>
       </c>
       <c r="C74" s="5">
-        <f>AVERAGE(D74,E74,E74,F74,G74,H74,H74,I74)</f>
+        <f t="shared" si="2"/>
         <v>7.05</v>
       </c>
       <c r="D74" s="1">
@@ -6697,7 +6742,7 @@
         <v>221</v>
       </c>
       <c r="C75" s="5">
-        <f>AVERAGE(D75,E75,E75,F75,G75,H75,H75,I75)</f>
+        <f t="shared" si="2"/>
         <v>7.0250000000000004</v>
       </c>
       <c r="D75" s="1">
@@ -6724,7 +6769,7 @@
         <v>95</v>
       </c>
       <c r="C76" s="5">
-        <f>AVERAGE(D76,E76,E76,F76,G76,H76,H76,I76)</f>
+        <f t="shared" si="2"/>
         <v>6.9375</v>
       </c>
       <c r="D76" s="1">
@@ -6751,7 +6796,7 @@
         <v>164</v>
       </c>
       <c r="C77" s="5">
-        <f>AVERAGE(D77,E77,E77,F77,G77,H77,H77,I77)</f>
+        <f t="shared" si="2"/>
         <v>6.9124999999999996</v>
       </c>
       <c r="D77" s="1">
@@ -6778,7 +6823,7 @@
         <v>157</v>
       </c>
       <c r="C78" s="5">
-        <f>AVERAGE(D78,E78,E78,F78,G78,H78,H78,I78)</f>
+        <f t="shared" si="2"/>
         <v>6.8999999999999995</v>
       </c>
       <c r="D78" s="1">
@@ -6805,7 +6850,7 @@
         <v>88</v>
       </c>
       <c r="C79" s="5">
-        <f>AVERAGE(D79,E79,E79,F79,G79,H79,H79,I79)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D79" s="1">
@@ -6832,7 +6877,7 @@
         <v>184</v>
       </c>
       <c r="C80" s="5">
-        <f>AVERAGE(D80,E80,E80,F80,G80,H80,H80,I80)</f>
+        <f t="shared" si="2"/>
         <v>6.8624999999999989</v>
       </c>
       <c r="D80" s="1">
@@ -6859,7 +6904,7 @@
         <v>119</v>
       </c>
       <c r="C81" s="5">
-        <f>AVERAGE(D81,E81,E81,F81,G81,H81,H81,I81)</f>
+        <f t="shared" si="2"/>
         <v>6.85</v>
       </c>
       <c r="D81" s="1">
@@ -6886,7 +6931,7 @@
         <v>196</v>
       </c>
       <c r="C82" s="5">
-        <f>AVERAGE(D82,E82,E82,F82,G82,H82,H82,I82)</f>
+        <f t="shared" si="2"/>
         <v>6.7999999999999989</v>
       </c>
       <c r="D82" s="1">
@@ -6913,7 +6958,7 @@
         <v>57</v>
       </c>
       <c r="C83" s="5">
-        <f>AVERAGE(D83,E83,E83,F83,G83,H83,H83,I83)</f>
+        <f t="shared" si="2"/>
         <v>6.6999999999999993</v>
       </c>
       <c r="D83" s="1">
@@ -6940,7 +6985,7 @@
         <v>87</v>
       </c>
       <c r="C84" s="5">
-        <f>AVERAGE(D84,E84,E84,F84,G84,H84,H84,I84)</f>
+        <f t="shared" si="2"/>
         <v>6.6875</v>
       </c>
       <c r="D84" s="1">
@@ -6967,7 +7012,7 @@
         <v>211</v>
       </c>
       <c r="C85" s="5">
-        <f>AVERAGE(D85,E85,E85,F85,G85,H85,H85,I85)</f>
+        <f t="shared" si="2"/>
         <v>6.6375000000000002</v>
       </c>
       <c r="D85" s="1">
@@ -6994,7 +7039,7 @@
         <v>219</v>
       </c>
       <c r="C86" s="5">
-        <f>AVERAGE(D86,E86,E86,F86,G86,H86,H86,I86)</f>
+        <f t="shared" si="2"/>
         <v>6.6374999999999993</v>
       </c>
       <c r="D86" s="1">
@@ -7017,11 +7062,11 @@
       </c>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B87" s="9" t="s">
+      <c r="B87" s="2" t="s">
         <v>255</v>
       </c>
       <c r="C87" s="5">
-        <f>AVERAGE(D87,E87,E87,F87,G87,H87,H87,I87)</f>
+        <f t="shared" si="2"/>
         <v>6.6124999999999998</v>
       </c>
       <c r="D87" s="1">
@@ -7048,7 +7093,7 @@
         <v>41</v>
       </c>
       <c r="C88" s="5">
-        <f>AVERAGE(D88,E88,E88,F88,G88,H88,H88,I88)</f>
+        <f t="shared" si="2"/>
         <v>6.6124999999999989</v>
       </c>
       <c r="D88" s="1">
@@ -7075,7 +7120,7 @@
         <v>117</v>
       </c>
       <c r="C89" s="5">
-        <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D89" s="1">
@@ -7102,7 +7147,7 @@
         <v>179</v>
       </c>
       <c r="C90" s="5">
-        <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
+        <f t="shared" si="2"/>
         <v>6.5874999999999995</v>
       </c>
       <c r="D90" s="1">
@@ -7129,7 +7174,7 @@
         <v>215</v>
       </c>
       <c r="C91" s="5">
-        <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
+        <f t="shared" si="2"/>
         <v>6.5750000000000002</v>
       </c>
       <c r="D91" s="1">
@@ -7156,7 +7201,7 @@
         <v>249</v>
       </c>
       <c r="C92" s="5">
-        <f>AVERAGE(D92,E92,E92,F92,G92,H92,H92,I92)</f>
+        <f t="shared" si="2"/>
         <v>6.5625</v>
       </c>
       <c r="D92" s="1">
@@ -7183,7 +7228,7 @@
         <v>168</v>
       </c>
       <c r="C93" s="5">
-        <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
+        <f t="shared" si="2"/>
         <v>6.5499999999999989</v>
       </c>
       <c r="D93" s="1">
@@ -7210,7 +7255,7 @@
         <v>197</v>
       </c>
       <c r="C94" s="5">
-        <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
+        <f t="shared" si="2"/>
         <v>6.5375000000000005</v>
       </c>
       <c r="D94" s="1">
@@ -7233,11 +7278,11 @@
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B95" s="9" t="s">
+      <c r="B95" s="2" t="s">
         <v>252</v>
       </c>
       <c r="C95" s="5">
-        <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
+        <f t="shared" si="2"/>
         <v>6.4749999999999996</v>
       </c>
       <c r="D95" s="1">
@@ -7260,11 +7305,11 @@
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B96" s="9" t="s">
+      <c r="B96" s="2" t="s">
         <v>254</v>
       </c>
       <c r="C96" s="5">
-        <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
+        <f t="shared" si="2"/>
         <v>6.4124999999999996</v>
       </c>
       <c r="D96" s="1">
@@ -7291,7 +7336,7 @@
         <v>202</v>
       </c>
       <c r="C97" s="5">
-        <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
+        <f t="shared" si="2"/>
         <v>6.3999999999999995</v>
       </c>
       <c r="D97" s="1">
@@ -7314,11 +7359,11 @@
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B98" s="9" t="s">
+      <c r="B98" s="2" t="s">
         <v>256</v>
       </c>
       <c r="C98" s="5">
-        <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
+        <f t="shared" si="2"/>
         <v>6.3625000000000007</v>
       </c>
       <c r="D98" s="1">
@@ -7345,7 +7390,7 @@
         <v>183</v>
       </c>
       <c r="C99" s="5">
-        <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
+        <f t="shared" ref="C99:C130" si="3">AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D99" s="1">
@@ -7372,7 +7417,7 @@
         <v>200</v>
       </c>
       <c r="C100" s="5">
-        <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
+        <f t="shared" si="3"/>
         <v>6.3624999999999998</v>
       </c>
       <c r="D100" s="1">
@@ -7399,7 +7444,7 @@
         <v>188</v>
       </c>
       <c r="C101" s="5">
-        <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
+        <f t="shared" si="3"/>
         <v>6.35</v>
       </c>
       <c r="D101" s="1">
@@ -7426,7 +7471,7 @@
         <v>208</v>
       </c>
       <c r="C102" s="5">
-        <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
+        <f t="shared" si="3"/>
         <v>6.35</v>
       </c>
       <c r="D102" s="1">
@@ -7453,7 +7498,7 @@
         <v>134</v>
       </c>
       <c r="C103" s="5">
-        <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
+        <f t="shared" si="3"/>
         <v>6.3125</v>
       </c>
       <c r="D103" s="1">
@@ -7480,7 +7525,7 @@
         <v>144</v>
       </c>
       <c r="C104" s="5">
-        <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
+        <f t="shared" si="3"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D104" s="1">
@@ -7507,7 +7552,7 @@
         <v>64</v>
       </c>
       <c r="C105" s="5">
-        <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
+        <f t="shared" si="3"/>
         <v>6.2749999999999995</v>
       </c>
       <c r="D105" s="1">
@@ -7534,7 +7579,7 @@
         <v>75</v>
       </c>
       <c r="C106" s="5">
-        <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
+        <f t="shared" si="3"/>
         <v>6.2125000000000004</v>
       </c>
       <c r="D106" s="1">
@@ -7561,7 +7606,7 @@
         <v>19</v>
       </c>
       <c r="C107" s="5">
-        <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
+        <f t="shared" si="3"/>
         <v>6.2124999999999995</v>
       </c>
       <c r="D107" s="1">
@@ -7588,7 +7633,7 @@
         <v>101</v>
       </c>
       <c r="C108" s="5">
-        <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
+        <f t="shared" si="3"/>
         <v>6.15</v>
       </c>
       <c r="D108" s="1">
@@ -7615,7 +7660,7 @@
         <v>240</v>
       </c>
       <c r="C109" s="5">
-        <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
+        <f t="shared" si="3"/>
         <v>6.1250000000000009</v>
       </c>
       <c r="D109" s="1">
@@ -7642,7 +7687,7 @@
         <v>158</v>
       </c>
       <c r="C110" s="5">
-        <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
+        <f t="shared" si="3"/>
         <v>6.0874999999999995</v>
       </c>
       <c r="D110" s="1">
@@ -7669,7 +7714,7 @@
         <v>222</v>
       </c>
       <c r="C111" s="5">
-        <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
+        <f t="shared" si="3"/>
         <v>6.0625</v>
       </c>
       <c r="D111" s="1">
@@ -7696,7 +7741,7 @@
         <v>214</v>
       </c>
       <c r="C112" s="5">
-        <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
+        <f t="shared" si="3"/>
         <v>6.0500000000000007</v>
       </c>
       <c r="D112" s="1">
@@ -7723,7 +7768,7 @@
         <v>160</v>
       </c>
       <c r="C113" s="5">
-        <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D113" s="1">
@@ -7750,7 +7795,7 @@
         <v>206</v>
       </c>
       <c r="C114" s="5">
-        <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
+        <f t="shared" si="3"/>
         <v>6.05</v>
       </c>
       <c r="D114" s="1">
@@ -7777,7 +7822,7 @@
         <v>159</v>
       </c>
       <c r="C115" s="5">
-        <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
+        <f t="shared" si="3"/>
         <v>5.9499999999999993</v>
       </c>
       <c r="D115" s="1">
@@ -7800,11 +7845,11 @@
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B116" s="9" t="s">
+      <c r="B116" s="2" t="s">
         <v>257</v>
       </c>
       <c r="C116" s="5">
-        <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
+        <f t="shared" si="3"/>
         <v>5.9250000000000007</v>
       </c>
       <c r="D116" s="1">
@@ -7831,7 +7876,7 @@
         <v>195</v>
       </c>
       <c r="C117" s="5">
-        <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
+        <f t="shared" si="3"/>
         <v>5.8875000000000011</v>
       </c>
       <c r="D117" s="1">
@@ -7858,7 +7903,7 @@
         <v>186</v>
       </c>
       <c r="C118" s="5">
-        <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
+        <f t="shared" si="3"/>
         <v>5.8125000000000009</v>
       </c>
       <c r="D118" s="1">
@@ -7885,7 +7930,7 @@
         <v>209</v>
       </c>
       <c r="C119" s="5">
-        <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
+        <f t="shared" si="3"/>
         <v>5.8000000000000007</v>
       </c>
       <c r="D119" s="1">
@@ -7912,7 +7957,7 @@
         <v>113</v>
       </c>
       <c r="C120" s="5">
-        <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
+        <f t="shared" si="3"/>
         <v>5.7374999999999989</v>
       </c>
       <c r="D120" s="1">
@@ -7939,7 +7984,7 @@
         <v>187</v>
       </c>
       <c r="C121" s="5">
-        <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
+        <f t="shared" si="3"/>
         <v>5.7250000000000005</v>
       </c>
       <c r="D121" s="1">
@@ -7962,11 +8007,11 @@
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B122" s="9" t="s">
+      <c r="B122" s="2" t="s">
         <v>253</v>
       </c>
       <c r="C122" s="5">
-        <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
+        <f t="shared" si="3"/>
         <v>5.6875000000000009</v>
       </c>
       <c r="D122" s="1">
@@ -7993,7 +8038,7 @@
         <v>26</v>
       </c>
       <c r="C123" s="5">
-        <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
+        <f t="shared" si="3"/>
         <v>5.6749999999999998</v>
       </c>
       <c r="D123" s="1">
@@ -8020,7 +8065,7 @@
         <v>149</v>
       </c>
       <c r="C124" s="5">
-        <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D124" s="1">
@@ -8047,7 +8092,7 @@
         <v>156</v>
       </c>
       <c r="C125" s="5">
-        <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
+        <f t="shared" si="3"/>
         <v>5.5624999999999991</v>
       </c>
       <c r="D125" s="1">
@@ -8074,7 +8119,7 @@
         <v>229</v>
       </c>
       <c r="C126" s="5">
-        <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
+        <f t="shared" si="3"/>
         <v>5.5375000000000005</v>
       </c>
       <c r="D126" s="1">
@@ -8101,7 +8146,7 @@
         <v>245</v>
       </c>
       <c r="C127" s="5">
-        <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
+        <f t="shared" si="3"/>
         <v>5.5125000000000011</v>
       </c>
       <c r="D127" s="1">
@@ -8128,7 +8173,7 @@
         <v>166</v>
       </c>
       <c r="C128" s="5">
-        <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D128" s="1">
@@ -8155,7 +8200,7 @@
         <v>191</v>
       </c>
       <c r="C129" s="5">
-        <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
+        <f t="shared" si="3"/>
         <v>5.4874999999999989</v>
       </c>
       <c r="D129" s="1">
@@ -8182,7 +8227,7 @@
         <v>228</v>
       </c>
       <c r="C130" s="5">
-        <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
+        <f t="shared" si="3"/>
         <v>5.3875000000000011</v>
       </c>
       <c r="D130" s="1">
@@ -8209,7 +8254,7 @@
         <v>204</v>
       </c>
       <c r="C131" s="5">
-        <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
+        <f t="shared" ref="C131:C162" si="4">AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
         <v>5.3750000000000009</v>
       </c>
       <c r="D131" s="1">
@@ -8236,7 +8281,7 @@
         <v>190</v>
       </c>
       <c r="C132" s="5">
-        <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
+        <f t="shared" si="4"/>
         <v>5.375</v>
       </c>
       <c r="D132" s="1">
@@ -8263,7 +8308,7 @@
         <v>182</v>
       </c>
       <c r="C133" s="5">
-        <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
+        <f t="shared" si="4"/>
         <v>5.2875000000000005</v>
       </c>
       <c r="D133" s="1">
@@ -8290,7 +8335,7 @@
         <v>242</v>
       </c>
       <c r="C134" s="5">
-        <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
+        <f t="shared" si="4"/>
         <v>5.25</v>
       </c>
       <c r="D134" s="1">
@@ -8317,7 +8362,7 @@
         <v>232</v>
       </c>
       <c r="C135" s="5">
-        <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
+        <f t="shared" si="4"/>
         <v>5.2</v>
       </c>
       <c r="D135" s="1">
@@ -8344,7 +8389,7 @@
         <v>74</v>
       </c>
       <c r="C136" s="5">
-        <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
+        <f t="shared" si="4"/>
         <v>5.1875</v>
       </c>
       <c r="D136" s="1">
@@ -8371,7 +8416,7 @@
         <v>145</v>
       </c>
       <c r="C137" s="5">
-        <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
+        <f t="shared" si="4"/>
         <v>5.1124999999999998</v>
       </c>
       <c r="D137" s="1">
@@ -8398,7 +8443,7 @@
         <v>223</v>
       </c>
       <c r="C138" s="5">
-        <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
+        <f t="shared" si="4"/>
         <v>5.0750000000000002</v>
       </c>
       <c r="D138" s="1">
@@ -8425,7 +8470,7 @@
         <v>21</v>
       </c>
       <c r="C139" s="5">
-        <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
+        <f t="shared" si="4"/>
         <v>5.05</v>
       </c>
       <c r="D139" s="1">
@@ -8452,7 +8497,7 @@
         <v>203</v>
       </c>
       <c r="C140" s="5">
-        <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
+        <f t="shared" si="4"/>
         <v>4.9875000000000007</v>
       </c>
       <c r="D140" s="1">
@@ -8479,7 +8524,7 @@
         <v>169</v>
       </c>
       <c r="C141" s="5">
-        <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
+        <f t="shared" si="4"/>
         <v>4.9874999999999998</v>
       </c>
       <c r="D141" s="1">
@@ -8506,7 +8551,7 @@
         <v>241</v>
       </c>
       <c r="C142" s="5">
-        <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
+        <f t="shared" si="4"/>
         <v>4.9249999999999998</v>
       </c>
       <c r="D142" s="1">
@@ -8533,7 +8578,7 @@
         <v>163</v>
       </c>
       <c r="C143" s="5">
-        <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
+        <f t="shared" si="4"/>
         <v>4.8499999999999996</v>
       </c>
       <c r="D143" s="1">
@@ -8560,7 +8605,7 @@
         <v>162</v>
       </c>
       <c r="C144" s="5">
-        <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
+        <f t="shared" si="4"/>
         <v>4.7875000000000005</v>
       </c>
       <c r="D144" s="1">
@@ -8587,7 +8632,7 @@
         <v>213</v>
       </c>
       <c r="C145" s="5">
-        <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
+        <f t="shared" si="4"/>
         <v>4.6124999999999998</v>
       </c>
       <c r="D145" s="1">
@@ -8614,7 +8659,7 @@
         <v>154</v>
       </c>
       <c r="C146" s="5">
-        <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
+        <f t="shared" si="4"/>
         <v>4.5999999999999996</v>
       </c>
       <c r="D146" s="1">
@@ -8641,7 +8686,7 @@
         <v>135</v>
       </c>
       <c r="C147" s="5">
-        <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
+        <f t="shared" si="4"/>
         <v>4.5874999999999995</v>
       </c>
       <c r="D147" s="1">
@@ -8668,7 +8713,7 @@
         <v>243</v>
       </c>
       <c r="C148" s="5">
-        <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
+        <f t="shared" si="4"/>
         <v>4.5</v>
       </c>
       <c r="D148" s="1">
@@ -8695,7 +8740,7 @@
         <v>161</v>
       </c>
       <c r="C149" s="5">
-        <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
+        <f t="shared" si="4"/>
         <v>4.4249999999999998</v>
       </c>
       <c r="D149" s="1">
@@ -8722,7 +8767,7 @@
         <v>114</v>
       </c>
       <c r="C150" s="5">
-        <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
+        <f t="shared" si="4"/>
         <v>4.4124999999999996</v>
       </c>
       <c r="D150" s="1">
@@ -8749,7 +8794,7 @@
         <v>207</v>
       </c>
       <c r="C151" s="5">
-        <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
+        <f t="shared" si="4"/>
         <v>4.3375000000000004</v>
       </c>
       <c r="D151" s="1">
@@ -8776,7 +8821,7 @@
         <v>150</v>
       </c>
       <c r="C152" s="5">
-        <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
+        <f t="shared" si="4"/>
         <v>4.3374999999999995</v>
       </c>
       <c r="D152" s="1">
@@ -8803,7 +8848,7 @@
         <v>173</v>
       </c>
       <c r="C153" s="5">
-        <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
+        <f t="shared" si="4"/>
         <v>4.3125</v>
       </c>
       <c r="D153" s="1">
@@ -8826,11 +8871,11 @@
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B154" s="9" t="s">
+      <c r="B154" s="2" t="s">
         <v>258</v>
       </c>
       <c r="C154" s="5">
-        <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
+        <f t="shared" si="4"/>
         <v>4.3000000000000007</v>
       </c>
       <c r="D154" s="1">
@@ -8857,7 +8902,7 @@
         <v>212</v>
       </c>
       <c r="C155" s="5">
-        <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
+        <f t="shared" si="4"/>
         <v>4.3</v>
       </c>
       <c r="D155" s="1">
@@ -8884,7 +8929,7 @@
         <v>167</v>
       </c>
       <c r="C156" s="5">
-        <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
+        <f t="shared" si="4"/>
         <v>4.2749999999999995</v>
       </c>
       <c r="D156" s="1">
@@ -8911,7 +8956,7 @@
         <v>236</v>
       </c>
       <c r="C157" s="5">
-        <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
+        <f t="shared" si="4"/>
         <v>4.1749999999999998</v>
       </c>
       <c r="D157" s="1">
@@ -8938,7 +8983,7 @@
         <v>233</v>
       </c>
       <c r="C158" s="5">
-        <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
+        <f t="shared" si="4"/>
         <v>4.1625000000000005</v>
       </c>
       <c r="D158" s="1">
@@ -8965,7 +9010,7 @@
         <v>68</v>
       </c>
       <c r="C159" s="5">
-        <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
+        <f t="shared" si="4"/>
         <v>4.1124999999999998</v>
       </c>
       <c r="D159" s="1">
@@ -8992,7 +9037,7 @@
         <v>218</v>
       </c>
       <c r="C160" s="5">
-        <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
+        <f t="shared" si="4"/>
         <v>3.9499999999999997</v>
       </c>
       <c r="D160" s="1">
@@ -9019,7 +9064,7 @@
         <v>199</v>
       </c>
       <c r="C161" s="5">
-        <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
+        <f t="shared" si="4"/>
         <v>3.7375000000000003</v>
       </c>
       <c r="D161" s="1">
@@ -9046,7 +9091,7 @@
         <v>250</v>
       </c>
       <c r="C162" s="5">
-        <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
+        <f t="shared" si="4"/>
         <v>3.6624999999999996</v>
       </c>
       <c r="D162" s="1">
@@ -9073,7 +9118,7 @@
         <v>246</v>
       </c>
       <c r="C163" s="5">
-        <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
+        <f t="shared" ref="C163:C194" si="5">AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
         <v>3.5749999999999997</v>
       </c>
       <c r="D163" s="1">
@@ -9100,7 +9145,7 @@
         <v>180</v>
       </c>
       <c r="C164" s="5">
-        <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
+        <f t="shared" si="5"/>
         <v>3.5625000000000004</v>
       </c>
       <c r="D164" s="1">
@@ -9127,7 +9172,7 @@
         <v>216</v>
       </c>
       <c r="C165" s="5">
-        <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
+        <f t="shared" si="5"/>
         <v>3.5375000000000005</v>
       </c>
       <c r="D165" s="1">
@@ -9154,7 +9199,7 @@
         <v>248</v>
       </c>
       <c r="C166" s="5">
-        <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
+        <f t="shared" si="5"/>
         <v>3.3375000000000004</v>
       </c>
       <c r="D166" s="1">
@@ -9181,7 +9226,7 @@
         <v>189</v>
       </c>
       <c r="C167" s="5">
-        <f>AVERAGE(D167,E167,E167,F167,G167,H167,H167,I167)</f>
+        <f t="shared" si="5"/>
         <v>3.3250000000000002</v>
       </c>
       <c r="D167" s="1">
@@ -9208,7 +9253,7 @@
         <v>194</v>
       </c>
       <c r="C168" s="5">
-        <f>AVERAGE(D168,E168,E168,F168,G168,H168,H168,I168)</f>
+        <f t="shared" si="5"/>
         <v>3.2749999999999995</v>
       </c>
       <c r="D168" s="1">
@@ -9235,7 +9280,7 @@
         <v>155</v>
       </c>
       <c r="C169" s="5">
-        <f>AVERAGE(D169,E169,E169,F169,G169,H169,H169,I169)</f>
+        <f t="shared" si="5"/>
         <v>2.9124999999999996</v>
       </c>
       <c r="D169" s="1">
@@ -9262,7 +9307,7 @@
         <v>237</v>
       </c>
       <c r="C170" s="5">
-        <f>AVERAGE(D170,E170,E170,F170,G170,H170,H170,I170)</f>
+        <f t="shared" si="5"/>
         <v>2.8125</v>
       </c>
       <c r="D170" s="1">
@@ -9289,7 +9334,7 @@
         <v>239</v>
       </c>
       <c r="C171" s="5">
-        <f>AVERAGE(D171,E171,E171,F171,G171,H171,H171,I171)</f>
+        <f t="shared" si="5"/>
         <v>2.7625000000000002</v>
       </c>
       <c r="D171" s="1">
@@ -9312,11 +9357,11 @@
       </c>
     </row>
     <row r="172" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B172" s="9" t="s">
+      <c r="B172" s="2" t="s">
         <v>251</v>
       </c>
       <c r="C172" s="5">
-        <f>AVERAGE(D172,E172,E172,F172,G172,H172,H172,I172)</f>
+        <f t="shared" si="5"/>
         <v>2.65</v>
       </c>
       <c r="D172" s="1">
@@ -9343,7 +9388,7 @@
         <v>174</v>
       </c>
       <c r="C173" s="5">
-        <f>AVERAGE(D173,E173,E173,F173,G173,H173,H173,I173)</f>
+        <f t="shared" si="5"/>
         <v>2.6375000000000002</v>
       </c>
       <c r="D173" s="1">
@@ -9370,7 +9415,7 @@
         <v>226</v>
       </c>
       <c r="C174" s="5">
-        <f>AVERAGE(D174,E174,E174,F174,G174,H174,H174,I174)</f>
+        <f t="shared" si="5"/>
         <v>2.5125000000000002</v>
       </c>
       <c r="D174" s="1">

</xml_diff>

<commit_message>
V. 149 "Susurran tu nombre"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B93FE6E-FD7D-41F2-9070-2867263E6C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC43094-04D3-423F-B0FC-A6F467964139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -639,7 +639,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="262">
   <si>
     <t>Película</t>
   </si>
@@ -1422,6 +1422,9 @@
   </si>
   <si>
     <t>La captura</t>
+  </si>
+  <si>
+    <t>Susurran tu nombre</t>
   </si>
 </sst>
 </file>
@@ -1525,13 +1528,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1543,45 +1546,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1622,6 +1586,45 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1748,48 +1751,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M75" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}" name="Tabla245" displayName="Tabla245" ref="B2:M75" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B2:M75" xr:uid="{84882D50-2FDD-4492-A7EE-A56F022A40B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:M75">
     <sortCondition descending="1" ref="C2:C75"/>
   </sortState>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{72A2CB77-15BB-4AA7-8CE3-1A83E67BCC54}" name="Serie" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D20FF574-119A-4C5C-B6E2-E6116B88CECE}" name="Puntuación total" dataDxfId="10">
       <calculatedColumnFormula>AVERAGE(D3,E3,F3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{8DEB5362-455C-4BD9-AC5C-697A0CD42F56}" name="Adicción" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{E96E9843-A8C4-46F1-B720-AECB465AA377}" name="Visualmente" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{4403B32D-52FF-4AC4-9D4C-D3F597FF7C4A}" name="Impresión personal" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{98819486-D7B4-49C2-9DBA-8EF8CB45E089}" name="Audio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{AE89980C-F672-4D83-BC6C-9D834B9DCB47}" name="IMDb" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{CDFF34D7-6389-437E-B3A8-EABF3538508F}" name="Filmaffinity" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{56E55214-A8DF-4868-B9DD-DE618A22CB0B}" name="N" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{B4467319-F04C-4E05-AF98-FABFAC9071D9}" name="P" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9719DF8A-39E9-4708-BA0C-589DA380A38E}" name="D" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{500D2897-05EF-4DC7-9723-D302899DED5C}" name="M" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I175" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I175" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I175">
-    <sortCondition descending="1" ref="C2:C175"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I176" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I176" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I176">
+    <sortCondition descending="1" ref="C2:C176"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6C6ED398-D2C9-428D-BF53-EA4F14903295}" name="Puntuación total" dataDxfId="20">
       <calculatedColumnFormula>AVERAGE(D3,E3,E3,F3,G3,H3,H3,I3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{23B9D8F5-026D-4193-8AE6-5F1DA8430A6D}" name="Visualmente" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{6D046514-7226-41C1-B7E5-3CDF91CE1FE6}" name="Impresión personal" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{31F9BA2E-487F-484E-8E53-40465539C756}" name="Ritmo" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{64A01C2F-A4B0-4AD2-9AFC-C73A75D660A7}" name="Audio" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{1D59F2E8-C7B0-4BBF-94F0-20411C4104C9}" name="IMDb" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{29CE3653-810C-46DD-B239-92B468054CBE}" name="Filmaffinity" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2297,7 +2300,7 @@
       <c r="M2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="8" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2333,7 +2336,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -2400,7 +2403,7 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2438,7 +2441,7 @@
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="O6" s="6"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -2472,7 +2475,7 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="O7" s="6"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -4435,7 +4438,7 @@
         <v>32</v>
       </c>
       <c r="C67" s="5">
-        <f t="shared" ref="C67:C98" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
+        <f t="shared" ref="C67:C75" si="2">AVERAGE(D67,E67,F67,F67,G67,H67,H67,I67)</f>
         <v>6.2250000000000005</v>
       </c>
       <c r="D67" s="1">
@@ -4749,7 +4752,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K175"/>
+  <dimension ref="B2:K176"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4787,7 +4790,7 @@
       <c r="I2" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="6" t="s">
         <v>151</v>
       </c>
     </row>
@@ -4817,7 +4820,7 @@
       <c r="I3" s="3">
         <v>7.2</v>
       </c>
-      <c r="K3" s="8"/>
+      <c r="K3" s="7"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -4845,7 +4848,7 @@
       <c r="I4" s="3">
         <v>6.9</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -6846,7 +6849,7 @@
       </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B79" s="9" t="s">
+      <c r="B79" s="2" t="s">
         <v>260</v>
       </c>
       <c r="C79" s="5">
@@ -7602,123 +7605,123 @@
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B107" s="2" t="s">
-        <v>75</v>
+      <c r="B107" s="9" t="s">
+        <v>261</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2375000000000007</v>
       </c>
       <c r="D107" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F107" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G107" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H107" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I107" s="3">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D108" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E108" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F108" s="1">
         <v>8</v>
       </c>
       <c r="G108" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H108" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I108" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D109" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E109" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F109" s="1">
         <v>8</v>
       </c>
       <c r="G109" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H109" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I109" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>240</v>
+        <v>101</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>6.1250000000000009</v>
+        <v>6.15</v>
       </c>
       <c r="D110" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E110" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F110" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G110" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H110" s="3">
-        <v>6.7</v>
+        <v>5</v>
       </c>
       <c r="I110" s="3">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>158</v>
+        <v>240</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>6.0874999999999995</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D111" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E111" s="1">
         <v>7</v>
@@ -7730,46 +7733,46 @@
         <v>7</v>
       </c>
       <c r="H111" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I111" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D112" s="1">
         <v>7</v>
       </c>
       <c r="E112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H112" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I112" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D113" s="1">
         <v>7</v>
@@ -7778,25 +7781,25 @@
         <v>6</v>
       </c>
       <c r="F113" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G113" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H113" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I113" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D114" s="1">
         <v>7</v>
@@ -7808,49 +7811,49 @@
         <v>7</v>
       </c>
       <c r="G114" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H114" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I114" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
         <v>6.05</v>
       </c>
       <c r="D115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E115" s="1">
         <v>6</v>
       </c>
       <c r="F115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H115" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I115" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D116" s="1">
         <v>6</v>
@@ -7859,25 +7862,25 @@
         <v>6</v>
       </c>
       <c r="F116" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G116" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I116" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>257</v>
+        <v>159</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.9250000000000007</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D117" s="1">
         <v>6</v>
@@ -7886,133 +7889,133 @@
         <v>6</v>
       </c>
       <c r="F117" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G117" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H117" s="3">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="I117" s="3">
-        <v>5.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>195</v>
+        <v>257</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9250000000000007</v>
       </c>
       <c r="D118" s="1">
         <v>6</v>
       </c>
       <c r="E118" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G118" s="1">
         <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
       <c r="I118" s="3">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D119" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E119" s="1">
         <v>5</v>
       </c>
       <c r="F119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G119" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I119" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D120" s="1">
         <v>7</v>
       </c>
       <c r="E120" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F120" s="1">
         <v>5</v>
       </c>
       <c r="G120" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H120" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I120" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D121" s="1">
         <v>7</v>
       </c>
       <c r="E121" s="1">
+        <v>6</v>
+      </c>
+      <c r="F121" s="1">
         <v>5</v>
       </c>
-      <c r="F121" s="1">
-        <v>4</v>
-      </c>
       <c r="G121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H121" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I121" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D122" s="1">
         <v>7</v>
@@ -8024,115 +8027,115 @@
         <v>4</v>
       </c>
       <c r="G122" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H122" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I122" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>253</v>
+        <v>187</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.6875000000000009</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D123" s="1">
+        <v>7</v>
+      </c>
+      <c r="E123" s="1">
         <v>5</v>
       </c>
-      <c r="E123" s="1">
+      <c r="F123" s="1">
         <v>4</v>
       </c>
-      <c r="F123" s="1">
+      <c r="G123" s="1">
         <v>5</v>
-      </c>
-      <c r="G123" s="1">
-        <v>8</v>
       </c>
       <c r="H123" s="3">
         <v>6.7</v>
       </c>
       <c r="I123" s="3">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>26</v>
+        <v>253</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.6749999999999998</v>
+        <v>5.6875000000000009</v>
       </c>
       <c r="D124" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E124" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F124" s="1">
         <v>5</v>
       </c>
       <c r="G124" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H124" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I124" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D125" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E125" s="1">
+        <v>3</v>
+      </c>
+      <c r="F125" s="1">
         <v>5</v>
       </c>
-      <c r="F125" s="1">
-        <v>6</v>
-      </c>
       <c r="G125" s="1">
         <v>6</v>
       </c>
       <c r="H125" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I125" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D126" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E126" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G126" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H126" s="3">
         <v>5.8</v>
@@ -8143,26 +8146,26 @@
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>229</v>
+        <v>156</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>5.5375000000000005</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D127" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E127" s="1">
+        <v>6</v>
+      </c>
+      <c r="F127" s="1">
+        <v>8</v>
+      </c>
+      <c r="G127" s="1">
         <v>5</v>
       </c>
-      <c r="F127" s="1">
-        <v>6</v>
-      </c>
-      <c r="G127" s="1">
-        <v>6</v>
-      </c>
       <c r="H127" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I127" s="3">
         <v>4.9000000000000004</v>
@@ -8170,11 +8173,11 @@
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.5125000000000011</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D128" s="1">
         <v>6</v>
@@ -8192,22 +8195,22 @@
         <v>5.7</v>
       </c>
       <c r="I128" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>166</v>
+        <v>245</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D129" s="1">
         <v>6</v>
       </c>
       <c r="E129" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F129" s="1">
         <v>6</v>
@@ -8216,349 +8219,349 @@
         <v>6</v>
       </c>
       <c r="H129" s="3">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="I129" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D130" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E130" s="1">
         <v>6</v>
       </c>
       <c r="F130" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G130" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I130" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>228</v>
+        <v>191</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>5.3875000000000011</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D131" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E131" s="1">
         <v>6</v>
       </c>
       <c r="F131" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G131" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H131" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I131" s="3">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>5.3750000000000009</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D132" s="1">
         <v>6</v>
       </c>
       <c r="E132" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F132" s="1">
         <v>6</v>
       </c>
       <c r="G132" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H132" s="3">
         <v>4.7</v>
       </c>
       <c r="I132" s="3">
-        <v>4.5999999999999996</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D133" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E133" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F133" s="1">
         <v>6</v>
       </c>
       <c r="G133" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H133" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I133" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D134" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E134" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F134" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G134" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H134" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I134" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>242</v>
+        <v>182</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>5.25</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D135" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E135" s="1">
         <v>5</v>
       </c>
       <c r="F135" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G135" s="1">
         <v>5</v>
       </c>
       <c r="H135" s="3">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="I135" s="3">
-        <v>5.6</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>5.2</v>
+        <v>5.25</v>
       </c>
       <c r="D136" s="1">
         <v>6</v>
       </c>
       <c r="E136" s="1">
+        <v>5</v>
+      </c>
+      <c r="F136" s="1">
         <v>4</v>
-      </c>
-      <c r="F136" s="1">
-        <v>2</v>
       </c>
       <c r="G136" s="1">
         <v>5</v>
       </c>
       <c r="H136" s="3">
-        <v>7.1</v>
+        <v>5.7</v>
       </c>
       <c r="I136" s="3">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>74</v>
+        <v>232</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>5.1875</v>
+        <v>5.2</v>
       </c>
       <c r="D137" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E137" s="1">
+        <v>4</v>
+      </c>
+      <c r="F137" s="1">
+        <v>2</v>
+      </c>
+      <c r="G137" s="1">
         <v>5</v>
       </c>
-      <c r="F137" s="1">
-        <v>6</v>
-      </c>
-      <c r="G137" s="1">
-        <v>6</v>
-      </c>
       <c r="H137" s="3">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="I137" s="3">
-        <v>3.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D138" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E138" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F138" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G138" s="1">
         <v>6</v>
       </c>
       <c r="H138" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I138" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D139" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E139" s="1">
         <v>4</v>
       </c>
       <c r="F139" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G139" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H139" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I139" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D140" s="1">
         <v>5</v>
       </c>
       <c r="E140" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F140" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G140" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H140" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I140" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D141" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E141" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F141" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G141" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H141" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I141" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D142" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E142" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F142" s="1">
         <v>5</v>
@@ -8567,25 +8570,25 @@
         <v>6</v>
       </c>
       <c r="H142" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I142" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>241</v>
+        <v>169</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.9249999999999998</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D143" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E143" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F143" s="1">
         <v>5</v>
@@ -8594,154 +8597,154 @@
         <v>6</v>
       </c>
       <c r="H143" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I143" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>163</v>
+        <v>241</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D144" s="1">
         <v>5</v>
       </c>
       <c r="E144" s="1">
+        <v>4</v>
+      </c>
+      <c r="F144" s="1">
         <v>5</v>
       </c>
-      <c r="F144" s="1">
-        <v>3</v>
-      </c>
       <c r="G144" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H144" s="3">
         <v>5.5</v>
       </c>
       <c r="I144" s="3">
-        <v>4.8</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D145" s="1">
         <v>5</v>
       </c>
       <c r="E145" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F145" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G145" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H145" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I145" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I145" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>213</v>
+        <v>162</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.6124999999999998</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D146" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E146" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F146" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G146" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H146" s="3">
-        <v>6.7</v>
+        <v>4.8</v>
       </c>
       <c r="I146" s="3">
-        <v>5.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D147" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E147" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F147" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G147" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H147" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I147" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D148" s="1">
         <v>5</v>
       </c>
       <c r="E148" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F148" s="1">
         <v>5</v>
       </c>
       <c r="G148" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H148" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I148" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>243</v>
+        <v>135</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>4.5</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D149" s="1">
         <v>5</v>
@@ -8750,349 +8753,349 @@
         <v>4</v>
       </c>
       <c r="F149" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G149" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H149" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I149" s="3">
-        <v>5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>161</v>
+        <v>243</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5</v>
       </c>
       <c r="D150" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E150" s="1">
         <v>4</v>
       </c>
       <c r="F150" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G150" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H150" s="3">
         <v>5.5</v>
       </c>
       <c r="I150" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D151" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E151" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F151" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G151" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H151" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I151" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>207</v>
+        <v>114</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>4.3375000000000004</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D152" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E152" s="1">
+        <v>0</v>
+      </c>
+      <c r="F152" s="1">
         <v>2</v>
       </c>
-      <c r="F152" s="1">
-        <v>4</v>
-      </c>
       <c r="G152" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H152" s="3">
-        <v>6</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I152" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D153" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E153" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F153" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G153" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H153" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I153" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D154" s="1">
+        <v>5</v>
+      </c>
+      <c r="E154" s="1">
         <v>3</v>
       </c>
-      <c r="E154" s="1">
-        <v>4</v>
-      </c>
       <c r="F154" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G154" s="1">
         <v>4</v>
       </c>
       <c r="H154" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I154" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>258</v>
+        <v>173</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>4.3000000000000007</v>
+        <v>4.3125</v>
       </c>
       <c r="D155" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E155" s="1">
         <v>4</v>
       </c>
       <c r="F155" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G155" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H155" s="3">
-        <v>6.6</v>
+        <v>5.4</v>
       </c>
       <c r="I155" s="3">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>212</v>
+        <v>258</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>4.3</v>
+        <v>4.3000000000000007</v>
       </c>
       <c r="D156" s="1">
+        <v>2</v>
+      </c>
+      <c r="E156" s="1">
         <v>4</v>
-      </c>
-      <c r="E156" s="1">
-        <v>3</v>
       </c>
       <c r="F156" s="1">
         <v>3</v>
       </c>
       <c r="G156" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H156" s="3">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="I156" s="3">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D157" s="1">
         <v>4</v>
       </c>
       <c r="E157" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F157" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G157" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H157" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I157" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>4.1749999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D158" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E158" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F158" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G158" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H158" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I158" s="3">
-        <v>3.6</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>4.1625000000000005</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D159" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E159" s="1">
         <v>3</v>
       </c>
       <c r="F159" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G159" s="1">
         <v>4</v>
       </c>
       <c r="H159" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I159" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D160" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E160" s="1">
+        <v>3</v>
+      </c>
+      <c r="F160" s="1">
+        <v>3</v>
+      </c>
+      <c r="G160" s="1">
         <v>4</v>
       </c>
-      <c r="F160" s="1">
-        <v>2</v>
-      </c>
-      <c r="G160" s="1">
-        <v>5</v>
-      </c>
       <c r="H160" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I160" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D161" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E161" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F161" s="1">
         <v>2</v>
       </c>
       <c r="G161" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H161" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I161" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D162" s="1">
         <v>3</v>
@@ -9101,31 +9104,31 @@
         <v>3</v>
       </c>
       <c r="F162" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G162" s="1">
         <v>4</v>
       </c>
       <c r="H162" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="I162" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I162" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>250</v>
+        <v>199</v>
       </c>
       <c r="C163" s="5">
         <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>3.6624999999999996</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D163" s="1">
         <v>3</v>
       </c>
       <c r="E163" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F163" s="1">
         <v>3</v>
@@ -9134,333 +9137,360 @@
         <v>4</v>
       </c>
       <c r="H163" s="3">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="I163" s="3">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="164" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B164" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C164" s="5">
         <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
-        <v>3.5749999999999997</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="D164" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E164" s="1">
         <v>2</v>
       </c>
       <c r="F164" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G164" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H164" s="3">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="I164" s="3">
-        <v>5.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="165" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B165" s="2">
-        <v>180</v>
+      <c r="B165" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="C165" s="5">
         <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
-        <v>3.5625000000000004</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D165" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E165" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F165" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G165" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H165" s="3">
-        <v>4.5999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I165" s="3">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="166" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B166" s="2" t="s">
-        <v>216</v>
+      <c r="B166" s="2">
+        <v>180</v>
       </c>
       <c r="C166" s="5">
         <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D166" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E166" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F166" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G166" s="1">
         <v>3</v>
       </c>
       <c r="H166" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I166" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="167" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B167" s="2" t="s">
-        <v>248</v>
+        <v>216</v>
       </c>
       <c r="C167" s="5">
         <f>AVERAGE(D167,E167,E167,F167,G167,H167,H167,I167)</f>
-        <v>3.3375000000000004</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D167" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E167" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F167" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G167" s="1">
         <v>3</v>
       </c>
       <c r="H167" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="I167" s="3">
         <v>4.0999999999999996</v>
-      </c>
-      <c r="I167" s="3">
-        <v>3.5</v>
       </c>
     </row>
     <row r="168" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B168" s="2" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
       <c r="C168" s="5">
         <f>AVERAGE(D168,E168,E168,F168,G168,H168,H168,I168)</f>
-        <v>3.3250000000000002</v>
+        <v>3.3375000000000004</v>
       </c>
       <c r="D168" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E168" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F168" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G168" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H168" s="3">
-        <v>5.8</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I168" s="3">
-        <v>5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="169" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B169" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C169" s="5">
         <f>AVERAGE(D169,E169,E169,F169,G169,H169,H169,I169)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D169" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E169" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F169" s="1">
         <v>2</v>
       </c>
       <c r="G169" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H169" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I169" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="170" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B170" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C170" s="5">
         <f>AVERAGE(D170,E170,E170,F170,G170,H170,H170,I170)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D170" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E170" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F170" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G170" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H170" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I170" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="171" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B171" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C171" s="5">
         <f>AVERAGE(D171,E171,E171,F171,G171,H171,H171,I171)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D171" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E171" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F171" s="1">
         <v>0</v>
       </c>
       <c r="G171" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H171" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I171" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="172" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B172" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C172" s="5">
         <f>AVERAGE(D172,E172,E172,F172,G172,H172,H172,I172)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D172" s="1">
         <v>2</v>
       </c>
       <c r="E172" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F172" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G172" s="1">
         <v>2</v>
       </c>
       <c r="H172" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I172" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I172" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="173" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B173" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="C173" s="5">
         <f>AVERAGE(D173,E173,E173,F173,G173,H173,H173,I173)</f>
-        <v>2.65</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D173" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E173" s="1">
         <v>1</v>
       </c>
       <c r="F173" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G173" s="1">
         <v>2</v>
       </c>
       <c r="H173" s="3">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
       <c r="I173" s="3">
-        <v>3.8</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="174" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B174" s="2" t="s">
-        <v>174</v>
+        <v>251</v>
       </c>
       <c r="C174" s="5">
         <f>AVERAGE(D174,E174,E174,F174,G174,H174,H174,I174)</f>
-        <v>2.6375000000000002</v>
+        <v>2.65</v>
       </c>
       <c r="D174" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E174" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F174" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G174" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H174" s="3">
-        <v>7.6</v>
+        <v>4.2</v>
       </c>
       <c r="I174" s="3">
-        <v>5.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="175" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B175" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C175" s="5">
         <f>AVERAGE(D175,E175,E175,F175,G175,H175,H175,I175)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D175" s="1">
+        <v>0</v>
+      </c>
+      <c r="E175" s="1">
+        <v>0</v>
+      </c>
+      <c r="F175" s="1">
+        <v>0</v>
+      </c>
+      <c r="G175" s="1">
+        <v>0</v>
+      </c>
+      <c r="H175" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I175" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="176" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B176" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C176" s="5">
+        <f>AVERAGE(D176,E176,E176,F176,G176,H176,H176,I176)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D175" s="1">
+      <c r="D176" s="1">
         <v>2</v>
       </c>
-      <c r="E175" s="1">
+      <c r="E176" s="1">
         <v>1</v>
       </c>
-      <c r="F175" s="1">
+      <c r="F176" s="1">
         <v>2</v>
       </c>
-      <c r="G175" s="1">
+      <c r="G176" s="1">
         <v>2</v>
       </c>
-      <c r="H175" s="3">
+      <c r="H176" s="3">
         <v>4.3</v>
       </c>
-      <c r="I175" s="3">
+      <c r="I176" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 150 Varias películas de golpe
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC43094-04D3-423F-B0FC-A6F467964139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3F193DC-18E8-4847-878E-0EE50310B89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Películas" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -639,7 +640,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="265">
   <si>
     <t>Película</t>
   </si>
@@ -1425,6 +1426,15 @@
   </si>
   <si>
     <t>Susurran tu nombre</t>
+  </si>
+  <si>
+    <t>Novocaine</t>
+  </si>
+  <si>
+    <t>Pequeños detalles</t>
+  </si>
+  <si>
+    <t>Gracias equipo</t>
   </si>
 </sst>
 </file>
@@ -1513,7 +1523,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1536,9 +1546,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1777,10 +1784,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I176" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I176" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I176">
-    <sortCondition descending="1" ref="C2:C176"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I179" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I179" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I179">
+    <sortCondition descending="1" ref="C2:C179"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4752,7 +4759,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K176"/>
+  <dimension ref="B2:K179"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -7605,7 +7612,7 @@
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B107" s="9" t="s">
+      <c r="B107" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C107" s="5">
@@ -7687,68 +7694,68 @@
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>101</v>
+        <v>263</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>6.15</v>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D110" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E110" s="1">
         <v>6</v>
       </c>
       <c r="F110" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G110" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H110" s="3">
-        <v>5</v>
+        <v>6.3</v>
       </c>
       <c r="I110" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>240</v>
+        <v>101</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>6.1250000000000009</v>
+        <v>6.15</v>
       </c>
       <c r="D111" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E111" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F111" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G111" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H111" s="3">
-        <v>6.7</v>
+        <v>5</v>
       </c>
       <c r="I111" s="3">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>158</v>
+        <v>240</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>6.0874999999999995</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D112" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E112" s="1">
         <v>7</v>
@@ -7760,46 +7767,46 @@
         <v>7</v>
       </c>
       <c r="H112" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I112" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D113" s="1">
         <v>7</v>
       </c>
       <c r="E113" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F113" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G113" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H113" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I113" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D114" s="1">
         <v>7</v>
@@ -7808,25 +7815,25 @@
         <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G114" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H114" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I114" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D115" s="1">
         <v>7</v>
@@ -7838,49 +7845,49 @@
         <v>7</v>
       </c>
       <c r="G115" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H115" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I115" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
         <v>6.05</v>
       </c>
       <c r="D116" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E116" s="1">
         <v>6</v>
       </c>
       <c r="F116" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G116" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H116" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I116" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D117" s="1">
         <v>6</v>
@@ -7889,25 +7896,25 @@
         <v>6</v>
       </c>
       <c r="F117" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I117" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>257</v>
+        <v>159</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>5.9250000000000007</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D118" s="1">
         <v>6</v>
@@ -7916,133 +7923,133 @@
         <v>6</v>
       </c>
       <c r="F118" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G118" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H118" s="3">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="I118" s="3">
-        <v>5.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>195</v>
+        <v>257</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9250000000000007</v>
       </c>
       <c r="D119" s="1">
         <v>6</v>
       </c>
       <c r="E119" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F119" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G119" s="1">
         <v>6</v>
       </c>
       <c r="H119" s="3">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
       <c r="I119" s="3">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D120" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E120" s="1">
         <v>5</v>
       </c>
       <c r="F120" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G120" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I120" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D121" s="1">
         <v>7</v>
       </c>
       <c r="E121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F121" s="1">
         <v>5</v>
       </c>
       <c r="G121" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H121" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I121" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D122" s="1">
         <v>7</v>
       </c>
       <c r="E122" s="1">
+        <v>6</v>
+      </c>
+      <c r="F122" s="1">
         <v>5</v>
       </c>
-      <c r="F122" s="1">
-        <v>4</v>
-      </c>
       <c r="G122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H122" s="3">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="I122" s="3">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D123" s="1">
         <v>7</v>
@@ -8054,115 +8061,115 @@
         <v>4</v>
       </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I123" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>253</v>
+        <v>187</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.6875000000000009</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D124" s="1">
+        <v>7</v>
+      </c>
+      <c r="E124" s="1">
         <v>5</v>
       </c>
-      <c r="E124" s="1">
+      <c r="F124" s="1">
         <v>4</v>
       </c>
-      <c r="F124" s="1">
+      <c r="G124" s="1">
         <v>5</v>
-      </c>
-      <c r="G124" s="1">
-        <v>8</v>
       </c>
       <c r="H124" s="3">
         <v>6.7</v>
       </c>
       <c r="I124" s="3">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>26</v>
+        <v>253</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.6749999999999998</v>
+        <v>5.6875000000000009</v>
       </c>
       <c r="D125" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E125" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F125" s="1">
         <v>5</v>
       </c>
       <c r="G125" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H125" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I125" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D126" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E126" s="1">
+        <v>3</v>
+      </c>
+      <c r="F126" s="1">
         <v>5</v>
       </c>
-      <c r="F126" s="1">
-        <v>6</v>
-      </c>
       <c r="G126" s="1">
         <v>6</v>
       </c>
       <c r="H126" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I126" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D127" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E127" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F127" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G127" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H127" s="3">
         <v>5.8</v>
@@ -8173,26 +8180,26 @@
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>229</v>
+        <v>156</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.5375000000000005</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D128" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E128" s="1">
+        <v>6</v>
+      </c>
+      <c r="F128" s="1">
+        <v>8</v>
+      </c>
+      <c r="G128" s="1">
         <v>5</v>
       </c>
-      <c r="F128" s="1">
-        <v>6</v>
-      </c>
-      <c r="G128" s="1">
-        <v>6</v>
-      </c>
       <c r="H128" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I128" s="3">
         <v>4.9000000000000004</v>
@@ -8200,11 +8207,11 @@
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>5.5125000000000011</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D129" s="1">
         <v>6</v>
@@ -8222,22 +8229,22 @@
         <v>5.7</v>
       </c>
       <c r="I129" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>166</v>
+        <v>245</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D130" s="1">
         <v>6</v>
       </c>
       <c r="E130" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F130" s="1">
         <v>6</v>
@@ -8246,349 +8253,349 @@
         <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="I130" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E131" s="1">
         <v>6</v>
       </c>
       <c r="F131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G131" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H131" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I131" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>228</v>
+        <v>191</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>5.3875000000000011</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E132" s="1">
         <v>6</v>
       </c>
       <c r="F132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H132" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I132" s="3">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>5.3750000000000009</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D133" s="1">
         <v>6</v>
       </c>
       <c r="E133" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F133" s="1">
         <v>6</v>
       </c>
       <c r="G133" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H133" s="3">
         <v>4.7</v>
       </c>
       <c r="I133" s="3">
-        <v>4.5999999999999996</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D134" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E134" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F134" s="1">
         <v>6</v>
       </c>
       <c r="G134" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H134" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I134" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D135" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E135" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F135" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G135" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H135" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I135" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>242</v>
+        <v>182</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>5.25</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D136" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E136" s="1">
         <v>5</v>
       </c>
       <c r="F136" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G136" s="1">
         <v>5</v>
       </c>
       <c r="H136" s="3">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="I136" s="3">
-        <v>5.6</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>5.2</v>
+        <v>5.25</v>
       </c>
       <c r="D137" s="1">
         <v>6</v>
       </c>
       <c r="E137" s="1">
+        <v>5</v>
+      </c>
+      <c r="F137" s="1">
         <v>4</v>
-      </c>
-      <c r="F137" s="1">
-        <v>2</v>
       </c>
       <c r="G137" s="1">
         <v>5</v>
       </c>
       <c r="H137" s="3">
-        <v>7.1</v>
+        <v>5.7</v>
       </c>
       <c r="I137" s="3">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>74</v>
+        <v>232</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>5.1875</v>
+        <v>5.2</v>
       </c>
       <c r="D138" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E138" s="1">
+        <v>4</v>
+      </c>
+      <c r="F138" s="1">
+        <v>2</v>
+      </c>
+      <c r="G138" s="1">
         <v>5</v>
       </c>
-      <c r="F138" s="1">
-        <v>6</v>
-      </c>
-      <c r="G138" s="1">
-        <v>6</v>
-      </c>
       <c r="H138" s="3">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="I138" s="3">
-        <v>3.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D139" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E139" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F139" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G139" s="1">
         <v>6</v>
       </c>
       <c r="H139" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I139" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D140" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E140" s="1">
         <v>4</v>
       </c>
       <c r="F140" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G140" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H140" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I140" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D141" s="1">
         <v>5</v>
       </c>
       <c r="E141" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F141" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G141" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H141" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I141" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D142" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E142" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F142" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G142" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H142" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I142" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D143" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E143" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F143" s="1">
         <v>5</v>
@@ -8597,25 +8604,25 @@
         <v>6</v>
       </c>
       <c r="H143" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I143" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>241</v>
+        <v>169</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.9249999999999998</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D144" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E144" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F144" s="1">
         <v>5</v>
@@ -8624,19 +8631,19 @@
         <v>6</v>
       </c>
       <c r="H144" s="3">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I144" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>163</v>
+        <v>264</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D145" s="1">
         <v>5</v>
@@ -8645,325 +8652,325 @@
         <v>5</v>
       </c>
       <c r="F145" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G145" s="1">
         <v>5</v>
       </c>
       <c r="H145" s="3">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="I145" s="3">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>162</v>
+        <v>241</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.7875000000000005</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D146" s="1">
         <v>5</v>
       </c>
       <c r="E146" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F146" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G146" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H146" s="3">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
       <c r="I146" s="3">
-        <v>3.7</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>213</v>
+        <v>163</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>4.6124999999999998</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E147" s="1">
+        <v>5</v>
+      </c>
+      <c r="F147" s="1">
         <v>3</v>
       </c>
-      <c r="F147" s="1">
-        <v>4</v>
-      </c>
       <c r="G147" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H147" s="3">
-        <v>6.7</v>
+        <v>5.5</v>
       </c>
       <c r="I147" s="3">
-        <v>5.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.5999999999999996</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D148" s="1">
         <v>5</v>
       </c>
       <c r="E148" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F148" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G148" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H148" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.8</v>
       </c>
       <c r="I148" s="3">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>135</v>
+        <v>262</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>4.5874999999999995</v>
+        <v>4.7125000000000004</v>
       </c>
       <c r="D149" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E149" s="1">
+        <v>3</v>
+      </c>
+      <c r="F149" s="1">
         <v>4</v>
-      </c>
-      <c r="F149" s="1">
-        <v>5</v>
       </c>
       <c r="G149" s="1">
         <v>5</v>
       </c>
       <c r="H149" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.5</v>
       </c>
       <c r="I149" s="3">
-        <v>3.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>4.5</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D150" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E150" s="1">
+        <v>3</v>
+      </c>
+      <c r="F150" s="1">
         <v>4</v>
-      </c>
-      <c r="F150" s="1">
-        <v>3</v>
       </c>
       <c r="G150" s="1">
         <v>4</v>
       </c>
       <c r="H150" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I150" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I150" s="3">
-        <v>5</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D151" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E151" s="1">
+        <v>5</v>
+      </c>
+      <c r="F151" s="1">
+        <v>5</v>
+      </c>
+      <c r="G151" s="1">
+        <v>3</v>
+      </c>
+      <c r="H151" s="3">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I151" s="3">
         <v>4</v>
-      </c>
-      <c r="F151" s="1">
-        <v>6</v>
-      </c>
-      <c r="G151" s="1">
-        <v>5</v>
-      </c>
-      <c r="H151" s="3">
-        <v>5.5</v>
-      </c>
-      <c r="I151" s="3">
-        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>4.4124999999999996</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D152" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E152" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F152" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G152" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H152" s="3">
-        <v>8.1999999999999993</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I152" s="3">
-        <v>7.9</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>207</v>
+        <v>243</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>4.3375000000000004</v>
+        <v>4.5</v>
       </c>
       <c r="D153" s="1">
+        <v>5</v>
+      </c>
+      <c r="E153" s="1">
+        <v>4</v>
+      </c>
+      <c r="F153" s="1">
         <v>3</v>
       </c>
-      <c r="E153" s="1">
-        <v>2</v>
-      </c>
-      <c r="F153" s="1">
+      <c r="G153" s="1">
         <v>4</v>
       </c>
-      <c r="G153" s="1">
-        <v>7</v>
-      </c>
       <c r="H153" s="3">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="I153" s="3">
-        <v>4.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>4.3374999999999995</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D154" s="1">
+        <v>1</v>
+      </c>
+      <c r="E154" s="1">
+        <v>4</v>
+      </c>
+      <c r="F154" s="1">
+        <v>6</v>
+      </c>
+      <c r="G154" s="1">
         <v>5</v>
       </c>
-      <c r="E154" s="1">
-        <v>3</v>
-      </c>
-      <c r="F154" s="1">
-        <v>3</v>
-      </c>
-      <c r="G154" s="1">
-        <v>4</v>
-      </c>
       <c r="H154" s="3">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="I154" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>173</v>
+        <v>114</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>4.3125</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D155" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E155" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F155" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G155" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H155" s="3">
-        <v>5.4</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I155" s="3">
-        <v>4.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>258</v>
+        <v>207</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>4.3000000000000007</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D156" s="1">
+        <v>3</v>
+      </c>
+      <c r="E156" s="1">
         <v>2</v>
       </c>
-      <c r="E156" s="1">
+      <c r="F156" s="1">
         <v>4</v>
       </c>
-      <c r="F156" s="1">
-        <v>3</v>
-      </c>
       <c r="G156" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H156" s="3">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="I156" s="3">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>212</v>
+        <v>150</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>4.3</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D157" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E157" s="1">
         <v>3</v>
@@ -8975,73 +8982,73 @@
         <v>4</v>
       </c>
       <c r="H157" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I157" s="3">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3125</v>
       </c>
       <c r="D158" s="1">
+        <v>3</v>
+      </c>
+      <c r="E158" s="1">
         <v>4</v>
       </c>
-      <c r="E158" s="1">
-        <v>2</v>
-      </c>
       <c r="F158" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G158" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H158" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.4</v>
       </c>
       <c r="I158" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>236</v>
+        <v>258</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>4.1749999999999998</v>
+        <v>4.3000000000000007</v>
       </c>
       <c r="D159" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E159" s="1">
+        <v>4</v>
+      </c>
+      <c r="F159" s="1">
         <v>3</v>
       </c>
-      <c r="F159" s="1">
-        <v>4</v>
-      </c>
       <c r="G159" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H159" s="3">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
       <c r="I159" s="3">
-        <v>3.6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>233</v>
+        <v>212</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>4.1625000000000005</v>
+        <v>4.3</v>
       </c>
       <c r="D160" s="1">
         <v>4</v>
@@ -9056,76 +9063,76 @@
         <v>4</v>
       </c>
       <c r="H160" s="3">
-        <v>5.8</v>
+        <v>6.3</v>
       </c>
       <c r="I160" s="3">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>68</v>
+        <v>167</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>4.1124999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D161" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E161" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F161" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G161" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H161" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I161" s="3">
-        <v>3.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D162" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E162" s="1">
         <v>3</v>
       </c>
       <c r="F162" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G162" s="1">
         <v>4</v>
       </c>
       <c r="H162" s="3">
-        <v>5.9</v>
+        <v>5.4</v>
       </c>
       <c r="I162" s="3">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>199</v>
+        <v>233</v>
       </c>
       <c r="C163" s="5">
         <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>3.7375000000000003</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D163" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E163" s="1">
         <v>3</v>
@@ -9137,73 +9144,73 @@
         <v>4</v>
       </c>
       <c r="H163" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I163" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="164" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B164" s="2" t="s">
-        <v>250</v>
+        <v>68</v>
       </c>
       <c r="C164" s="5">
         <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
-        <v>3.6624999999999996</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D164" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E164" s="1">
+        <v>4</v>
+      </c>
+      <c r="F164" s="1">
         <v>2</v>
       </c>
-      <c r="F164" s="1">
-        <v>3</v>
-      </c>
       <c r="G164" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H164" s="3">
-        <v>5.4</v>
+        <v>4.5</v>
       </c>
       <c r="I164" s="3">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="165" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B165" s="2" t="s">
-        <v>246</v>
+        <v>218</v>
       </c>
       <c r="C165" s="5">
         <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
-        <v>3.5749999999999997</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D165" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E165" s="1">
+        <v>3</v>
+      </c>
+      <c r="F165" s="1">
         <v>2</v>
       </c>
-      <c r="F165" s="1">
-        <v>0</v>
-      </c>
       <c r="G165" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H165" s="3">
-        <v>6.2</v>
+        <v>5.9</v>
       </c>
       <c r="I165" s="3">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="166" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B166" s="2">
-        <v>180</v>
+      <c r="B166" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="C166" s="5">
         <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
-        <v>3.5625000000000004</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D166" s="1">
         <v>3</v>
@@ -9215,10 +9222,10 @@
         <v>3</v>
       </c>
       <c r="G166" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H166" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I166" s="3">
         <v>4.3</v>
@@ -9226,95 +9233,95 @@
     </row>
     <row r="167" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B167" s="2" t="s">
-        <v>216</v>
+        <v>250</v>
       </c>
       <c r="C167" s="5">
         <f>AVERAGE(D167,E167,E167,F167,G167,H167,H167,I167)</f>
-        <v>3.5375000000000005</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="D167" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E167" s="1">
         <v>2</v>
       </c>
       <c r="F167" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G167" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H167" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.4</v>
       </c>
       <c r="I167" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="168" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B168" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C168" s="5">
         <f>AVERAGE(D168,E168,E168,F168,G168,H168,H168,I168)</f>
-        <v>3.3375000000000004</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D168" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E168" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F168" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G168" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H168" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I168" s="3">
-        <v>3.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="169" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B169" s="2" t="s">
-        <v>189</v>
+      <c r="B169" s="2">
+        <v>180</v>
       </c>
       <c r="C169" s="5">
         <f>AVERAGE(D169,E169,E169,F169,G169,H169,H169,I169)</f>
-        <v>3.3250000000000002</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D169" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E169" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F169" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G169" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H169" s="3">
-        <v>5.8</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I169" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="170" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B170" s="2" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="C170" s="5">
         <f>AVERAGE(D170,E170,E170,F170,G170,H170,H170,I170)</f>
-        <v>3.2749999999999995</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D170" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E170" s="1">
         <v>2</v>
@@ -9326,154 +9333,154 @@
         <v>3</v>
       </c>
       <c r="H170" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I170" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="171" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B171" s="2" t="s">
-        <v>155</v>
+        <v>248</v>
       </c>
       <c r="C171" s="5">
         <f>AVERAGE(D171,E171,E171,F171,G171,H171,H171,I171)</f>
-        <v>2.9124999999999996</v>
+        <v>3.3375000000000004</v>
       </c>
       <c r="D171" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E171" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F171" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G171" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H171" s="3">
-        <v>6.7</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I171" s="3">
-        <v>5.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="172" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B172" s="2" t="s">
-        <v>237</v>
+        <v>189</v>
       </c>
       <c r="C172" s="5">
         <f>AVERAGE(D172,E172,E172,F172,G172,H172,H172,I172)</f>
-        <v>2.8125</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D172" s="1">
+        <v>4</v>
+      </c>
+      <c r="E172" s="1">
+        <v>1</v>
+      </c>
+      <c r="F172" s="1">
         <v>2</v>
-      </c>
-      <c r="E172" s="1">
-        <v>2</v>
-      </c>
-      <c r="F172" s="1">
-        <v>0</v>
       </c>
       <c r="G172" s="1">
         <v>2</v>
       </c>
       <c r="H172" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I172" s="3">
-        <v>5.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B173" s="2" t="s">
-        <v>239</v>
+        <v>194</v>
       </c>
       <c r="C173" s="5">
         <f>AVERAGE(D173,E173,E173,F173,G173,H173,H173,I173)</f>
-        <v>2.7625000000000002</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D173" s="1">
         <v>2</v>
       </c>
       <c r="E173" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F173" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G173" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H173" s="3">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="I173" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="174" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B174" s="2" t="s">
-        <v>251</v>
+        <v>155</v>
       </c>
       <c r="C174" s="5">
         <f>AVERAGE(D174,E174,E174,F174,G174,H174,H174,I174)</f>
-        <v>2.65</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D174" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E174" s="1">
         <v>1</v>
       </c>
       <c r="F174" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G174" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H174" s="3">
-        <v>4.2</v>
+        <v>6.7</v>
       </c>
       <c r="I174" s="3">
-        <v>3.8</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="175" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B175" s="2" t="s">
-        <v>174</v>
+        <v>237</v>
       </c>
       <c r="C175" s="5">
         <f>AVERAGE(D175,E175,E175,F175,G175,H175,H175,I175)</f>
-        <v>2.6375000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D175" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E175" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F175" s="1">
         <v>0</v>
       </c>
       <c r="G175" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H175" s="3">
-        <v>7.6</v>
+        <v>4.5</v>
       </c>
       <c r="I175" s="3">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="176" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B176" s="2" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C176" s="5">
         <f>AVERAGE(D176,E176,E176,F176,G176,H176,H176,I176)</f>
-        <v>2.5125000000000002</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D176" s="1">
         <v>2</v>
@@ -9482,15 +9489,96 @@
         <v>1</v>
       </c>
       <c r="F176" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G176" s="1">
         <v>2</v>
       </c>
       <c r="H176" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I176" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="177" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B177" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C177" s="5">
+        <f>AVERAGE(D177,E177,E177,F177,G177,H177,H177,I177)</f>
+        <v>2.65</v>
+      </c>
+      <c r="D177" s="1">
+        <v>3</v>
+      </c>
+      <c r="E177" s="1">
+        <v>1</v>
+      </c>
+      <c r="F177" s="1">
+        <v>2</v>
+      </c>
+      <c r="G177" s="1">
+        <v>2</v>
+      </c>
+      <c r="H177" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="I177" s="3">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="178" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B178" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C178" s="5">
+        <f>AVERAGE(D178,E178,E178,F178,G178,H178,H178,I178)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D178" s="1">
+        <v>0</v>
+      </c>
+      <c r="E178" s="1">
+        <v>0</v>
+      </c>
+      <c r="F178" s="1">
+        <v>0</v>
+      </c>
+      <c r="G178" s="1">
+        <v>0</v>
+      </c>
+      <c r="H178" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I178" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="179" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B179" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C179" s="5">
+        <f>AVERAGE(D179,E179,E179,F179,G179,H179,H179,I179)</f>
+        <v>2.5125000000000002</v>
+      </c>
+      <c r="D179" s="1">
+        <v>2</v>
+      </c>
+      <c r="E179" s="1">
+        <v>1</v>
+      </c>
+      <c r="F179" s="1">
+        <v>2</v>
+      </c>
+      <c r="G179" s="1">
+        <v>2</v>
+      </c>
+      <c r="H179" s="3">
         <v>4.3</v>
       </c>
-      <c r="I176" s="3">
+      <c r="I179" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 152 "Cada día nace un listo"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E192F189-692B-4127-8050-079E5A3A55F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC24B533-169C-4F69-947B-4B47FB6284D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -639,7 +639,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="273">
   <si>
     <t>Película</t>
   </si>
@@ -1437,6 +1437,27 @@
   </si>
   <si>
     <t>La odisea</t>
+  </si>
+  <si>
+    <t>Mickey 17</t>
+  </si>
+  <si>
+    <t>Al otro barrio</t>
+  </si>
+  <si>
+    <t>Unabomber</t>
+  </si>
+  <si>
+    <t>Las desapariciones</t>
+  </si>
+  <si>
+    <t>Animales</t>
+  </si>
+  <si>
+    <t>Kraven the Hunter</t>
+  </si>
+  <si>
+    <t>Cada día nace un listo</t>
   </si>
 </sst>
 </file>
@@ -1789,10 +1810,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I180" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I180" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I180">
-    <sortCondition descending="1" ref="C2:C180"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I187" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I187" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I187">
+    <sortCondition descending="1" ref="C2:C187"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4764,7 +4785,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K180"/>
+  <dimension ref="B2:K187"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -4807,7 +4828,7 @@
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="2" t="s">
         <v>265</v>
       </c>
       <c r="C3" s="5">
@@ -6268,17 +6289,17 @@
     </row>
     <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="2" t="s">
-        <v>103</v>
+        <v>181</v>
       </c>
       <c r="C57" s="5">
         <f>AVERAGE(D57,E57,E57,F57,G57,H57,H57,I57)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D57" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E57" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F57" s="1">
         <v>8</v>
@@ -6287,25 +6308,25 @@
         <v>8</v>
       </c>
       <c r="H57" s="3">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="I57" s="3">
-        <v>6</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="2" t="s">
-        <v>181</v>
+        <v>103</v>
       </c>
       <c r="C58" s="5">
         <f>AVERAGE(D58,E58,E58,F58,G58,H58,H58,I58)</f>
         <v>7.2750000000000004</v>
       </c>
       <c r="D58" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E58" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F58" s="1">
         <v>8</v>
@@ -6314,10 +6335,10 @@
         <v>8</v>
       </c>
       <c r="H58" s="3">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="I58" s="3">
-        <v>5.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
@@ -6619,68 +6640,68 @@
     </row>
     <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="2" t="s">
-        <v>98</v>
+        <v>171</v>
       </c>
       <c r="C70" s="5">
         <f>AVERAGE(D70,E70,E70,F70,G70,H70,H70,I70)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D70" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E70" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F70" s="1">
         <v>8</v>
       </c>
       <c r="G70" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H70" s="3">
-        <v>7.2</v>
+        <v>6.2</v>
       </c>
       <c r="I70" s="3">
-        <v>6.2</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
-        <v>171</v>
+        <v>98</v>
       </c>
       <c r="C71" s="5">
         <f>AVERAGE(D71,E71,E71,F71,G71,H71,H71,I71)</f>
         <v>7.0750000000000011</v>
       </c>
       <c r="D71" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E71" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" s="1">
         <v>8</v>
       </c>
       <c r="G71" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H71" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="I71" s="3">
         <v>6.2</v>
-      </c>
-      <c r="I71" s="3">
-        <v>5.2</v>
       </c>
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="C72" s="5">
         <f>AVERAGE(D72,E72,E72,F72,G72,H72,H72,I72)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D72" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E72" s="1">
         <v>7</v>
@@ -6689,25 +6710,25 @@
         <v>8</v>
       </c>
       <c r="G72" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H72" s="3">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="I72" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="2" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="C73" s="5">
         <f>AVERAGE(D73,E73,E73,F73,G73,H73,H73,I73)</f>
         <v>7.0750000000000002</v>
       </c>
       <c r="D73" s="1">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E73" s="1">
         <v>7</v>
@@ -6716,13 +6737,13 @@
         <v>8</v>
       </c>
       <c r="G73" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H73" s="3">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="I73" s="3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
@@ -7132,83 +7153,83 @@
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="2" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
       <c r="C89" s="5">
         <f>AVERAGE(D89,E89,E89,F89,G89,H89,H89,I89)</f>
-        <v>6.6124999999999998</v>
+        <v>6.6249999999999991</v>
       </c>
       <c r="D89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F89" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G89" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H89" s="3">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="I89" s="3">
-        <v>5.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="2" t="s">
-        <v>41</v>
+        <v>255</v>
       </c>
       <c r="C90" s="5">
         <f>AVERAGE(D90,E90,E90,F90,G90,H90,H90,I90)</f>
-        <v>6.6124999999999989</v>
+        <v>6.6124999999999998</v>
       </c>
       <c r="D90" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E90" s="1">
         <v>6</v>
       </c>
       <c r="F90" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G90" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H90" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I90" s="3">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="2" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="C91" s="5">
         <f>AVERAGE(D91,E91,E91,F91,G91,H91,H91,I91)</f>
-        <v>6.5874999999999995</v>
+        <v>6.6124999999999989</v>
       </c>
       <c r="D91" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E91" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G91" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H91" s="3">
         <v>6.3</v>
       </c>
       <c r="I91" s="3">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
@@ -7240,11 +7261,11 @@
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="2" t="s">
-        <v>215</v>
+        <v>117</v>
       </c>
       <c r="C93" s="5">
         <f>AVERAGE(D93,E93,E93,F93,G93,H93,H93,I93)</f>
-        <v>6.5750000000000002</v>
+        <v>6.5874999999999995</v>
       </c>
       <c r="D93" s="1">
         <v>7</v>
@@ -7259,46 +7280,46 @@
         <v>6</v>
       </c>
       <c r="H93" s="3">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="I93" s="3">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="2" t="s">
-        <v>249</v>
+        <v>215</v>
       </c>
       <c r="C94" s="5">
         <f>AVERAGE(D94,E94,E94,F94,G94,H94,H94,I94)</f>
-        <v>6.5625</v>
+        <v>6.5750000000000002</v>
       </c>
       <c r="D94" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E94" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F94" s="1">
         <v>7</v>
       </c>
       <c r="G94" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H94" s="3">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="I94" s="3">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="2" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C95" s="5">
         <f>AVERAGE(D95,E95,E95,F95,G95,H95,H95,I95)</f>
-        <v>6.5499999999999989</v>
+        <v>6.5625</v>
       </c>
       <c r="D95" s="1">
         <v>8</v>
@@ -7310,190 +7331,190 @@
         <v>7</v>
       </c>
       <c r="G95" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H95" s="3">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="I95" s="3">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="2" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="C96" s="5">
         <f>AVERAGE(D96,E96,E96,F96,G96,H96,H96,I96)</f>
-        <v>6.5375000000000005</v>
+        <v>6.5499999999999989</v>
       </c>
       <c r="D96" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E96" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" s="1">
         <v>7</v>
       </c>
       <c r="G96" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H96" s="3">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I96" s="3">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="2" t="s">
-        <v>252</v>
+        <v>197</v>
       </c>
       <c r="C97" s="5">
         <f>AVERAGE(D97,E97,E97,F97,G97,H97,H97,I97)</f>
-        <v>6.4749999999999996</v>
+        <v>6.5375000000000005</v>
       </c>
       <c r="D97" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E97" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F97" s="1">
         <v>7</v>
       </c>
       <c r="G97" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H97" s="3">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="I97" s="3">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C98" s="5">
         <f>AVERAGE(D98,E98,E98,F98,G98,H98,H98,I98)</f>
-        <v>6.4124999999999996</v>
+        <v>6.4749999999999996</v>
       </c>
       <c r="D98" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E98" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G98" s="1">
         <v>7</v>
       </c>
       <c r="H98" s="3">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="I98" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
-        <v>202</v>
+        <v>254</v>
       </c>
       <c r="C99" s="5">
         <f>AVERAGE(D99,E99,E99,F99,G99,H99,H99,I99)</f>
-        <v>6.3999999999999995</v>
+        <v>6.4124999999999996</v>
       </c>
       <c r="D99" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E99" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F99" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G99" s="1">
         <v>7</v>
       </c>
       <c r="H99" s="3">
-        <v>6.4</v>
+        <v>6.8</v>
       </c>
       <c r="I99" s="3">
-        <v>6.4</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
-        <v>256</v>
+        <v>202</v>
       </c>
       <c r="C100" s="5">
         <f>AVERAGE(D100,E100,E100,F100,G100,H100,H100,I100)</f>
-        <v>6.3625000000000007</v>
+        <v>6.3999999999999995</v>
       </c>
       <c r="D100" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E100" s="1">
         <v>6</v>
       </c>
       <c r="F100" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G100" s="1">
         <v>7</v>
       </c>
       <c r="H100" s="3">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="I100" s="3">
-        <v>5.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
-        <v>183</v>
+        <v>256</v>
       </c>
       <c r="C101" s="5">
         <f>AVERAGE(D101,E101,E101,F101,G101,H101,H101,I101)</f>
-        <v>6.3624999999999998</v>
+        <v>6.3625000000000007</v>
       </c>
       <c r="D101" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E101" s="1">
         <v>6</v>
       </c>
       <c r="F101" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G101" s="1">
         <v>7</v>
       </c>
       <c r="H101" s="3">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="I101" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
-        <v>200</v>
+        <v>183</v>
       </c>
       <c r="C102" s="5">
         <f>AVERAGE(D102,E102,E102,F102,G102,H102,H102,I102)</f>
         <v>6.3624999999999998</v>
       </c>
       <c r="D102" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E102" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F102" s="1">
         <v>7</v>
@@ -7502,79 +7523,79 @@
         <v>7</v>
       </c>
       <c r="H102" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="I102" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C103" s="5">
         <f>AVERAGE(D103,E103,E103,F103,G103,H103,H103,I103)</f>
-        <v>6.35</v>
+        <v>6.3624999999999998</v>
       </c>
       <c r="D103" s="1">
         <v>7</v>
       </c>
       <c r="E103" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F103" s="1">
         <v>7</v>
       </c>
       <c r="G103" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H103" s="3">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I103" s="3">
-        <v>5.8</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="2" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="C104" s="5">
         <f>AVERAGE(D104,E104,E104,F104,G104,H104,H104,I104)</f>
         <v>6.35</v>
       </c>
       <c r="D104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E104" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F104" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G104" s="1">
         <v>6</v>
       </c>
       <c r="H104" s="3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I104" s="3">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="2" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C105" s="5">
         <f>AVERAGE(D105,E105,E105,F105,G105,H105,H105,I105)</f>
-        <v>6.3125</v>
+        <v>6.35</v>
       </c>
       <c r="D105" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E105" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F105" s="1">
         <v>6</v>
@@ -7583,42 +7604,42 @@
         <v>6</v>
       </c>
       <c r="H105" s="3">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="I105" s="3">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="2" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C106" s="5">
         <f>AVERAGE(D106,E106,E106,F106,G106,H106,H106,I106)</f>
-        <v>6.2749999999999995</v>
+        <v>6.3125</v>
       </c>
       <c r="D106" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E106" s="1">
         <v>6</v>
       </c>
       <c r="F106" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G106" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H106" s="3">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="I106" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="2" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="C107" s="5">
         <f>AVERAGE(D107,E107,E107,F107,G107,H107,H107,I107)</f>
@@ -7628,271 +7649,271 @@
         <v>6</v>
       </c>
       <c r="E107" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G107" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H107" s="3">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="I107" s="3">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="2" t="s">
-        <v>261</v>
+        <v>64</v>
       </c>
       <c r="C108" s="5">
         <f>AVERAGE(D108,E108,E108,F108,G108,H108,H108,I108)</f>
-        <v>6.2375000000000007</v>
+        <v>6.2749999999999995</v>
       </c>
       <c r="D108" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E108" s="1">
         <v>7</v>
       </c>
       <c r="F108" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G108" s="1">
         <v>6</v>
       </c>
       <c r="H108" s="3">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="I108" s="3">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="2" t="s">
-        <v>75</v>
+        <v>261</v>
       </c>
       <c r="C109" s="5">
         <f>AVERAGE(D109,E109,E109,F109,G109,H109,H109,I109)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2375000000000007</v>
       </c>
       <c r="D109" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E109" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F109" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G109" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H109" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I109" s="3">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="2" t="s">
-        <v>19</v>
+        <v>268</v>
       </c>
       <c r="C110" s="5">
         <f>AVERAGE(D110,E110,E110,F110,G110,H110,H110,I110)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2250000000000005</v>
       </c>
       <c r="D110" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E110" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F110" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G110" s="1">
         <v>7</v>
       </c>
       <c r="H110" s="3">
-        <v>4.3</v>
+        <v>6.2</v>
       </c>
       <c r="I110" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="2" t="s">
-        <v>263</v>
+        <v>75</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>6.1624999999999996</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D111" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E111" s="1">
         <v>6</v>
       </c>
       <c r="F111" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G111" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H111" s="3">
-        <v>6.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I111" s="3">
-        <v>5.7</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>6.15</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D112" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E112" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F112" s="1">
         <v>8</v>
       </c>
       <c r="G112" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H112" s="3">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="I112" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>240</v>
+        <v>263</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>6.1250000000000009</v>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D113" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E113" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F113" s="1">
         <v>7</v>
       </c>
       <c r="G113" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H113" s="3">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="I113" s="3">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>6.0874999999999995</v>
+        <v>6.15</v>
       </c>
       <c r="D114" s="1">
         <v>7</v>
       </c>
       <c r="E114" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G114" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H114" s="3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="I114" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>6.0625</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D115" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G115" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H115" s="3">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
       <c r="I115" s="3">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>214</v>
+        <v>158</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D116" s="1">
         <v>7</v>
       </c>
       <c r="E116" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F116" s="1">
         <v>7</v>
       </c>
       <c r="G116" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H116" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I116" s="3">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>160</v>
+        <v>222</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>6.05</v>
+        <v>6.0625</v>
       </c>
       <c r="D117" s="1">
         <v>7</v>
@@ -7901,79 +7922,79 @@
         <v>6</v>
       </c>
       <c r="F117" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H117" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I117" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E118" s="1">
         <v>6</v>
       </c>
       <c r="F118" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G118" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H118" s="3">
-        <v>6.5</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I118" s="3">
-        <v>5.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D119" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E119" s="1">
         <v>6</v>
       </c>
       <c r="F119" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G119" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H119" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I119" s="3">
-        <v>5</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>257</v>
+        <v>206</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
-        <v>5.9250000000000007</v>
+        <v>6.05</v>
       </c>
       <c r="D120" s="1">
         <v>6</v>
@@ -7982,106 +8003,106 @@
         <v>6</v>
       </c>
       <c r="F120" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G120" s="1">
         <v>6</v>
       </c>
       <c r="H120" s="3">
-        <v>5.6</v>
+        <v>6.5</v>
       </c>
       <c r="I120" s="3">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D121" s="1">
         <v>6</v>
       </c>
       <c r="E121" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F121" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G121" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H121" s="3">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="I121" s="3">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>186</v>
+        <v>257</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.8125000000000009</v>
+        <v>5.9250000000000007</v>
       </c>
       <c r="D122" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E122" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F122" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G122" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H122" s="3">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="I122" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D123" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E123" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>6.1</v>
+        <v>6.7</v>
       </c>
       <c r="I123" s="3">
-        <v>5.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>113</v>
+        <v>186</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D124" s="1">
         <v>7</v>
@@ -8090,187 +8111,187 @@
         <v>5</v>
       </c>
       <c r="F124" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G124" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H124" s="3">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="I124" s="3">
-        <v>5.3</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>187</v>
+        <v>209</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.7250000000000005</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D125" s="1">
         <v>7</v>
       </c>
       <c r="E125" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F125" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G125" s="1">
         <v>5</v>
       </c>
       <c r="H125" s="3">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
       <c r="I125" s="3">
-        <v>6.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
-        <v>5.6875000000000009</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D126" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E126" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F126" s="1">
         <v>5</v>
       </c>
       <c r="G126" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H126" s="3">
         <v>6.7</v>
       </c>
       <c r="I126" s="3">
-        <v>6.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>26</v>
+        <v>113</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>5.6749999999999998</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D127" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E127" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F127" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G127" s="1">
         <v>6</v>
       </c>
       <c r="H127" s="3">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="I127" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>149</v>
+        <v>187</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.5624999999999991</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D128" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E128" s="1">
         <v>5</v>
       </c>
       <c r="F128" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G128" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H128" s="3">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
       <c r="I128" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>156</v>
+        <v>253</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6875000000000009</v>
       </c>
       <c r="D129" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E129" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F129" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G129" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H129" s="3">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
       <c r="I129" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>229</v>
+        <v>26</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>5.5375000000000005</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D130" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E130" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F130" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G130" s="1">
         <v>6</v>
       </c>
       <c r="H130" s="3">
-        <v>5.7</v>
+        <v>7</v>
       </c>
       <c r="I130" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>245</v>
+        <v>149</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>5.5125000000000011</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D131" s="1">
         <v>6</v>
@@ -8285,79 +8306,79 @@
         <v>6</v>
       </c>
       <c r="H131" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I131" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D132" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E132" s="1">
         <v>6</v>
       </c>
       <c r="F132" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H132" s="3">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="I132" s="3">
-        <v>4.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>191</v>
+        <v>229</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D133" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E133" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F133" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G133" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H133" s="3">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="I133" s="3">
-        <v>5.3</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>228</v>
+        <v>245</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>5.3875000000000011</v>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D134" s="1">
         <v>6</v>
       </c>
       <c r="E134" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F134" s="1">
         <v>6</v>
@@ -8366,100 +8387,100 @@
         <v>6</v>
       </c>
       <c r="H134" s="3">
+        <v>5.7</v>
+      </c>
+      <c r="I134" s="3">
         <v>4.7</v>
-      </c>
-      <c r="I134" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>204</v>
+        <v>166</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>5.3750000000000009</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D135" s="1">
         <v>6</v>
       </c>
       <c r="E135" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F135" s="1">
         <v>6</v>
       </c>
       <c r="G135" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H135" s="3">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="I135" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
-        <v>5.375</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D136" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E136" s="1">
         <v>6</v>
       </c>
       <c r="F136" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G136" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H136" s="3">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="I136" s="3">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>182</v>
+        <v>228</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>5.2875000000000005</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G137" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H137" s="3">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="I137" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>242</v>
+        <v>204</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>5.25</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D138" s="1">
         <v>6</v>
@@ -8468,160 +8489,160 @@
         <v>5</v>
       </c>
       <c r="F138" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G138" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H138" s="3">
-        <v>5.7</v>
+        <v>4.7</v>
       </c>
       <c r="I138" s="3">
-        <v>5.6</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>232</v>
+        <v>190</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>5.2</v>
+        <v>5.375</v>
       </c>
       <c r="D139" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E139" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F139" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G139" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H139" s="3">
-        <v>7.1</v>
+        <v>5.6</v>
       </c>
       <c r="I139" s="3">
-        <v>6.4</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>5.1875</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D140" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E140" s="1">
         <v>5</v>
       </c>
       <c r="F140" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G140" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H140" s="3">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="I140" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>145</v>
+        <v>242</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>5.1124999999999998</v>
+        <v>5.25</v>
       </c>
       <c r="D141" s="1">
         <v>6</v>
       </c>
       <c r="E141" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F141" s="1">
         <v>4</v>
       </c>
       <c r="G141" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H141" s="3">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="I141" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>223</v>
+        <v>271</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>5.0750000000000002</v>
+        <v>5.2374999999999998</v>
       </c>
       <c r="D142" s="1">
         <v>5</v>
       </c>
       <c r="E142" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F142" s="1">
         <v>5</v>
       </c>
       <c r="G142" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H142" s="3">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="I142" s="3">
-        <v>5</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>21</v>
+        <v>232</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>5.05</v>
+        <v>5.2</v>
       </c>
       <c r="D143" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E143" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F143" s="1">
         <v>2</v>
       </c>
       <c r="G143" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H143" s="3">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="I143" s="3">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>203</v>
+        <v>74</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>4.9875000000000007</v>
+        <v>5.1875</v>
       </c>
       <c r="D144" s="1">
         <v>7</v>
@@ -8630,58 +8651,58 @@
         <v>5</v>
       </c>
       <c r="F144" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G144" s="1">
         <v>6</v>
       </c>
       <c r="H144" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="I144" s="3">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>4.9874999999999998</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D145" s="1">
         <v>6</v>
       </c>
       <c r="E145" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F145" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G145" s="1">
         <v>6</v>
       </c>
       <c r="H145" s="3">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="I145" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>264</v>
+        <v>223</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>4.9874999999999998</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D146" s="1">
         <v>5</v>
       </c>
       <c r="E146" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F146" s="1">
         <v>5</v>
@@ -8690,154 +8711,154 @@
         <v>5</v>
       </c>
       <c r="H146" s="3">
-        <v>5.2</v>
+        <v>6.3</v>
       </c>
       <c r="I146" s="3">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>241</v>
+        <v>21</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>4.9249999999999998</v>
+        <v>5.05</v>
       </c>
       <c r="D147" s="1">
         <v>5</v>
       </c>
       <c r="E147" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F147" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G147" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H147" s="3">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
       <c r="I147" s="3">
-        <v>4.4000000000000004</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>163</v>
+        <v>203</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D148" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E148" s="1">
         <v>5</v>
       </c>
       <c r="F148" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G148" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H148" s="3">
-        <v>5.5</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I148" s="3">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>4.7875000000000005</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D149" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E149" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F149" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G149" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H149" s="3">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="I149" s="3">
-        <v>3.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
-        <v>4.7125000000000004</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D150" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E150" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F150" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G150" s="1">
         <v>5</v>
       </c>
       <c r="H150" s="3">
-        <v>6.5</v>
+        <v>5.2</v>
       </c>
       <c r="I150" s="3">
-        <v>5.7</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>4.6124999999999998</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D151" s="1">
+        <v>5</v>
+      </c>
+      <c r="E151" s="1">
         <v>4</v>
       </c>
-      <c r="E151" s="1">
-        <v>3</v>
-      </c>
       <c r="F151" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G151" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H151" s="3">
-        <v>6.7</v>
+        <v>5.5</v>
       </c>
       <c r="I151" s="3">
-        <v>5.5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>4.5999999999999996</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D152" s="1">
         <v>5</v>
@@ -8846,268 +8867,268 @@
         <v>5</v>
       </c>
       <c r="F152" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G152" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H152" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.5</v>
       </c>
       <c r="I152" s="3">
-        <v>4</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>4.5874999999999995</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D153" s="1">
         <v>5</v>
       </c>
       <c r="E153" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F153" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G153" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H153" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.8</v>
       </c>
       <c r="I153" s="3">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>243</v>
+        <v>262</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>4.5</v>
+        <v>4.7125000000000004</v>
       </c>
       <c r="D154" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E154" s="1">
+        <v>3</v>
+      </c>
+      <c r="F154" s="1">
         <v>4</v>
       </c>
-      <c r="F154" s="1">
-        <v>3</v>
-      </c>
       <c r="G154" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H154" s="3">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="I154" s="3">
-        <v>5</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>161</v>
+        <v>270</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>4.4249999999999998</v>
+        <v>4.6875</v>
       </c>
       <c r="D155" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E155" s="1">
         <v>4</v>
       </c>
       <c r="F155" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G155" s="1">
         <v>5</v>
       </c>
       <c r="H155" s="3">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="I155" s="3">
-        <v>4.4000000000000004</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>114</v>
+        <v>213</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>4.4124999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D156" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E156" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F156" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G156" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H156" s="3">
-        <v>8.1999999999999993</v>
+        <v>6.7</v>
       </c>
       <c r="I156" s="3">
-        <v>7.9</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>207</v>
+        <v>154</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>4.3375000000000004</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D157" s="1">
+        <v>5</v>
+      </c>
+      <c r="E157" s="1">
+        <v>5</v>
+      </c>
+      <c r="F157" s="1">
+        <v>5</v>
+      </c>
+      <c r="G157" s="1">
         <v>3</v>
       </c>
-      <c r="E157" s="1">
-        <v>2</v>
-      </c>
-      <c r="F157" s="1">
+      <c r="H157" s="3">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I157" s="3">
         <v>4</v>
-      </c>
-      <c r="G157" s="1">
-        <v>7</v>
-      </c>
-      <c r="H157" s="3">
-        <v>6</v>
-      </c>
-      <c r="I157" s="3">
-        <v>4.7</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>4.3374999999999995</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D158" s="1">
         <v>5</v>
       </c>
       <c r="E158" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F158" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G158" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H158" s="3">
-        <v>5.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I158" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>173</v>
+        <v>243</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>4.3125</v>
+        <v>4.5</v>
       </c>
       <c r="D159" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E159" s="1">
         <v>4</v>
       </c>
       <c r="F159" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G159" s="1">
         <v>4</v>
       </c>
       <c r="H159" s="3">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="I159" s="3">
-        <v>4.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>258</v>
+        <v>161</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>4.3000000000000007</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D160" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E160" s="1">
         <v>4</v>
       </c>
       <c r="F160" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G160" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H160" s="3">
-        <v>6.6</v>
+        <v>5.5</v>
       </c>
       <c r="I160" s="3">
-        <v>5.2</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>212</v>
+        <v>114</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>4.3</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D161" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E161" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F161" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G161" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H161" s="3">
-        <v>6.3</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I161" s="3">
-        <v>4.8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>167</v>
+        <v>267</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
-        <v>4.2749999999999995</v>
+        <v>4.375</v>
       </c>
       <c r="D162" s="1">
         <v>4</v>
@@ -9122,49 +9143,49 @@
         <v>6</v>
       </c>
       <c r="H162" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.2</v>
       </c>
       <c r="I162" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="C163" s="5">
         <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>4.1749999999999998</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D163" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E163" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F163" s="1">
         <v>4</v>
       </c>
       <c r="G163" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H163" s="3">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="I163" s="3">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="164" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B164" s="2" t="s">
-        <v>233</v>
+        <v>150</v>
       </c>
       <c r="C164" s="5">
         <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
-        <v>4.1625000000000005</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D164" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E164" s="1">
         <v>3</v>
@@ -9176,76 +9197,76 @@
         <v>4</v>
       </c>
       <c r="H164" s="3">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="I164" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="165" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B165" s="2" t="s">
-        <v>68</v>
+        <v>173</v>
       </c>
       <c r="C165" s="5">
         <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
-        <v>4.1124999999999998</v>
+        <v>4.3125</v>
       </c>
       <c r="D165" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E165" s="1">
         <v>4</v>
       </c>
       <c r="F165" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G165" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H165" s="3">
-        <v>4.5</v>
+        <v>5.4</v>
       </c>
       <c r="I165" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="166" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B166" s="2" t="s">
-        <v>218</v>
+        <v>258</v>
       </c>
       <c r="C166" s="5">
         <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
-        <v>3.9499999999999997</v>
+        <v>4.3000000000000007</v>
       </c>
       <c r="D166" s="1">
+        <v>2</v>
+      </c>
+      <c r="E166" s="1">
+        <v>4</v>
+      </c>
+      <c r="F166" s="1">
         <v>3</v>
       </c>
-      <c r="E166" s="1">
+      <c r="G166" s="1">
         <v>3</v>
       </c>
-      <c r="F166" s="1">
-        <v>2</v>
-      </c>
-      <c r="G166" s="1">
-        <v>4</v>
-      </c>
       <c r="H166" s="3">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="I166" s="3">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="167" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B167" s="2" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C167" s="5">
         <f>AVERAGE(D167,E167,E167,F167,G167,H167,H167,I167)</f>
-        <v>3.7375000000000003</v>
+        <v>4.3</v>
       </c>
       <c r="D167" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E167" s="1">
         <v>3</v>
@@ -9257,76 +9278,76 @@
         <v>4</v>
       </c>
       <c r="H167" s="3">
+        <v>6.3</v>
+      </c>
+      <c r="I167" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I167" s="3">
-        <v>4.3</v>
       </c>
     </row>
     <row r="168" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B168" s="2" t="s">
-        <v>250</v>
+        <v>167</v>
       </c>
       <c r="C168" s="5">
         <f>AVERAGE(D168,E168,E168,F168,G168,H168,H168,I168)</f>
-        <v>3.6624999999999996</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D168" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E168" s="1">
         <v>2</v>
       </c>
       <c r="F168" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G168" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H168" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I168" s="3">
-        <v>4.5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="169" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B169" s="2" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="C169" s="5">
         <f>AVERAGE(D169,E169,E169,F169,G169,H169,H169,I169)</f>
-        <v>3.5749999999999997</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D169" s="1">
         <v>5</v>
       </c>
       <c r="E169" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F169" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G169" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H169" s="3">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="I169" s="3">
-        <v>5.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="170" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B170" s="2">
-        <v>180</v>
+      <c r="B170" s="2" t="s">
+        <v>233</v>
       </c>
       <c r="C170" s="5">
         <f>AVERAGE(D170,E170,E170,F170,G170,H170,H170,I170)</f>
-        <v>3.5625000000000004</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D170" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E170" s="1">
         <v>3</v>
@@ -9335,49 +9356,49 @@
         <v>3</v>
       </c>
       <c r="G170" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H170" s="3">
-        <v>4.5999999999999996</v>
+        <v>5.8</v>
       </c>
       <c r="I170" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="171" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B171" s="2" t="s">
-        <v>216</v>
+        <v>68</v>
       </c>
       <c r="C171" s="5">
         <f>AVERAGE(D171,E171,E171,F171,G171,H171,H171,I171)</f>
-        <v>3.5375000000000005</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D171" s="1">
         <v>5</v>
       </c>
       <c r="E171" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F171" s="1">
         <v>2</v>
       </c>
       <c r="G171" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H171" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="I171" s="3">
-        <v>4.0999999999999996</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="172" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B172" s="2" t="s">
-        <v>248</v>
+        <v>218</v>
       </c>
       <c r="C172" s="5">
         <f>AVERAGE(D172,E172,E172,F172,G172,H172,H172,I172)</f>
-        <v>3.3375000000000004</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D172" s="1">
         <v>3</v>
@@ -9386,109 +9407,109 @@
         <v>3</v>
       </c>
       <c r="F172" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G172" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H172" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I172" s="3">
-        <v>3.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="173" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B173" s="2" t="s">
-        <v>189</v>
+      <c r="B173" s="9" t="s">
+        <v>272</v>
       </c>
       <c r="C173" s="5">
         <f>AVERAGE(D173,E173,E173,F173,G173,H173,H173,I173)</f>
-        <v>3.3250000000000002</v>
+        <v>3.9125000000000001</v>
       </c>
       <c r="D173" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E173" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F173" s="1">
         <v>2</v>
       </c>
       <c r="G173" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H173" s="3">
-        <v>5.8</v>
+        <v>5.3</v>
       </c>
       <c r="I173" s="3">
-        <v>5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="174" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B174" s="2" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C174" s="5">
         <f>AVERAGE(D174,E174,E174,F174,G174,H174,H174,I174)</f>
-        <v>3.2749999999999995</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D174" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E174" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F174" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G174" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H174" s="3">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="I174" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="175" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B175" s="2" t="s">
-        <v>155</v>
+        <v>250</v>
       </c>
       <c r="C175" s="5">
         <f>AVERAGE(D175,E175,E175,F175,G175,H175,H175,I175)</f>
-        <v>2.9124999999999996</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="D175" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E175" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F175" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G175" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H175" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I175" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="176" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B176" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C176" s="5">
         <f>AVERAGE(D176,E176,E176,F176,G176,H176,H176,I176)</f>
-        <v>2.8125</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D176" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E176" s="1">
         <v>2</v>
@@ -9500,103 +9521,103 @@
         <v>2</v>
       </c>
       <c r="H176" s="3">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
       <c r="I176" s="3">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="177" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B177" s="2" t="s">
-        <v>239</v>
+      <c r="B177" s="2">
+        <v>180</v>
       </c>
       <c r="C177" s="5">
         <f>AVERAGE(D177,E177,E177,F177,G177,H177,H177,I177)</f>
-        <v>2.7625000000000002</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D177" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E177" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F177" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G177" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H177" s="3">
-        <v>5.5</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I177" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="178" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B178" s="2" t="s">
-        <v>251</v>
+        <v>216</v>
       </c>
       <c r="C178" s="5">
         <f>AVERAGE(D178,E178,E178,F178,G178,H178,H178,I178)</f>
-        <v>2.65</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D178" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E178" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F178" s="1">
         <v>2</v>
       </c>
       <c r="G178" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H178" s="3">
-        <v>4.2</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I178" s="3">
-        <v>3.8</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="179" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B179" s="2" t="s">
-        <v>174</v>
+        <v>248</v>
       </c>
       <c r="C179" s="5">
         <f>AVERAGE(D179,E179,E179,F179,G179,H179,H179,I179)</f>
-        <v>2.6375000000000002</v>
+        <v>3.3375000000000004</v>
       </c>
       <c r="D179" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E179" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F179" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G179" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H179" s="3">
-        <v>7.6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I179" s="3">
-        <v>5.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="180" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B180" s="2" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="C180" s="5">
         <f>AVERAGE(D180,E180,E180,F180,G180,H180,H180,I180)</f>
-        <v>2.5125000000000002</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D180" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E180" s="1">
         <v>1</v>
@@ -9608,9 +9629,198 @@
         <v>2</v>
       </c>
       <c r="H180" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="I180" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="181" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B181" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C181" s="5">
+        <f>AVERAGE(D181,E181,E181,F181,G181,H181,H181,I181)</f>
+        <v>3.2749999999999995</v>
+      </c>
+      <c r="D181" s="1">
+        <v>2</v>
+      </c>
+      <c r="E181" s="1">
+        <v>2</v>
+      </c>
+      <c r="F181" s="1">
+        <v>2</v>
+      </c>
+      <c r="G181" s="1">
+        <v>3</v>
+      </c>
+      <c r="H181" s="3">
+        <v>5.4</v>
+      </c>
+      <c r="I181" s="3">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="182" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B182" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C182" s="5">
+        <f>AVERAGE(D182,E182,E182,F182,G182,H182,H182,I182)</f>
+        <v>2.9124999999999996</v>
+      </c>
+      <c r="D182" s="1">
+        <v>1</v>
+      </c>
+      <c r="E182" s="1">
+        <v>1</v>
+      </c>
+      <c r="F182" s="1">
+        <v>0</v>
+      </c>
+      <c r="G182" s="1">
+        <v>1</v>
+      </c>
+      <c r="H182" s="3">
+        <v>6.7</v>
+      </c>
+      <c r="I182" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="183" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B183" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C183" s="5">
+        <f>AVERAGE(D183,E183,E183,F183,G183,H183,H183,I183)</f>
+        <v>2.8125</v>
+      </c>
+      <c r="D183" s="1">
+        <v>2</v>
+      </c>
+      <c r="E183" s="1">
+        <v>2</v>
+      </c>
+      <c r="F183" s="1">
+        <v>0</v>
+      </c>
+      <c r="G183" s="1">
+        <v>2</v>
+      </c>
+      <c r="H183" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I183" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="184" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B184" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C184" s="5">
+        <f>AVERAGE(D184,E184,E184,F184,G184,H184,H184,I184)</f>
+        <v>2.7625000000000002</v>
+      </c>
+      <c r="D184" s="1">
+        <v>2</v>
+      </c>
+      <c r="E184" s="1">
+        <v>1</v>
+      </c>
+      <c r="F184" s="1">
+        <v>1</v>
+      </c>
+      <c r="G184" s="1">
+        <v>2</v>
+      </c>
+      <c r="H184" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I184" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="185" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B185" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C185" s="5">
+        <f>AVERAGE(D185,E185,E185,F185,G185,H185,H185,I185)</f>
+        <v>2.65</v>
+      </c>
+      <c r="D185" s="1">
+        <v>3</v>
+      </c>
+      <c r="E185" s="1">
+        <v>1</v>
+      </c>
+      <c r="F185" s="1">
+        <v>2</v>
+      </c>
+      <c r="G185" s="1">
+        <v>2</v>
+      </c>
+      <c r="H185" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="I185" s="3">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="186" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B186" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C186" s="5">
+        <f>AVERAGE(D186,E186,E186,F186,G186,H186,H186,I186)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D186" s="1">
+        <v>0</v>
+      </c>
+      <c r="E186" s="1">
+        <v>0</v>
+      </c>
+      <c r="F186" s="1">
+        <v>0</v>
+      </c>
+      <c r="G186" s="1">
+        <v>0</v>
+      </c>
+      <c r="H186" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I186" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="187" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B187" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C187" s="5">
+        <f>AVERAGE(D187,E187,E187,F187,G187,H187,H187,I187)</f>
+        <v>2.5125000000000002</v>
+      </c>
+      <c r="D187" s="1">
+        <v>2</v>
+      </c>
+      <c r="E187" s="1">
+        <v>1</v>
+      </c>
+      <c r="F187" s="1">
+        <v>2</v>
+      </c>
+      <c r="G187" s="1">
+        <v>2</v>
+      </c>
+      <c r="H187" s="3">
         <v>4.3</v>
       </c>
-      <c r="I180" s="3">
+      <c r="I187" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
V. 153 "Sangre y oro"
</commit_message>
<xml_diff>
--- a/Calificacion.xlsx
+++ b/Calificacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC24B533-169C-4F69-947B-4B47FB6284D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C966779-701A-405E-B539-EE58EE986564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -639,7 +639,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="274">
   <si>
     <t>Película</t>
   </si>
@@ -1458,6 +1458,9 @@
   </si>
   <si>
     <t>Cada día nace un listo</t>
+  </si>
+  <si>
+    <t>Sangre y oro</t>
   </si>
 </sst>
 </file>
@@ -1810,10 +1813,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I187" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="B2:I187" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I187">
-    <sortCondition descending="1" ref="C2:C187"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}" name="Tabla24" displayName="Tabla24" ref="B2:I188" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="B2:I188" xr:uid="{BCA867C2-0242-44D1-BB58-FF0B1A23C5D8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:I188">
+    <sortCondition descending="1" ref="C2:C188"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{349FB812-864A-4C0A-99F7-6285DFA6525F}" name="Película" dataDxfId="21"/>
@@ -4785,7 +4788,7 @@
     <tabColor theme="9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K187"/>
+  <dimension ref="B2:K188"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
@@ -7746,150 +7749,150 @@
       </c>
     </row>
     <row r="111" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B111" s="2" t="s">
-        <v>75</v>
+      <c r="B111" s="9" t="s">
+        <v>273</v>
       </c>
       <c r="C111" s="5">
         <f>AVERAGE(D111,E111,E111,F111,G111,H111,H111,I111)</f>
-        <v>6.2125000000000004</v>
+        <v>6.2249999999999996</v>
       </c>
       <c r="D111" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E111" s="1">
         <v>6</v>
       </c>
       <c r="F111" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G111" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H111" s="3">
-        <v>5.0999999999999996</v>
+        <v>6.5</v>
       </c>
       <c r="I111" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="2" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C112" s="5">
         <f>AVERAGE(D112,E112,E112,F112,G112,H112,H112,I112)</f>
-        <v>6.2124999999999995</v>
+        <v>6.2125000000000004</v>
       </c>
       <c r="D112" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E112" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F112" s="1">
         <v>8</v>
       </c>
       <c r="G112" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H112" s="3">
-        <v>4.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I112" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="2" t="s">
-        <v>263</v>
+        <v>19</v>
       </c>
       <c r="C113" s="5">
         <f>AVERAGE(D113,E113,E113,F113,G113,H113,H113,I113)</f>
-        <v>6.1624999999999996</v>
+        <v>6.2124999999999995</v>
       </c>
       <c r="D113" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E113" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F113" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G113" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H113" s="3">
-        <v>6.3</v>
+        <v>4.3</v>
       </c>
       <c r="I113" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="2" t="s">
-        <v>101</v>
+        <v>263</v>
       </c>
       <c r="C114" s="5">
         <f>AVERAGE(D114,E114,E114,F114,G114,H114,H114,I114)</f>
-        <v>6.15</v>
+        <v>6.1624999999999996</v>
       </c>
       <c r="D114" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E114" s="1">
         <v>6</v>
       </c>
       <c r="F114" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G114" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H114" s="3">
-        <v>5</v>
+        <v>6.3</v>
       </c>
       <c r="I114" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="2" t="s">
-        <v>240</v>
+        <v>101</v>
       </c>
       <c r="C115" s="5">
         <f>AVERAGE(D115,E115,E115,F115,G115,H115,H115,I115)</f>
-        <v>6.1250000000000009</v>
+        <v>6.15</v>
       </c>
       <c r="D115" s="1">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E115" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F115" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G115" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H115" s="3">
-        <v>6.7</v>
+        <v>5</v>
       </c>
       <c r="I115" s="3">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="2" t="s">
-        <v>158</v>
+        <v>240</v>
       </c>
       <c r="C116" s="5">
         <f>AVERAGE(D116,E116,E116,F116,G116,H116,H116,I116)</f>
-        <v>6.0874999999999995</v>
+        <v>6.1250000000000009</v>
       </c>
       <c r="D116" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E116" s="1">
         <v>7</v>
@@ -7901,46 +7904,46 @@
         <v>7</v>
       </c>
       <c r="H116" s="3">
-        <v>4.8</v>
+        <v>6.7</v>
       </c>
       <c r="I116" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="2" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="C117" s="5">
         <f>AVERAGE(D117,E117,E117,F117,G117,H117,H117,I117)</f>
-        <v>6.0625</v>
+        <v>6.0874999999999995</v>
       </c>
       <c r="D117" s="1">
         <v>7</v>
       </c>
       <c r="E117" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F117" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G117" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H117" s="3">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="I117" s="3">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C118" s="5">
         <f>AVERAGE(D118,E118,E118,F118,G118,H118,H118,I118)</f>
-        <v>6.0500000000000007</v>
+        <v>6.0625</v>
       </c>
       <c r="D118" s="1">
         <v>7</v>
@@ -7949,25 +7952,25 @@
         <v>6</v>
       </c>
       <c r="F118" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G118" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H118" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.9</v>
       </c>
       <c r="I118" s="3">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="2" t="s">
-        <v>160</v>
+        <v>214</v>
       </c>
       <c r="C119" s="5">
         <f>AVERAGE(D119,E119,E119,F119,G119,H119,H119,I119)</f>
-        <v>6.05</v>
+        <v>6.0500000000000007</v>
       </c>
       <c r="D119" s="1">
         <v>7</v>
@@ -7979,49 +7982,49 @@
         <v>7</v>
       </c>
       <c r="G119" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H119" s="3">
-        <v>5.4</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="I119" s="3">
-        <v>4.5999999999999996</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="2" t="s">
-        <v>206</v>
+        <v>160</v>
       </c>
       <c r="C120" s="5">
         <f>AVERAGE(D120,E120,E120,F120,G120,H120,H120,I120)</f>
         <v>6.05</v>
       </c>
       <c r="D120" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E120" s="1">
         <v>6</v>
       </c>
       <c r="F120" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G120" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H120" s="3">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="I120" s="3">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="2" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
       <c r="C121" s="5">
         <f>AVERAGE(D121,E121,E121,F121,G121,H121,H121,I121)</f>
-        <v>5.9499999999999993</v>
+        <v>6.05</v>
       </c>
       <c r="D121" s="1">
         <v>6</v>
@@ -8030,25 +8033,25 @@
         <v>6</v>
       </c>
       <c r="F121" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G121" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H121" s="3">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="I121" s="3">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="2" t="s">
-        <v>257</v>
+        <v>159</v>
       </c>
       <c r="C122" s="5">
         <f>AVERAGE(D122,E122,E122,F122,G122,H122,H122,I122)</f>
-        <v>5.9250000000000007</v>
+        <v>5.9499999999999993</v>
       </c>
       <c r="D122" s="1">
         <v>6</v>
@@ -8057,102 +8060,102 @@
         <v>6</v>
       </c>
       <c r="F122" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G122" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H122" s="3">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="I122" s="3">
-        <v>5.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="2" t="s">
-        <v>195</v>
+        <v>257</v>
       </c>
       <c r="C123" s="5">
         <f>AVERAGE(D123,E123,E123,F123,G123,H123,H123,I123)</f>
-        <v>5.8875000000000011</v>
+        <v>5.9250000000000007</v>
       </c>
       <c r="D123" s="1">
         <v>6</v>
       </c>
       <c r="E123" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F123" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G123" s="1">
         <v>6</v>
       </c>
       <c r="H123" s="3">
-        <v>6.7</v>
+        <v>5.6</v>
       </c>
       <c r="I123" s="3">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="2" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C124" s="5">
         <f>AVERAGE(D124,E124,E124,F124,G124,H124,H124,I124)</f>
-        <v>5.8125000000000009</v>
+        <v>5.8875000000000011</v>
       </c>
       <c r="D124" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E124" s="1">
         <v>5</v>
       </c>
       <c r="F124" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G124" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H124" s="3">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
       <c r="I124" s="3">
-        <v>5.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="2" t="s">
-        <v>209</v>
+        <v>186</v>
       </c>
       <c r="C125" s="5">
         <f>AVERAGE(D125,E125,E125,F125,G125,H125,H125,I125)</f>
-        <v>5.8000000000000007</v>
+        <v>5.8125000000000009</v>
       </c>
       <c r="D125" s="1">
         <v>7</v>
       </c>
       <c r="E125" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F125" s="1">
         <v>5</v>
       </c>
       <c r="G125" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H125" s="3">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="I125" s="3">
-        <v>5.2</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="2" t="s">
-        <v>266</v>
+        <v>209</v>
       </c>
       <c r="C126" s="5">
         <f>AVERAGE(D126,E126,E126,F126,G126,H126,H126,I126)</f>
@@ -8162,7 +8165,7 @@
         <v>7</v>
       </c>
       <c r="E126" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F126" s="1">
         <v>5</v>
@@ -8171,19 +8174,19 @@
         <v>5</v>
       </c>
       <c r="H126" s="3">
-        <v>6.7</v>
+        <v>6.1</v>
       </c>
       <c r="I126" s="3">
-        <v>6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="2" t="s">
-        <v>113</v>
+        <v>266</v>
       </c>
       <c r="C127" s="5">
         <f>AVERAGE(D127,E127,E127,F127,G127,H127,H127,I127)</f>
-        <v>5.7374999999999989</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D127" s="1">
         <v>7</v>
@@ -8192,25 +8195,25 @@
         <v>5</v>
       </c>
       <c r="F127" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G127" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H127" s="3">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="I127" s="3">
-        <v>5.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="2" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="C128" s="5">
         <f>AVERAGE(D128,E128,E128,F128,G128,H128,H128,I128)</f>
-        <v>5.7250000000000005</v>
+        <v>5.7374999999999989</v>
       </c>
       <c r="D128" s="1">
         <v>7</v>
@@ -8222,115 +8225,115 @@
         <v>4</v>
       </c>
       <c r="G128" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H128" s="3">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="I128" s="3">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="2" t="s">
-        <v>253</v>
+        <v>187</v>
       </c>
       <c r="C129" s="5">
         <f>AVERAGE(D129,E129,E129,F129,G129,H129,H129,I129)</f>
-        <v>5.6875000000000009</v>
+        <v>5.7250000000000005</v>
       </c>
       <c r="D129" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E129" s="1">
+        <v>5</v>
+      </c>
+      <c r="F129" s="1">
         <v>4</v>
       </c>
-      <c r="F129" s="1">
-        <v>5</v>
-      </c>
       <c r="G129" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H129" s="3">
         <v>6.7</v>
       </c>
       <c r="I129" s="3">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="2" t="s">
-        <v>26</v>
+        <v>253</v>
       </c>
       <c r="C130" s="5">
         <f>AVERAGE(D130,E130,E130,F130,G130,H130,H130,I130)</f>
-        <v>5.6749999999999998</v>
+        <v>5.6875000000000009</v>
       </c>
       <c r="D130" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E130" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F130" s="1">
         <v>5</v>
       </c>
       <c r="G130" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H130" s="3">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="I130" s="3">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="2" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="C131" s="5">
         <f>AVERAGE(D131,E131,E131,F131,G131,H131,H131,I131)</f>
-        <v>5.5624999999999991</v>
+        <v>5.6749999999999998</v>
       </c>
       <c r="D131" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E131" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F131" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G131" s="1">
         <v>6</v>
       </c>
       <c r="H131" s="3">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="I131" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C132" s="5">
         <f>AVERAGE(D132,E132,E132,F132,G132,H132,H132,I132)</f>
         <v>5.5624999999999991</v>
       </c>
       <c r="D132" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E132" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F132" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G132" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H132" s="3">
         <v>5.8</v>
@@ -8341,26 +8344,26 @@
     </row>
     <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="2" t="s">
-        <v>229</v>
+        <v>156</v>
       </c>
       <c r="C133" s="5">
         <f>AVERAGE(D133,E133,E133,F133,G133,H133,H133,I133)</f>
-        <v>5.5375000000000005</v>
+        <v>5.5624999999999991</v>
       </c>
       <c r="D133" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E133" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F133" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G133" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H133" s="3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="I133" s="3">
         <v>4.9000000000000004</v>
@@ -8368,11 +8371,11 @@
     </row>
     <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="2" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="C134" s="5">
         <f>AVERAGE(D134,E134,E134,F134,G134,H134,H134,I134)</f>
-        <v>5.5125000000000011</v>
+        <v>5.5375000000000005</v>
       </c>
       <c r="D134" s="1">
         <v>6</v>
@@ -8390,22 +8393,22 @@
         <v>5.7</v>
       </c>
       <c r="I134" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="2" t="s">
-        <v>166</v>
+        <v>245</v>
       </c>
       <c r="C135" s="5">
         <f>AVERAGE(D135,E135,E135,F135,G135,H135,H135,I135)</f>
-        <v>5.4874999999999989</v>
+        <v>5.5125000000000011</v>
       </c>
       <c r="D135" s="1">
         <v>6</v>
       </c>
       <c r="E135" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F135" s="1">
         <v>6</v>
@@ -8414,376 +8417,376 @@
         <v>6</v>
       </c>
       <c r="H135" s="3">
-        <v>4.8</v>
+        <v>5.7</v>
       </c>
       <c r="I135" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="2" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C136" s="5">
         <f>AVERAGE(D136,E136,E136,F136,G136,H136,H136,I136)</f>
         <v>5.4874999999999989</v>
       </c>
       <c r="D136" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E136" s="1">
         <v>6</v>
       </c>
       <c r="F136" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G136" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H136" s="3">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="I136" s="3">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="2" t="s">
-        <v>228</v>
+        <v>191</v>
       </c>
       <c r="C137" s="5">
         <f>AVERAGE(D137,E137,E137,F137,G137,H137,H137,I137)</f>
-        <v>5.3875000000000011</v>
+        <v>5.4874999999999989</v>
       </c>
       <c r="D137" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E137" s="1">
         <v>6</v>
       </c>
       <c r="F137" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G137" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H137" s="3">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="I137" s="3">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="2" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="C138" s="5">
         <f>AVERAGE(D138,E138,E138,F138,G138,H138,H138,I138)</f>
-        <v>5.3750000000000009</v>
+        <v>5.3875000000000011</v>
       </c>
       <c r="D138" s="1">
         <v>6</v>
       </c>
       <c r="E138" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F138" s="1">
         <v>6</v>
       </c>
       <c r="G138" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H138" s="3">
         <v>4.7</v>
       </c>
       <c r="I138" s="3">
-        <v>4.5999999999999996</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="2" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C139" s="5">
         <f>AVERAGE(D139,E139,E139,F139,G139,H139,H139,I139)</f>
-        <v>5.375</v>
+        <v>5.3750000000000009</v>
       </c>
       <c r="D139" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E139" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F139" s="1">
         <v>6</v>
       </c>
       <c r="G139" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H139" s="3">
-        <v>5.6</v>
+        <v>4.7</v>
       </c>
       <c r="I139" s="3">
-        <v>4.8</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C140" s="5">
         <f>AVERAGE(D140,E140,E140,F140,G140,H140,H140,I140)</f>
-        <v>5.2875000000000005</v>
+        <v>5.375</v>
       </c>
       <c r="D140" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E140" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F140" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G140" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H140" s="3">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="I140" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="2" t="s">
-        <v>242</v>
+        <v>182</v>
       </c>
       <c r="C141" s="5">
         <f>AVERAGE(D141,E141,E141,F141,G141,H141,H141,I141)</f>
-        <v>5.25</v>
+        <v>5.2875000000000005</v>
       </c>
       <c r="D141" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E141" s="1">
         <v>5</v>
       </c>
       <c r="F141" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G141" s="1">
         <v>5</v>
       </c>
       <c r="H141" s="3">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="I141" s="3">
-        <v>5.6</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="2" t="s">
-        <v>271</v>
+        <v>242</v>
       </c>
       <c r="C142" s="5">
         <f>AVERAGE(D142,E142,E142,F142,G142,H142,H142,I142)</f>
-        <v>5.2374999999999998</v>
+        <v>5.25</v>
       </c>
       <c r="D142" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E142" s="1">
         <v>5</v>
       </c>
       <c r="F142" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G142" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H142" s="3">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="I142" s="3">
-        <v>4.9000000000000004</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="2" t="s">
-        <v>232</v>
+        <v>271</v>
       </c>
       <c r="C143" s="5">
         <f>AVERAGE(D143,E143,E143,F143,G143,H143,H143,I143)</f>
-        <v>5.2</v>
+        <v>5.2374999999999998</v>
       </c>
       <c r="D143" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E143" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F143" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G143" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H143" s="3">
-        <v>7.1</v>
+        <v>5.5</v>
       </c>
       <c r="I143" s="3">
-        <v>6.4</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="2" t="s">
-        <v>74</v>
+        <v>232</v>
       </c>
       <c r="C144" s="5">
         <f>AVERAGE(D144,E144,E144,F144,G144,H144,H144,I144)</f>
-        <v>5.1875</v>
+        <v>5.2</v>
       </c>
       <c r="D144" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E144" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F144" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G144" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H144" s="3">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="I144" s="3">
-        <v>3.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="2" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="C145" s="5">
         <f>AVERAGE(D145,E145,E145,F145,G145,H145,H145,I145)</f>
-        <v>5.1124999999999998</v>
+        <v>5.1875</v>
       </c>
       <c r="D145" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E145" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F145" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G145" s="1">
         <v>6</v>
       </c>
       <c r="H145" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I145" s="3">
-        <v>5.0999999999999996</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="2" t="s">
-        <v>223</v>
+        <v>145</v>
       </c>
       <c r="C146" s="5">
         <f>AVERAGE(D146,E146,E146,F146,G146,H146,H146,I146)</f>
-        <v>5.0750000000000002</v>
+        <v>5.1124999999999998</v>
       </c>
       <c r="D146" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E146" s="1">
         <v>4</v>
       </c>
       <c r="F146" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G146" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H146" s="3">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I146" s="3">
-        <v>5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="2" t="s">
-        <v>21</v>
+        <v>223</v>
       </c>
       <c r="C147" s="5">
         <f>AVERAGE(D147,E147,E147,F147,G147,H147,H147,I147)</f>
-        <v>5.05</v>
+        <v>5.0750000000000002</v>
       </c>
       <c r="D147" s="1">
         <v>5</v>
       </c>
       <c r="E147" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F147" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G147" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H147" s="3">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="I147" s="3">
-        <v>5.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="2" t="s">
-        <v>203</v>
+        <v>21</v>
       </c>
       <c r="C148" s="5">
         <f>AVERAGE(D148,E148,E148,F148,G148,H148,H148,I148)</f>
-        <v>4.9875000000000007</v>
+        <v>5.05</v>
       </c>
       <c r="D148" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E148" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F148" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G148" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H148" s="3">
-        <v>4.0999999999999996</v>
+        <v>6.8</v>
       </c>
       <c r="I148" s="3">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="2" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="C149" s="5">
         <f>AVERAGE(D149,E149,E149,F149,G149,H149,H149,I149)</f>
-        <v>4.9874999999999998</v>
+        <v>4.9875000000000007</v>
       </c>
       <c r="D149" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E149" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F149" s="1">
         <v>5</v>
@@ -8792,262 +8795,262 @@
         <v>6</v>
       </c>
       <c r="H149" s="3">
-        <v>6</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I149" s="3">
-        <v>4.9000000000000004</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="2" t="s">
-        <v>264</v>
+        <v>169</v>
       </c>
       <c r="C150" s="5">
         <f>AVERAGE(D150,E150,E150,F150,G150,H150,H150,I150)</f>
         <v>4.9874999999999998</v>
       </c>
       <c r="D150" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E150" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F150" s="1">
         <v>5</v>
       </c>
       <c r="G150" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H150" s="3">
-        <v>5.2</v>
+        <v>6</v>
       </c>
       <c r="I150" s="3">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="2" t="s">
-        <v>241</v>
+        <v>264</v>
       </c>
       <c r="C151" s="5">
         <f>AVERAGE(D151,E151,E151,F151,G151,H151,H151,I151)</f>
-        <v>4.9249999999999998</v>
+        <v>4.9874999999999998</v>
       </c>
       <c r="D151" s="1">
         <v>5</v>
       </c>
       <c r="E151" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F151" s="1">
         <v>5</v>
       </c>
       <c r="G151" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H151" s="3">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="I151" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="2" t="s">
-        <v>163</v>
+        <v>241</v>
       </c>
       <c r="C152" s="5">
         <f>AVERAGE(D152,E152,E152,F152,G152,H152,H152,I152)</f>
-        <v>4.8499999999999996</v>
+        <v>4.9249999999999998</v>
       </c>
       <c r="D152" s="1">
         <v>5</v>
       </c>
       <c r="E152" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F152" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G152" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H152" s="3">
         <v>5.5</v>
       </c>
       <c r="I152" s="3">
-        <v>4.8</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C153" s="5">
         <f>AVERAGE(D153,E153,E153,F153,G153,H153,H153,I153)</f>
-        <v>4.7875000000000005</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="D153" s="1">
         <v>5</v>
       </c>
       <c r="E153" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F153" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G153" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H153" s="3">
+        <v>5.5</v>
+      </c>
+      <c r="I153" s="3">
         <v>4.8</v>
-      </c>
-      <c r="I153" s="3">
-        <v>3.7</v>
       </c>
     </row>
     <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="2" t="s">
-        <v>262</v>
+        <v>162</v>
       </c>
       <c r="C154" s="5">
         <f>AVERAGE(D154,E154,E154,F154,G154,H154,H154,I154)</f>
-        <v>4.7125000000000004</v>
+        <v>4.7875000000000005</v>
       </c>
       <c r="D154" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E154" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F154" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G154" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H154" s="3">
-        <v>6.5</v>
+        <v>4.8</v>
       </c>
       <c r="I154" s="3">
-        <v>5.7</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="C155" s="5">
         <f>AVERAGE(D155,E155,E155,F155,G155,H155,H155,I155)</f>
-        <v>4.6875</v>
+        <v>4.7125000000000004</v>
       </c>
       <c r="D155" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E155" s="1">
+        <v>3</v>
+      </c>
+      <c r="F155" s="1">
         <v>4</v>
       </c>
-      <c r="F155" s="1">
-        <v>3</v>
-      </c>
       <c r="G155" s="1">
         <v>5</v>
       </c>
       <c r="H155" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="I155" s="3">
         <v>5.7</v>
-      </c>
-      <c r="I155" s="3">
-        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="2" t="s">
-        <v>213</v>
+        <v>270</v>
       </c>
       <c r="C156" s="5">
         <f>AVERAGE(D156,E156,E156,F156,G156,H156,H156,I156)</f>
-        <v>4.6124999999999998</v>
+        <v>4.6875</v>
       </c>
       <c r="D156" s="1">
+        <v>5</v>
+      </c>
+      <c r="E156" s="1">
         <v>4</v>
       </c>
-      <c r="E156" s="1">
+      <c r="F156" s="1">
         <v>3</v>
       </c>
-      <c r="F156" s="1">
-        <v>4</v>
-      </c>
       <c r="G156" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H156" s="3">
-        <v>6.7</v>
+        <v>5.7</v>
       </c>
       <c r="I156" s="3">
-        <v>5.5</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="2" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="C157" s="5">
         <f>AVERAGE(D157,E157,E157,F157,G157,H157,H157,I157)</f>
-        <v>4.5999999999999996</v>
+        <v>4.6124999999999998</v>
       </c>
       <c r="D157" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E157" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F157" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G157" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H157" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
       <c r="I157" s="3">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="2" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C158" s="5">
         <f>AVERAGE(D158,E158,E158,F158,G158,H158,H158,I158)</f>
-        <v>4.5874999999999995</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D158" s="1">
         <v>5</v>
       </c>
       <c r="E158" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F158" s="1">
         <v>5</v>
       </c>
       <c r="G158" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H158" s="3">
         <v>4.9000000000000004</v>
       </c>
       <c r="I158" s="3">
-        <v>3.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="2" t="s">
-        <v>243</v>
+        <v>135</v>
       </c>
       <c r="C159" s="5">
         <f>AVERAGE(D159,E159,E159,F159,G159,H159,H159,I159)</f>
-        <v>4.5</v>
+        <v>4.5874999999999995</v>
       </c>
       <c r="D159" s="1">
         <v>5</v>
@@ -9056,436 +9059,436 @@
         <v>4</v>
       </c>
       <c r="F159" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G159" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H159" s="3">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I159" s="3">
-        <v>5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="2" t="s">
-        <v>161</v>
+        <v>243</v>
       </c>
       <c r="C160" s="5">
         <f>AVERAGE(D160,E160,E160,F160,G160,H160,H160,I160)</f>
-        <v>4.4249999999999998</v>
+        <v>4.5</v>
       </c>
       <c r="D160" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E160" s="1">
         <v>4</v>
       </c>
       <c r="F160" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G160" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H160" s="3">
         <v>5.5</v>
       </c>
       <c r="I160" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="2" t="s">
-        <v>114</v>
+        <v>161</v>
       </c>
       <c r="C161" s="5">
         <f>AVERAGE(D161,E161,E161,F161,G161,H161,H161,I161)</f>
-        <v>4.4124999999999996</v>
+        <v>4.4249999999999998</v>
       </c>
       <c r="D161" s="1">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E161" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F161" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G161" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H161" s="3">
-        <v>8.1999999999999993</v>
+        <v>5.5</v>
       </c>
       <c r="I161" s="3">
-        <v>7.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="2" t="s">
-        <v>267</v>
+        <v>114</v>
       </c>
       <c r="C162" s="5">
         <f>AVERAGE(D162,E162,E162,F162,G162,H162,H162,I162)</f>
-        <v>4.375</v>
+        <v>4.4124999999999996</v>
       </c>
       <c r="D162" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E162" s="1">
+        <v>0</v>
+      </c>
+      <c r="F162" s="1">
         <v>2</v>
       </c>
-      <c r="F162" s="1">
-        <v>6</v>
-      </c>
       <c r="G162" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H162" s="3">
-        <v>5.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I162" s="3">
-        <v>4.5999999999999996</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="2" t="s">
-        <v>207</v>
+        <v>267</v>
       </c>
       <c r="C163" s="5">
         <f>AVERAGE(D163,E163,E163,F163,G163,H163,H163,I163)</f>
-        <v>4.3375000000000004</v>
+        <v>4.375</v>
       </c>
       <c r="D163" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E163" s="1">
         <v>2</v>
       </c>
       <c r="F163" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G163" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H163" s="3">
-        <v>6</v>
+        <v>5.2</v>
       </c>
       <c r="I163" s="3">
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="164" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B164" s="2" t="s">
-        <v>150</v>
+        <v>207</v>
       </c>
       <c r="C164" s="5">
         <f>AVERAGE(D164,E164,E164,F164,G164,H164,H164,I164)</f>
-        <v>4.3374999999999995</v>
+        <v>4.3375000000000004</v>
       </c>
       <c r="D164" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E164" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F164" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G164" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H164" s="3">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I164" s="3">
-        <v>4.9000000000000004</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="165" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B165" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="C165" s="5">
         <f>AVERAGE(D165,E165,E165,F165,G165,H165,H165,I165)</f>
-        <v>4.3125</v>
+        <v>4.3374999999999995</v>
       </c>
       <c r="D165" s="1">
+        <v>5</v>
+      </c>
+      <c r="E165" s="1">
         <v>3</v>
       </c>
-      <c r="E165" s="1">
-        <v>4</v>
-      </c>
       <c r="F165" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G165" s="1">
         <v>4</v>
       </c>
       <c r="H165" s="3">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="I165" s="3">
-        <v>4.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="166" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B166" s="2" t="s">
-        <v>258</v>
+        <v>173</v>
       </c>
       <c r="C166" s="5">
         <f>AVERAGE(D166,E166,E166,F166,G166,H166,H166,I166)</f>
-        <v>4.3000000000000007</v>
+        <v>4.3125</v>
       </c>
       <c r="D166" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E166" s="1">
         <v>4</v>
       </c>
       <c r="F166" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G166" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H166" s="3">
-        <v>6.6</v>
+        <v>5.4</v>
       </c>
       <c r="I166" s="3">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="167" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B167" s="2" t="s">
-        <v>212</v>
+        <v>258</v>
       </c>
       <c r="C167" s="5">
         <f>AVERAGE(D167,E167,E167,F167,G167,H167,H167,I167)</f>
-        <v>4.3</v>
+        <v>4.3000000000000007</v>
       </c>
       <c r="D167" s="1">
+        <v>2</v>
+      </c>
+      <c r="E167" s="1">
         <v>4</v>
-      </c>
-      <c r="E167" s="1">
-        <v>3</v>
       </c>
       <c r="F167" s="1">
         <v>3</v>
       </c>
       <c r="G167" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H167" s="3">
-        <v>6.3</v>
+        <v>6.6</v>
       </c>
       <c r="I167" s="3">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="168" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B168" s="2" t="s">
-        <v>167</v>
+        <v>212</v>
       </c>
       <c r="C168" s="5">
         <f>AVERAGE(D168,E168,E168,F168,G168,H168,H168,I168)</f>
-        <v>4.2749999999999995</v>
+        <v>4.3</v>
       </c>
       <c r="D168" s="1">
         <v>4</v>
       </c>
       <c r="E168" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F168" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G168" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H168" s="3">
-        <v>4.9000000000000004</v>
+        <v>6.3</v>
       </c>
       <c r="I168" s="3">
-        <v>4.4000000000000004</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="169" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B169" s="2" t="s">
-        <v>236</v>
+        <v>167</v>
       </c>
       <c r="C169" s="5">
         <f>AVERAGE(D169,E169,E169,F169,G169,H169,H169,I169)</f>
-        <v>4.1749999999999998</v>
+        <v>4.2749999999999995</v>
       </c>
       <c r="D169" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E169" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F169" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G169" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H169" s="3">
-        <v>5.4</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="I169" s="3">
-        <v>3.6</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="170" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B170" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C170" s="5">
         <f>AVERAGE(D170,E170,E170,F170,G170,H170,H170,I170)</f>
-        <v>4.1625000000000005</v>
+        <v>4.1749999999999998</v>
       </c>
       <c r="D170" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E170" s="1">
         <v>3</v>
       </c>
       <c r="F170" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G170" s="1">
         <v>4</v>
       </c>
       <c r="H170" s="3">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I170" s="3">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="171" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B171" s="2" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C171" s="5">
         <f>AVERAGE(D171,E171,E171,F171,G171,H171,H171,I171)</f>
-        <v>4.1124999999999998</v>
+        <v>4.1625000000000005</v>
       </c>
       <c r="D171" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E171" s="1">
+        <v>3</v>
+      </c>
+      <c r="F171" s="1">
+        <v>3</v>
+      </c>
+      <c r="G171" s="1">
         <v>4</v>
       </c>
-      <c r="F171" s="1">
-        <v>2</v>
-      </c>
-      <c r="G171" s="1">
-        <v>5</v>
-      </c>
       <c r="H171" s="3">
-        <v>4.5</v>
+        <v>5.8</v>
       </c>
       <c r="I171" s="3">
-        <v>3.9</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="172" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B172" s="2" t="s">
-        <v>218</v>
+        <v>68</v>
       </c>
       <c r="C172" s="5">
         <f>AVERAGE(D172,E172,E172,F172,G172,H172,H172,I172)</f>
-        <v>3.9499999999999997</v>
+        <v>4.1124999999999998</v>
       </c>
       <c r="D172" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E172" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F172" s="1">
         <v>2</v>
       </c>
       <c r="G172" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H172" s="3">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="I172" s="3">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="173" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B173" s="9" t="s">
-        <v>272</v>
+      <c r="B173" s="2" t="s">
+        <v>218</v>
       </c>
       <c r="C173" s="5">
         <f>AVERAGE(D173,E173,E173,F173,G173,H173,H173,I173)</f>
-        <v>3.9125000000000001</v>
+        <v>3.9499999999999997</v>
       </c>
       <c r="D173" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E173" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F173" s="1">
         <v>2</v>
       </c>
       <c r="G173" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H173" s="3">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
       <c r="I173" s="3">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="174" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B174" s="2" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="C174" s="5">
         <f>AVERAGE(D174,E174,E174,F174,G174,H174,H174,I174)</f>
-        <v>3.7375000000000003</v>
+        <v>3.9125000000000001</v>
       </c>
       <c r="D174" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E174" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F174" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G174" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H174" s="3">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="I174" s="3">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="175" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B175" s="2" t="s">
-        <v>250</v>
+        <v>199</v>
       </c>
       <c r="C175" s="5">
         <f>AVERAGE(D175,E175,E175,F175,G175,H175,H175,I175)</f>
-        <v>3.6624999999999996</v>
+        <v>3.7375000000000003</v>
       </c>
       <c r="D175" s="1">
         <v>3</v>
       </c>
       <c r="E175" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F175" s="1">
         <v>3</v>
@@ -9494,333 +9497,360 @@
         <v>4</v>
       </c>
       <c r="H175" s="3">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="I175" s="3">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="176" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B176" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C176" s="5">
         <f>AVERAGE(D176,E176,E176,F176,G176,H176,H176,I176)</f>
-        <v>3.5749999999999997</v>
+        <v>3.6624999999999996</v>
       </c>
       <c r="D176" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E176" s="1">
         <v>2</v>
       </c>
       <c r="F176" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G176" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H176" s="3">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="I176" s="3">
-        <v>5.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="177" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B177" s="2">
-        <v>180</v>
+      <c r="B177" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="C177" s="5">
         <f>AVERAGE(D177,E177,E177,F177,G177,H177,H177,I177)</f>
-        <v>3.5625000000000004</v>
+        <v>3.5749999999999997</v>
       </c>
       <c r="D177" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E177" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F177" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G177" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H177" s="3">
-        <v>4.5999999999999996</v>
+        <v>6.2</v>
       </c>
       <c r="I177" s="3">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="178" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B178" s="2" t="s">
-        <v>216</v>
+      <c r="B178" s="2">
+        <v>180</v>
       </c>
       <c r="C178" s="5">
         <f>AVERAGE(D178,E178,E178,F178,G178,H178,H178,I178)</f>
-        <v>3.5375000000000005</v>
+        <v>3.5625000000000004</v>
       </c>
       <c r="D178" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E178" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F178" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G178" s="1">
         <v>3</v>
       </c>
       <c r="H178" s="3">
-        <v>5.0999999999999996</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="I178" s="3">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="179" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B179" s="2" t="s">
-        <v>248</v>
+        <v>216</v>
       </c>
       <c r="C179" s="5">
         <f>AVERAGE(D179,E179,E179,F179,G179,H179,H179,I179)</f>
-        <v>3.3375000000000004</v>
+        <v>3.5375000000000005</v>
       </c>
       <c r="D179" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E179" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F179" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G179" s="1">
         <v>3</v>
       </c>
       <c r="H179" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="I179" s="3">
         <v>4.0999999999999996</v>
-      </c>
-      <c r="I179" s="3">
-        <v>3.5</v>
       </c>
     </row>
     <row r="180" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B180" s="2" t="s">
-        <v>189</v>
+        <v>248</v>
       </c>
       <c r="C180" s="5">
         <f>AVERAGE(D180,E180,E180,F180,G180,H180,H180,I180)</f>
-        <v>3.3250000000000002</v>
+        <v>3.3375000000000004</v>
       </c>
       <c r="D180" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E180" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F180" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G180" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H180" s="3">
-        <v>5.8</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="I180" s="3">
-        <v>5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="181" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B181" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C181" s="5">
         <f>AVERAGE(D181,E181,E181,F181,G181,H181,H181,I181)</f>
-        <v>3.2749999999999995</v>
+        <v>3.3250000000000002</v>
       </c>
       <c r="D181" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E181" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F181" s="1">
         <v>2</v>
       </c>
       <c r="G181" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H181" s="3">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="I181" s="3">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
     </row>
     <row r="182" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B182" s="2" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C182" s="5">
         <f>AVERAGE(D182,E182,E182,F182,G182,H182,H182,I182)</f>
-        <v>2.9124999999999996</v>
+        <v>3.2749999999999995</v>
       </c>
       <c r="D182" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E182" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F182" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G182" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H182" s="3">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="I182" s="3">
-        <v>5.9</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="183" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B183" s="2" t="s">
-        <v>237</v>
+        <v>155</v>
       </c>
       <c r="C183" s="5">
         <f>AVERAGE(D183,E183,E183,F183,G183,H183,H183,I183)</f>
-        <v>2.8125</v>
+        <v>2.9124999999999996</v>
       </c>
       <c r="D183" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E183" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F183" s="1">
         <v>0</v>
       </c>
       <c r="G183" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H183" s="3">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="I183" s="3">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="184" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B184" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C184" s="5">
         <f>AVERAGE(D184,E184,E184,F184,G184,H184,H184,I184)</f>
-        <v>2.7625000000000002</v>
+        <v>2.8125</v>
       </c>
       <c r="D184" s="1">
         <v>2</v>
       </c>
       <c r="E184" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F184" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G184" s="1">
         <v>2</v>
       </c>
       <c r="H184" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I184" s="3">
         <v>5.5</v>
-      </c>
-      <c r="I184" s="3">
-        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="185" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B185" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="C185" s="5">
         <f>AVERAGE(D185,E185,E185,F185,G185,H185,H185,I185)</f>
-        <v>2.65</v>
+        <v>2.7625000000000002</v>
       </c>
       <c r="D185" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E185" s="1">
         <v>1</v>
       </c>
       <c r="F185" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G185" s="1">
         <v>2</v>
       </c>
       <c r="H185" s="3">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
       <c r="I185" s="3">
-        <v>3.8</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="186" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B186" s="2" t="s">
-        <v>174</v>
+        <v>251</v>
       </c>
       <c r="C186" s="5">
         <f>AVERAGE(D186,E186,E186,F186,G186,H186,H186,I186)</f>
-        <v>2.6375000000000002</v>
+        <v>2.65</v>
       </c>
       <c r="D186" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E186" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F186" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G186" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H186" s="3">
-        <v>7.6</v>
+        <v>4.2</v>
       </c>
       <c r="I186" s="3">
-        <v>5.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="187" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B187" s="2" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="C187" s="5">
         <f>AVERAGE(D187,E187,E187,F187,G187,H187,H187,I187)</f>
+        <v>2.6375000000000002</v>
+      </c>
+      <c r="D187" s="1">
+        <v>0</v>
+      </c>
+      <c r="E187" s="1">
+        <v>0</v>
+      </c>
+      <c r="F187" s="1">
+        <v>0</v>
+      </c>
+      <c r="G187" s="1">
+        <v>0</v>
+      </c>
+      <c r="H187" s="3">
+        <v>7.6</v>
+      </c>
+      <c r="I187" s="3">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="188" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B188" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C188" s="5">
+        <f>AVERAGE(D188,E188,E188,F188,G188,H188,H188,I188)</f>
         <v>2.5125000000000002</v>
       </c>
-      <c r="D187" s="1">
+      <c r="D188" s="1">
         <v>2</v>
       </c>
-      <c r="E187" s="1">
+      <c r="E188" s="1">
         <v>1</v>
       </c>
-      <c r="F187" s="1">
+      <c r="F188" s="1">
         <v>2</v>
       </c>
-      <c r="G187" s="1">
+      <c r="G188" s="1">
         <v>2</v>
       </c>
-      <c r="H187" s="3">
+      <c r="H188" s="3">
         <v>4.3</v>
       </c>
-      <c r="I187" s="3">
+      <c r="I188" s="3">
         <v>3.5</v>
       </c>
     </row>

</xml_diff>